<commit_message>
SGL Production Plan updated — 29/05/2026 09:37
</commit_message>
<xml_diff>
--- a/Production_Plan.xlsx
+++ b/Production_Plan.xlsx
@@ -13024,10 +13024,10 @@
         <v>3</v>
       </c>
       <c r="J269" t="str">
-        <v>2026-05-11</v>
+        <v>2026-05-14</v>
       </c>
       <c r="K269" t="str">
-        <v>2026-05-13</v>
+        <v>2026-05-16</v>
       </c>
       <c r="L269">
         <v>646</v>
@@ -13071,10 +13071,10 @@
         <v>3</v>
       </c>
       <c r="J270" t="str">
-        <v>2026-05-11</v>
+        <v>2026-05-14</v>
       </c>
       <c r="K270" t="str">
-        <v>2026-05-13</v>
+        <v>2026-05-16</v>
       </c>
       <c r="L270">
         <v>646</v>
@@ -13118,10 +13118,10 @@
         <v>3</v>
       </c>
       <c r="J271" t="str">
-        <v>2026-05-11</v>
+        <v>2026-05-14</v>
       </c>
       <c r="K271" t="str">
-        <v>2026-05-13</v>
+        <v>2026-05-16</v>
       </c>
       <c r="L271">
         <v>646</v>
@@ -13165,10 +13165,10 @@
         <v>3</v>
       </c>
       <c r="J272" t="str">
-        <v>2026-05-11</v>
+        <v>2026-05-14</v>
       </c>
       <c r="K272" t="str">
-        <v>2026-05-13</v>
+        <v>2026-05-16</v>
       </c>
       <c r="L272">
         <v>646</v>
@@ -13212,10 +13212,10 @@
         <v>3</v>
       </c>
       <c r="J273" t="str">
-        <v>2026-05-11</v>
+        <v>2026-05-14</v>
       </c>
       <c r="K273" t="str">
-        <v>2026-05-13</v>
+        <v>2026-05-16</v>
       </c>
       <c r="L273">
         <v>646</v>
@@ -13259,10 +13259,10 @@
         <v>3</v>
       </c>
       <c r="J274" t="str">
-        <v>2026-05-11</v>
+        <v>2026-05-14</v>
       </c>
       <c r="K274" t="str">
-        <v>2026-05-13</v>
+        <v>2026-05-16</v>
       </c>
       <c r="L274">
         <v>646</v>
@@ -13306,10 +13306,10 @@
         <v>3</v>
       </c>
       <c r="J275" t="str">
-        <v>2026-05-11</v>
+        <v>2026-05-14</v>
       </c>
       <c r="K275" t="str">
-        <v>2026-05-13</v>
+        <v>2026-05-16</v>
       </c>
       <c r="L275">
         <v>646</v>
@@ -13353,10 +13353,10 @@
         <v>3</v>
       </c>
       <c r="J276" t="str">
-        <v>2026-05-11</v>
+        <v>2026-05-14</v>
       </c>
       <c r="K276" t="str">
-        <v>2026-05-13</v>
+        <v>2026-05-16</v>
       </c>
       <c r="L276">
         <v>646</v>
@@ -13400,10 +13400,10 @@
         <v>3</v>
       </c>
       <c r="J277" t="str">
-        <v>2026-05-11</v>
+        <v>2026-05-14</v>
       </c>
       <c r="K277" t="str">
-        <v>2026-05-13</v>
+        <v>2026-05-16</v>
       </c>
       <c r="L277">
         <v>646</v>
@@ -13447,10 +13447,10 @@
         <v>3</v>
       </c>
       <c r="J278" t="str">
-        <v>2026-05-11</v>
+        <v>2026-05-14</v>
       </c>
       <c r="K278" t="str">
-        <v>2026-05-13</v>
+        <v>2026-05-16</v>
       </c>
       <c r="L278">
         <v>646</v>
@@ -13494,10 +13494,10 @@
         <v>3</v>
       </c>
       <c r="J279" t="str">
-        <v>2026-05-11</v>
+        <v>2026-05-14</v>
       </c>
       <c r="K279" t="str">
-        <v>2026-05-13</v>
+        <v>2026-05-16</v>
       </c>
       <c r="L279">
         <v>646</v>
@@ -13541,10 +13541,10 @@
         <v>3</v>
       </c>
       <c r="J280" t="str">
-        <v>2026-05-11</v>
+        <v>2026-05-14</v>
       </c>
       <c r="K280" t="str">
-        <v>2026-05-13</v>
+        <v>2026-05-16</v>
       </c>
       <c r="L280">
         <v>646</v>
@@ -13588,10 +13588,10 @@
         <v>3</v>
       </c>
       <c r="J281" t="str">
-        <v>2026-05-11</v>
+        <v>2026-05-14</v>
       </c>
       <c r="K281" t="str">
-        <v>2026-05-13</v>
+        <v>2026-05-16</v>
       </c>
       <c r="L281">
         <v>646</v>
@@ -13635,10 +13635,10 @@
         <v>3</v>
       </c>
       <c r="J282" t="str">
-        <v>2026-05-11</v>
+        <v>2026-05-14</v>
       </c>
       <c r="K282" t="str">
-        <v>2026-05-13</v>
+        <v>2026-05-16</v>
       </c>
       <c r="L282">
         <v>646</v>
@@ -13682,10 +13682,10 @@
         <v>3</v>
       </c>
       <c r="J283" t="str">
-        <v>2026-05-11</v>
+        <v>2026-05-14</v>
       </c>
       <c r="K283" t="str">
-        <v>2026-05-13</v>
+        <v>2026-05-16</v>
       </c>
       <c r="L283">
         <v>646</v>

</xml_diff>

<commit_message>
SGL Production Plan updated — 01/06/2026 10:06
</commit_message>
<xml_diff>
--- a/Production_Plan.xlsx
+++ b/Production_Plan.xlsx
@@ -13071,10 +13071,10 @@
         <v>3</v>
       </c>
       <c r="J270" t="str">
-        <v>2026-05-13</v>
+        <v>2026-05-15</v>
       </c>
       <c r="K270" t="str">
-        <v>2026-05-14</v>
+        <v>2026-05-18</v>
       </c>
       <c r="L270">
         <v>646</v>
@@ -13118,10 +13118,10 @@
         <v>3</v>
       </c>
       <c r="J271" t="str">
-        <v>2026-05-13</v>
+        <v>2026-05-15</v>
       </c>
       <c r="K271" t="str">
-        <v>2026-05-14</v>
+        <v>2026-05-18</v>
       </c>
       <c r="L271">
         <v>646</v>
@@ -13165,10 +13165,10 @@
         <v>3</v>
       </c>
       <c r="J272" t="str">
-        <v>2026-05-13</v>
+        <v>2026-05-15</v>
       </c>
       <c r="K272" t="str">
-        <v>2026-05-14</v>
+        <v>2026-05-18</v>
       </c>
       <c r="L272">
         <v>646</v>
@@ -13212,10 +13212,10 @@
         <v>3</v>
       </c>
       <c r="J273" t="str">
-        <v>2026-05-13</v>
+        <v>2026-05-15</v>
       </c>
       <c r="K273" t="str">
-        <v>2026-05-14</v>
+        <v>2026-05-18</v>
       </c>
       <c r="L273">
         <v>646</v>
@@ -13259,10 +13259,10 @@
         <v>3</v>
       </c>
       <c r="J274" t="str">
-        <v>2026-05-13</v>
+        <v>2026-05-15</v>
       </c>
       <c r="K274" t="str">
-        <v>2026-05-14</v>
+        <v>2026-05-18</v>
       </c>
       <c r="L274">
         <v>646</v>
@@ -13306,10 +13306,10 @@
         <v>3</v>
       </c>
       <c r="J275" t="str">
-        <v>2026-05-13</v>
+        <v>2026-05-15</v>
       </c>
       <c r="K275" t="str">
-        <v>2026-05-14</v>
+        <v>2026-05-18</v>
       </c>
       <c r="L275">
         <v>646</v>
@@ -13353,10 +13353,10 @@
         <v>3</v>
       </c>
       <c r="J276" t="str">
-        <v>2026-05-13</v>
+        <v>2026-05-15</v>
       </c>
       <c r="K276" t="str">
-        <v>2026-05-14</v>
+        <v>2026-05-18</v>
       </c>
       <c r="L276">
         <v>646</v>
@@ -13400,10 +13400,10 @@
         <v>3</v>
       </c>
       <c r="J277" t="str">
-        <v>2026-05-13</v>
+        <v>2026-05-15</v>
       </c>
       <c r="K277" t="str">
-        <v>2026-05-14</v>
+        <v>2026-05-18</v>
       </c>
       <c r="L277">
         <v>646</v>
@@ -13447,10 +13447,10 @@
         <v>3</v>
       </c>
       <c r="J278" t="str">
-        <v>2026-05-13</v>
+        <v>2026-05-15</v>
       </c>
       <c r="K278" t="str">
-        <v>2026-05-14</v>
+        <v>2026-05-18</v>
       </c>
       <c r="L278">
         <v>646</v>
@@ -13494,10 +13494,10 @@
         <v>3</v>
       </c>
       <c r="J279" t="str">
-        <v>2026-05-13</v>
+        <v>2026-05-15</v>
       </c>
       <c r="K279" t="str">
-        <v>2026-05-14</v>
+        <v>2026-05-18</v>
       </c>
       <c r="L279">
         <v>646</v>
@@ -13541,10 +13541,10 @@
         <v>3</v>
       </c>
       <c r="J280" t="str">
-        <v>2026-05-13</v>
+        <v>2026-05-15</v>
       </c>
       <c r="K280" t="str">
-        <v>2026-05-14</v>
+        <v>2026-05-18</v>
       </c>
       <c r="L280">
         <v>646</v>
@@ -13588,10 +13588,10 @@
         <v>3</v>
       </c>
       <c r="J281" t="str">
-        <v>2026-05-13</v>
+        <v>2026-05-15</v>
       </c>
       <c r="K281" t="str">
-        <v>2026-05-14</v>
+        <v>2026-05-18</v>
       </c>
       <c r="L281">
         <v>646</v>
@@ -13635,10 +13635,10 @@
         <v>3</v>
       </c>
       <c r="J282" t="str">
-        <v>2026-05-13</v>
+        <v>2026-05-15</v>
       </c>
       <c r="K282" t="str">
-        <v>2026-05-14</v>
+        <v>2026-05-18</v>
       </c>
       <c r="L282">
         <v>646</v>
@@ -13682,10 +13682,10 @@
         <v>3</v>
       </c>
       <c r="J283" t="str">
-        <v>2026-05-13</v>
+        <v>2026-05-15</v>
       </c>
       <c r="K283" t="str">
-        <v>2026-05-14</v>
+        <v>2026-05-18</v>
       </c>
       <c r="L283">
         <v>646</v>

</xml_diff>

<commit_message>
SGL FR Plan — 03/06/2026 11:03
</commit_message>
<xml_diff>
--- a/Production_Plan.xlsx
+++ b/Production_Plan.xlsx
@@ -4290,7 +4290,7 @@
     </row>
     <row r="63">
       <c r="A63" t="str">
-        <v>SGL 03</v>
+        <v>SGL 01</v>
       </c>
       <c r="B63">
         <v>847</v>
@@ -4349,7 +4349,7 @@
     </row>
     <row r="64">
       <c r="A64" t="str">
-        <v>SGL 03</v>
+        <v>SGL 01</v>
       </c>
       <c r="B64">
         <v>847</v>
@@ -4408,7 +4408,7 @@
     </row>
     <row r="65">
       <c r="A65" t="str">
-        <v>SGL 08</v>
+        <v>SGL 01</v>
       </c>
       <c r="B65">
         <v>847</v>
@@ -4467,7 +4467,7 @@
     </row>
     <row r="66">
       <c r="A66" t="str">
-        <v>SGL 08</v>
+        <v>SGL 01</v>
       </c>
       <c r="B66">
         <v>847</v>
@@ -4526,7 +4526,7 @@
     </row>
     <row r="67">
       <c r="A67" t="str">
-        <v>SGL 08</v>
+        <v>SGL 01</v>
       </c>
       <c r="B67">
         <v>847</v>
@@ -4585,7 +4585,7 @@
     </row>
     <row r="68">
       <c r="A68" t="str">
-        <v>SGL 08</v>
+        <v>SGL 01</v>
       </c>
       <c r="B68">
         <v>847</v>
@@ -4644,7 +4644,7 @@
     </row>
     <row r="69">
       <c r="A69" t="str">
-        <v>SGL 02</v>
+        <v>SGL 01</v>
       </c>
       <c r="B69">
         <v>847</v>
@@ -4703,7 +4703,7 @@
     </row>
     <row r="70">
       <c r="A70" t="str">
-        <v>SGL 02</v>
+        <v>SGL 01</v>
       </c>
       <c r="B70">
         <v>847</v>
@@ -6778,7 +6778,7 @@
     </row>
     <row r="104">
       <c r="A104" t="str">
-        <v>SGL 03</v>
+        <v>SGL 02</v>
       </c>
       <c r="B104">
         <v>820</v>
@@ -6846,7 +6846,7 @@
     </row>
     <row r="105">
       <c r="A105" t="str">
-        <v>SGL 03</v>
+        <v>SGL 02</v>
       </c>
       <c r="B105">
         <v>820</v>
@@ -6914,7 +6914,7 @@
     </row>
     <row r="106">
       <c r="A106" t="str">
-        <v>SGL 03</v>
+        <v>SGL 02</v>
       </c>
       <c r="C106" t="str">
         <v>BOT12550NA::SGSGBONOB2876::JK</v>
@@ -6941,10 +6941,10 @@
         <v>46191</v>
       </c>
       <c r="S106">
-        <v>46190</v>
+        <v>46193</v>
       </c>
       <c r="T106">
-        <v>46198</v>
+        <v>46203</v>
       </c>
       <c r="V106" t="str">
         <v>460 Minol Ridmaka</v>
@@ -7708,7 +7708,7 @@
     </row>
     <row r="119">
       <c r="A119" t="str">
-        <v>SGL 03</v>
+        <v>SGL 02</v>
       </c>
       <c r="B119">
         <v>847</v>
@@ -7767,7 +7767,7 @@
     </row>
     <row r="120">
       <c r="A120" t="str">
-        <v>SGL 03</v>
+        <v>SGL 02</v>
       </c>
       <c r="B120">
         <v>847</v>
@@ -7826,7 +7826,7 @@
     </row>
     <row r="121">
       <c r="A121" t="str">
-        <v>SGL 08</v>
+        <v>SGL 02</v>
       </c>
       <c r="B121">
         <v>847</v>
@@ -7885,7 +7885,7 @@
     </row>
     <row r="122">
       <c r="A122" t="str">
-        <v>SGL 08</v>
+        <v>SGL 02</v>
       </c>
       <c r="B122">
         <v>847</v>
@@ -7944,7 +7944,7 @@
     </row>
     <row r="123">
       <c r="A123" t="str">
-        <v>SGL 08</v>
+        <v>SGL 02</v>
       </c>
       <c r="B123">
         <v>847</v>
@@ -10811,7 +10811,7 @@
     </row>
     <row r="172">
       <c r="A172" t="str">
-        <v>SGL 08</v>
+        <v>SGL 03</v>
       </c>
       <c r="B172">
         <v>847</v>
@@ -10870,7 +10870,7 @@
     </row>
     <row r="173">
       <c r="A173" t="str">
-        <v>SGL 08</v>
+        <v>SGL 03</v>
       </c>
       <c r="B173">
         <v>847</v>
@@ -11242,7 +11242,7 @@
     </row>
     <row r="179">
       <c r="A179" t="str">
-        <v>SGL 09</v>
+        <v>SGL 04</v>
       </c>
       <c r="B179">
         <v>539</v>
@@ -11307,7 +11307,7 @@
     </row>
     <row r="180">
       <c r="A180" t="str">
-        <v>SGL 09</v>
+        <v>SGL 04</v>
       </c>
       <c r="B180">
         <v>539</v>
@@ -11372,7 +11372,7 @@
     </row>
     <row r="181">
       <c r="A181" t="str">
-        <v>SGL 09</v>
+        <v>SGL 04</v>
       </c>
       <c r="B181">
         <v>539</v>
@@ -11437,7 +11437,7 @@
     </row>
     <row r="182">
       <c r="A182" t="str">
-        <v>SGL 09</v>
+        <v>SGL 04</v>
       </c>
       <c r="B182">
         <v>539</v>
@@ -11502,7 +11502,7 @@
     </row>
     <row r="183">
       <c r="A183" t="str">
-        <v>SGL 09</v>
+        <v>SGL 04</v>
       </c>
       <c r="B183">
         <v>539</v>
@@ -11567,7 +11567,7 @@
     </row>
     <row r="184">
       <c r="A184" t="str">
-        <v>SGL 09</v>
+        <v>SGL 04</v>
       </c>
       <c r="B184">
         <v>539</v>
@@ -11632,7 +11632,7 @@
     </row>
     <row r="185">
       <c r="A185" t="str">
-        <v>SGL 09</v>
+        <v>SGL 04</v>
       </c>
       <c r="C185" t="str">
         <v>240754::SGSGMADWL2702::JK</v>
@@ -11662,7 +11662,7 @@
         <v>46174</v>
       </c>
       <c r="T185">
-        <v>46192</v>
+        <v>46193</v>
       </c>
       <c r="W185">
         <v>46181</v>
@@ -14728,7 +14728,7 @@
     </row>
     <row r="245">
       <c r="A245" t="str">
-        <v>SGL 09</v>
+        <v>SGL 04</v>
       </c>
       <c r="B245">
         <v>547</v>
@@ -14790,7 +14790,7 @@
     </row>
     <row r="246">
       <c r="A246" t="str">
-        <v>SGL 09</v>
+        <v>SGL 04</v>
       </c>
       <c r="C246" t="str">
         <v>558845X::OVOVLE-BO4518::BZ</v>
@@ -14817,10 +14817,10 @@
         <v>46231</v>
       </c>
       <c r="S246">
-        <v>46244</v>
+        <v>46233</v>
       </c>
       <c r="T246">
-        <v>46245</v>
+        <v>46235</v>
       </c>
       <c r="W246">
         <v>46247</v>
@@ -19814,7 +19814,7 @@
     </row>
     <row r="340">
       <c r="A340" t="str">
-        <v>SGL 08</v>
+        <v>SGL 05</v>
       </c>
       <c r="B340">
         <v>847</v>
@@ -19873,7 +19873,7 @@
     </row>
     <row r="341">
       <c r="A341" t="str">
-        <v>SGL 08</v>
+        <v>SGL 05</v>
       </c>
       <c r="B341">
         <v>847</v>
@@ -19932,7 +19932,7 @@
     </row>
     <row r="342">
       <c r="A342" t="str">
-        <v>SGL 08</v>
+        <v>SGL 05</v>
       </c>
       <c r="C342" t="str">
         <v>INQZIM RS27 DRS</v>
@@ -19959,7 +19959,7 @@
         <v>46258</v>
       </c>
       <c r="S342">
-        <v>46288</v>
+        <v>46260</v>
       </c>
       <c r="T342">
         <v>46290</v>

</xml_diff>

<commit_message>
SGL FR Plan — 03/06/2026 11:29
</commit_message>
<xml_diff>
--- a/Production_Plan.xlsx
+++ b/Production_Plan.xlsx
@@ -1370,7 +1370,7 @@
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="B16">
         <v>847</v>
@@ -1438,7 +1438,7 @@
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="B17">
         <v>847</v>
@@ -1506,7 +1506,7 @@
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="B18">
         <v>847</v>
@@ -1574,7 +1574,7 @@
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="B19">
         <v>847</v>
@@ -1642,7 +1642,7 @@
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="B20">
         <v>847</v>
@@ -1710,7 +1710,7 @@
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="B21">
         <v>847</v>
@@ -1778,7 +1778,7 @@
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="B22">
         <v>847</v>
@@ -1846,7 +1846,7 @@
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="B23">
         <v>847</v>
@@ -1914,7 +1914,7 @@
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="B24">
         <v>847</v>
@@ -1982,7 +1982,7 @@
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="B25">
         <v>847</v>
@@ -2050,7 +2050,7 @@
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="B26">
         <v>847</v>
@@ -2118,7 +2118,7 @@
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="B27">
         <v>847</v>
@@ -2186,7 +2186,7 @@
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="C28" t="str">
         <v>9676T::SGSGZIMER4233::BL</v>
@@ -2213,10 +2213,10 @@
         <v>-</v>
       </c>
       <c r="S28">
-        <v>46170</v>
+        <v>46204</v>
       </c>
       <c r="T28">
-        <v>46179</v>
+        <v>46213</v>
       </c>
       <c r="V28" t="str">
         <v>1675 Dinusha Guantillake</v>

</xml_diff>

<commit_message>
SGL FR Plan — 03/06/2026 11:45
</commit_message>
<xml_diff>
--- a/Production_Plan.xlsx
+++ b/Production_Plan.xlsx
@@ -32,8 +32,20 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
-  <numFmts count="1">
+  <numFmts count="13">
+    <numFmt numFmtId="5" formatCode="&quot;$&quot;#,##0_);\(&quot;$&quot;#,##0\)"/>
+    <numFmt numFmtId="6" formatCode="&quot;$&quot;#,##0_);[Red]\(&quot;$&quot;#,##0\)"/>
+    <numFmt numFmtId="7" formatCode="&quot;$&quot;#,##0.00_);\(&quot;$&quot;#,##0.00\)"/>
+    <numFmt numFmtId="8" formatCode="&quot;$&quot;#,##0.00_);[Red]\(&quot;$&quot;#,##0.00\)"/>
+    <numFmt numFmtId="41" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;_);_(@_)"/>
+    <numFmt numFmtId="42" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;_);_(@_)"/>
+    <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="56" formatCode="&quot;上午/下午 &quot;hh&quot;時&quot;mm&quot;分&quot;ss&quot;秒 &quot;"/>
+    <numFmt numFmtId="164" formatCode="_(&quot;$&quot;#,##0_);\(&quot;$&quot;#,##0\)"/>
+    <numFmt numFmtId="165" formatCode="_(&quot;$&quot;#,##0_);[Red]\(&quot;$&quot;#,##0\)"/>
+    <numFmt numFmtId="166" formatCode="_(&quot;$&quot;#,##0.00_);\(&quot;$&quot;#,##0.00\)"/>
+    <numFmt numFmtId="167" formatCode="_(&quot;$&quot;#,##0.00_);[Red]\(&quot;$&quot;#,##0.00\)"/>
   </numFmts>
   <fonts count="1">
     <font>
@@ -1370,7 +1382,7 @@
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>SGL 02</v>
+        <v>SGL 01</v>
       </c>
       <c r="B16">
         <v>847</v>
@@ -1438,7 +1450,7 @@
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>SGL 02</v>
+        <v>SGL 01</v>
       </c>
       <c r="B17">
         <v>847</v>
@@ -1506,7 +1518,7 @@
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>SGL 02</v>
+        <v>SGL 01</v>
       </c>
       <c r="B18">
         <v>847</v>
@@ -1574,7 +1586,7 @@
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>SGL 02</v>
+        <v>SGL 01</v>
       </c>
       <c r="B19">
         <v>847</v>
@@ -1642,7 +1654,7 @@
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>SGL 02</v>
+        <v>SGL 01</v>
       </c>
       <c r="B20">
         <v>847</v>
@@ -1710,7 +1722,7 @@
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>SGL 02</v>
+        <v>SGL 01</v>
       </c>
       <c r="B21">
         <v>847</v>
@@ -1778,7 +1790,7 @@
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>SGL 02</v>
+        <v>SGL 01</v>
       </c>
       <c r="B22">
         <v>847</v>
@@ -1846,7 +1858,7 @@
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>SGL 02</v>
+        <v>SGL 01</v>
       </c>
       <c r="B23">
         <v>847</v>
@@ -1914,7 +1926,7 @@
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>SGL 02</v>
+        <v>SGL 01</v>
       </c>
       <c r="B24">
         <v>847</v>
@@ -1982,7 +1994,7 @@
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>SGL 02</v>
+        <v>SGL 01</v>
       </c>
       <c r="B25">
         <v>847</v>
@@ -2050,7 +2062,7 @@
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>SGL 02</v>
+        <v>SGL 01</v>
       </c>
       <c r="B26">
         <v>847</v>
@@ -2118,7 +2130,7 @@
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>SGL 02</v>
+        <v>SGL 01</v>
       </c>
       <c r="B27">
         <v>847</v>
@@ -2186,7 +2198,7 @@
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>SGL 02</v>
+        <v>SGL 01</v>
       </c>
       <c r="C28" t="str">
         <v>9676T::SGSGZIMER4233::BL</v>
@@ -2213,10 +2225,10 @@
         <v>-</v>
       </c>
       <c r="S28">
-        <v>46204</v>
+        <v>46171</v>
       </c>
       <c r="T28">
-        <v>46212</v>
+        <v>46179</v>
       </c>
       <c r="V28" t="str">
         <v>1675 Dinusha Guantillake</v>

</xml_diff>

<commit_message>
SGL FR Plan — 03/06/2026 12:24
</commit_message>
<xml_diff>
--- a/Production_Plan.xlsx
+++ b/Production_Plan.xlsx
@@ -1382,7 +1382,7 @@
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="B16">
         <v>847</v>
@@ -1450,7 +1450,7 @@
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="B17">
         <v>847</v>
@@ -1518,7 +1518,7 @@
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="B18">
         <v>847</v>
@@ -1586,7 +1586,7 @@
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="B19">
         <v>847</v>
@@ -1654,7 +1654,7 @@
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="B20">
         <v>847</v>
@@ -1722,7 +1722,7 @@
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="B21">
         <v>847</v>
@@ -1790,7 +1790,7 @@
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="B22">
         <v>847</v>
@@ -1858,7 +1858,7 @@
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="B23">
         <v>847</v>
@@ -1926,7 +1926,7 @@
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="B24">
         <v>847</v>
@@ -1994,7 +1994,7 @@
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="B25">
         <v>847</v>
@@ -2062,7 +2062,7 @@
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="B26">
         <v>847</v>
@@ -2130,7 +2130,7 @@
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="B27">
         <v>847</v>
@@ -2198,7 +2198,7 @@
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="C28" t="str">
         <v>9676T::SGSGZIMER4233::BL</v>
@@ -2225,10 +2225,10 @@
         <v>-</v>
       </c>
       <c r="S28">
-        <v>46171</v>
+        <v>46204</v>
       </c>
       <c r="T28">
-        <v>46179</v>
+        <v>46212</v>
       </c>
       <c r="V28" t="str">
         <v>1675 Dinusha Guantillake</v>

</xml_diff>

<commit_message>
SGL FR Plan — 03/06/2026 13:47
</commit_message>
<xml_diff>
--- a/Production_Plan.xlsx
+++ b/Production_Plan.xlsx
@@ -409,7 +409,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:W526"/>
+  <dimension ref="A1:X526"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -481,6 +481,9 @@
       <c r="W1" t="str">
         <v>Del Date</v>
       </c>
+      <c r="X1" t="str">
+        <v>SGL_MergeGroup</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -1382,7 +1385,7 @@
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>SGL 02</v>
+        <v>SGL 01</v>
       </c>
       <c r="B16">
         <v>847</v>
@@ -1450,7 +1453,7 @@
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>SGL 02</v>
+        <v>SGL 01</v>
       </c>
       <c r="B17">
         <v>847</v>
@@ -1518,7 +1521,7 @@
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>SGL 02</v>
+        <v>SGL 01</v>
       </c>
       <c r="B18">
         <v>847</v>
@@ -1586,7 +1589,7 @@
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>SGL 02</v>
+        <v>SGL 01</v>
       </c>
       <c r="B19">
         <v>847</v>
@@ -1654,7 +1657,7 @@
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>SGL 02</v>
+        <v>SGL 01</v>
       </c>
       <c r="B20">
         <v>847</v>
@@ -1722,7 +1725,7 @@
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>SGL 02</v>
+        <v>SGL 01</v>
       </c>
       <c r="B21">
         <v>847</v>
@@ -1790,7 +1793,7 @@
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>SGL 02</v>
+        <v>SGL 01</v>
       </c>
       <c r="B22">
         <v>847</v>
@@ -1858,7 +1861,7 @@
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>SGL 02</v>
+        <v>SGL 01</v>
       </c>
       <c r="B23">
         <v>847</v>
@@ -1926,7 +1929,7 @@
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>SGL 02</v>
+        <v>SGL 01</v>
       </c>
       <c r="B24">
         <v>847</v>
@@ -1994,7 +1997,7 @@
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>SGL 02</v>
+        <v>SGL 01</v>
       </c>
       <c r="B25">
         <v>847</v>
@@ -2062,7 +2065,7 @@
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>SGL 02</v>
+        <v>SGL 01</v>
       </c>
       <c r="B26">
         <v>847</v>
@@ -2130,7 +2133,7 @@
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>SGL 02</v>
+        <v>SGL 01</v>
       </c>
       <c r="B27">
         <v>847</v>
@@ -2198,7 +2201,7 @@
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>SGL 02</v>
+        <v>SGL 01</v>
       </c>
       <c r="C28" t="str">
         <v>9676T::SGSGZIMER4233::BL</v>
@@ -2225,10 +2228,10 @@
         <v>-</v>
       </c>
       <c r="S28">
-        <v>46204</v>
+        <v>46171</v>
       </c>
       <c r="T28">
-        <v>46212</v>
+        <v>46179</v>
       </c>
       <c r="V28" t="str">
         <v>1675 Dinusha Guantillake</v>
@@ -30310,7 +30313,7 @@
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:W526"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:X526"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
SGL FR Plan — 03/06/2026 13:49
</commit_message>
<xml_diff>
--- a/Production_Plan.xlsx
+++ b/Production_Plan.xlsx
@@ -10997,6 +10997,9 @@
       <c r="W174">
         <v>46205</v>
       </c>
+      <c r="X174" t="str">
+        <v>MG-7utvvn</v>
+      </c>
     </row>
     <row r="175">
       <c r="A175" t="str">
@@ -11065,6 +11068,9 @@
       <c r="W175">
         <v>46205</v>
       </c>
+      <c r="X175" t="str">
+        <v>MG-7utvvn</v>
+      </c>
     </row>
     <row r="176">
       <c r="A176" t="str">
@@ -11106,6 +11112,9 @@
       <c r="W176">
         <v>46205</v>
       </c>
+      <c r="X176" t="str">
+        <v>MG-7utvvn</v>
+      </c>
     </row>
     <row r="177">
       <c r="A177" t="str">
@@ -11174,6 +11183,9 @@
       <c r="W177">
         <v>46205</v>
       </c>
+      <c r="X177" t="str">
+        <v>MG-7utvvn</v>
+      </c>
     </row>
     <row r="178">
       <c r="A178" t="str">
@@ -11215,6 +11227,9 @@
       <c r="W178">
         <v>46205</v>
       </c>
+      <c r="X178" t="str">
+        <v>MG-7utvvn</v>
+      </c>
     </row>
     <row r="179">
       <c r="A179" t="str">
@@ -11283,6 +11298,9 @@
       <c r="W179">
         <v>46205</v>
       </c>
+      <c r="X179" t="str">
+        <v>MG-7utvvn</v>
+      </c>
     </row>
     <row r="180">
       <c r="A180" t="str">
@@ -11323,6 +11341,9 @@
       </c>
       <c r="W180">
         <v>46205</v>
+      </c>
+      <c r="X180" t="str">
+        <v>MG-7utvvn</v>
       </c>
     </row>
     <row r="181">

</xml_diff>

<commit_message>
SGL FR Plan — 03/06/2026 14:08
</commit_message>
<xml_diff>
--- a/Production_Plan.xlsx
+++ b/Production_Plan.xlsx
@@ -10932,7 +10932,7 @@
     </row>
     <row r="174">
       <c r="A174" t="str">
-        <v>SGL 04</v>
+        <v>SGL 02</v>
       </c>
       <c r="B174">
         <v>212</v>
@@ -10998,12 +10998,12 @@
         <v>46205</v>
       </c>
       <c r="X174" t="str">
-        <v>MG-7utvvn</v>
+        <v>MG-e8x14v</v>
       </c>
     </row>
     <row r="175">
       <c r="A175" t="str">
-        <v>SGL 04</v>
+        <v>SGL 02</v>
       </c>
       <c r="B175">
         <v>212</v>
@@ -11069,12 +11069,12 @@
         <v>46205</v>
       </c>
       <c r="X175" t="str">
-        <v>MG-7utvvn</v>
+        <v>MG-e8x14v</v>
       </c>
     </row>
     <row r="176">
       <c r="A176" t="str">
-        <v>SGL 04</v>
+        <v>SGL 02</v>
       </c>
       <c r="C176" t="str">
         <v>556959R/R1::OVOVLANED3016::FJK</v>
@@ -11101,10 +11101,10 @@
         <v>46191</v>
       </c>
       <c r="S176">
-        <v>46193</v>
+        <v>46204</v>
       </c>
       <c r="T176">
-        <v>46198</v>
+        <v>46207</v>
       </c>
       <c r="V176" t="str">
         <v>710 Shimara Himahansi</v>
@@ -11113,12 +11113,12 @@
         <v>46205</v>
       </c>
       <c r="X176" t="str">
-        <v>MG-7utvvn</v>
+        <v>MG-e8x14v</v>
       </c>
     </row>
     <row r="177">
       <c r="A177" t="str">
-        <v>SGL 04</v>
+        <v>SGL 02</v>
       </c>
       <c r="B177">
         <v>212</v>
@@ -11184,12 +11184,12 @@
         <v>46205</v>
       </c>
       <c r="X177" t="str">
-        <v>MG-7utvvn</v>
+        <v>MG-e8x14v</v>
       </c>
     </row>
     <row r="178">
       <c r="A178" t="str">
-        <v>SGL 04</v>
+        <v>SGL 02</v>
       </c>
       <c r="C178" t="str">
         <v>556959S/R1::OVOVLANED3017::FJK</v>
@@ -11216,10 +11216,10 @@
         <v>46196</v>
       </c>
       <c r="S178">
-        <v>46198</v>
+        <v>46209</v>
       </c>
       <c r="T178">
-        <v>46199</v>
+        <v>46209</v>
       </c>
       <c r="V178" t="str">
         <v>710 Shimara Himahansi</v>
@@ -11228,12 +11228,12 @@
         <v>46205</v>
       </c>
       <c r="X178" t="str">
-        <v>MG-7utvvn</v>
+        <v>MG-e8x14v</v>
       </c>
     </row>
     <row r="179">
       <c r="A179" t="str">
-        <v>SGL 04</v>
+        <v>SGL 02</v>
       </c>
       <c r="B179">
         <v>212</v>
@@ -11299,12 +11299,12 @@
         <v>46205</v>
       </c>
       <c r="X179" t="str">
-        <v>MG-7utvvn</v>
+        <v>MG-e8x14v</v>
       </c>
     </row>
     <row r="180">
       <c r="A180" t="str">
-        <v>SGL 04</v>
+        <v>SGL 02</v>
       </c>
       <c r="C180" t="str">
         <v>556959L/R1::OVOVLANED3018::FJK</v>
@@ -11331,10 +11331,10 @@
         <v>46197</v>
       </c>
       <c r="S180">
-        <v>46199</v>
+        <v>46210</v>
       </c>
       <c r="T180">
-        <v>46199</v>
+        <v>46210</v>
       </c>
       <c r="V180" t="str">
         <v>710 Shimara Himahansi</v>
@@ -11343,7 +11343,7 @@
         <v>46205</v>
       </c>
       <c r="X180" t="str">
-        <v>MG-7utvvn</v>
+        <v>MG-e8x14v</v>
       </c>
     </row>
     <row r="181">

</xml_diff>

<commit_message>
SGL FR Plan — 03/06/2026 14:23
</commit_message>
<xml_diff>
--- a/Production_Plan.xlsx
+++ b/Production_Plan.xlsx
@@ -10997,9 +10997,6 @@
       <c r="W174">
         <v>46205</v>
       </c>
-      <c r="X174" t="str">
-        <v>MG-e8x14v</v>
-      </c>
     </row>
     <row r="175">
       <c r="A175" t="str">
@@ -11068,9 +11065,6 @@
       <c r="W175">
         <v>46205</v>
       </c>
-      <c r="X175" t="str">
-        <v>MG-e8x14v</v>
-      </c>
     </row>
     <row r="176">
       <c r="A176" t="str">
@@ -11112,9 +11106,6 @@
       <c r="W176">
         <v>46205</v>
       </c>
-      <c r="X176" t="str">
-        <v>MG-e8x14v</v>
-      </c>
     </row>
     <row r="177">
       <c r="A177" t="str">
@@ -11183,9 +11174,6 @@
       <c r="W177">
         <v>46205</v>
       </c>
-      <c r="X177" t="str">
-        <v>MG-e8x14v</v>
-      </c>
     </row>
     <row r="178">
       <c r="A178" t="str">
@@ -11227,9 +11215,6 @@
       <c r="W178">
         <v>46205</v>
       </c>
-      <c r="X178" t="str">
-        <v>MG-e8x14v</v>
-      </c>
     </row>
     <row r="179">
       <c r="A179" t="str">
@@ -11298,9 +11283,6 @@
       <c r="W179">
         <v>46205</v>
       </c>
-      <c r="X179" t="str">
-        <v>MG-e8x14v</v>
-      </c>
     </row>
     <row r="180">
       <c r="A180" t="str">
@@ -11341,9 +11323,6 @@
       </c>
       <c r="W180">
         <v>46205</v>
-      </c>
-      <c r="X180" t="str">
-        <v>MG-e8x14v</v>
       </c>
     </row>
     <row r="181">

</xml_diff>

<commit_message>
SGL FR Plan — 04/06/2026 09:37
</commit_message>
<xml_diff>
--- a/Production_Plan.xlsx
+++ b/Production_Plan.xlsx
@@ -1385,7 +1385,7 @@
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="B16">
         <v>847</v>
@@ -1453,7 +1453,7 @@
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="B17">
         <v>847</v>
@@ -1521,7 +1521,7 @@
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="B18">
         <v>847</v>
@@ -1589,7 +1589,7 @@
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="B19">
         <v>847</v>
@@ -1657,7 +1657,7 @@
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="B20">
         <v>847</v>
@@ -1725,7 +1725,7 @@
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="B21">
         <v>847</v>
@@ -1793,7 +1793,7 @@
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="B22">
         <v>847</v>
@@ -1861,7 +1861,7 @@
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="B23">
         <v>847</v>
@@ -1929,7 +1929,7 @@
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="B24">
         <v>847</v>
@@ -1997,7 +1997,7 @@
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="B25">
         <v>847</v>
@@ -2065,7 +2065,7 @@
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="B26">
         <v>847</v>
@@ -2133,7 +2133,7 @@
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="B27">
         <v>847</v>
@@ -2201,7 +2201,7 @@
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="C28" t="str">
         <v>9676T::SGSGZIMER4233::BL</v>
@@ -2228,10 +2228,10 @@
         <v>-</v>
       </c>
       <c r="S28">
-        <v>46171</v>
+        <v>46211</v>
       </c>
       <c r="T28">
-        <v>46179</v>
+        <v>46219</v>
       </c>
       <c r="V28" t="str">
         <v>1675 Dinusha Guantillake</v>

</xml_diff>

<commit_message>
SGL FR Plan — 04/06/2026 09:38
</commit_message>
<xml_diff>
--- a/Production_Plan.xlsx
+++ b/Production_Plan.xlsx
@@ -1385,7 +1385,7 @@
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>SGL 02</v>
+        <v>SGL 01</v>
       </c>
       <c r="B16">
         <v>847</v>
@@ -1453,7 +1453,7 @@
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>SGL 02</v>
+        <v>SGL 01</v>
       </c>
       <c r="B17">
         <v>847</v>
@@ -1521,7 +1521,7 @@
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>SGL 02</v>
+        <v>SGL 01</v>
       </c>
       <c r="B18">
         <v>847</v>
@@ -1589,7 +1589,7 @@
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>SGL 02</v>
+        <v>SGL 01</v>
       </c>
       <c r="B19">
         <v>847</v>
@@ -1657,7 +1657,7 @@
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>SGL 02</v>
+        <v>SGL 01</v>
       </c>
       <c r="B20">
         <v>847</v>
@@ -1725,7 +1725,7 @@
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>SGL 02</v>
+        <v>SGL 01</v>
       </c>
       <c r="B21">
         <v>847</v>
@@ -1793,7 +1793,7 @@
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>SGL 02</v>
+        <v>SGL 01</v>
       </c>
       <c r="B22">
         <v>847</v>
@@ -1861,7 +1861,7 @@
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>SGL 02</v>
+        <v>SGL 01</v>
       </c>
       <c r="B23">
         <v>847</v>
@@ -1929,7 +1929,7 @@
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>SGL 02</v>
+        <v>SGL 01</v>
       </c>
       <c r="B24">
         <v>847</v>
@@ -1997,7 +1997,7 @@
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>SGL 02</v>
+        <v>SGL 01</v>
       </c>
       <c r="B25">
         <v>847</v>
@@ -2065,7 +2065,7 @@
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>SGL 02</v>
+        <v>SGL 01</v>
       </c>
       <c r="B26">
         <v>847</v>
@@ -2133,7 +2133,7 @@
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>SGL 02</v>
+        <v>SGL 01</v>
       </c>
       <c r="B27">
         <v>847</v>
@@ -2201,7 +2201,7 @@
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>SGL 02</v>
+        <v>SGL 01</v>
       </c>
       <c r="C28" t="str">
         <v>9676T::SGSGZIMER4233::BL</v>
@@ -2228,10 +2228,10 @@
         <v>-</v>
       </c>
       <c r="S28">
-        <v>46211</v>
+        <v>46171</v>
       </c>
       <c r="T28">
-        <v>46219</v>
+        <v>46179</v>
       </c>
       <c r="V28" t="str">
         <v>1675 Dinusha Guantillake</v>

</xml_diff>

<commit_message>
SGL FR Plan — 04/06/2026 09:53
</commit_message>
<xml_diff>
--- a/Production_Plan.xlsx
+++ b/Production_Plan.xlsx
@@ -1385,7 +1385,7 @@
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="B16">
         <v>847</v>
@@ -1453,7 +1453,7 @@
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="B17">
         <v>847</v>
@@ -1521,7 +1521,7 @@
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="B18">
         <v>847</v>
@@ -1589,7 +1589,7 @@
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="B19">
         <v>847</v>
@@ -1657,7 +1657,7 @@
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="B20">
         <v>847</v>
@@ -1725,7 +1725,7 @@
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="B21">
         <v>847</v>
@@ -1793,7 +1793,7 @@
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="B22">
         <v>847</v>
@@ -1861,7 +1861,7 @@
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="B23">
         <v>847</v>
@@ -1929,7 +1929,7 @@
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="B24">
         <v>847</v>
@@ -1997,7 +1997,7 @@
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="B25">
         <v>847</v>
@@ -2065,7 +2065,7 @@
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="B26">
         <v>847</v>
@@ -2133,7 +2133,7 @@
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="B27">
         <v>847</v>
@@ -2201,7 +2201,7 @@
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="C28" t="str">
         <v>9676T::SGSGZIMER4233::BL</v>
@@ -2228,10 +2228,10 @@
         <v>-</v>
       </c>
       <c r="S28">
-        <v>46171</v>
+        <v>46211</v>
       </c>
       <c r="T28">
-        <v>46179</v>
+        <v>46219</v>
       </c>
       <c r="V28" t="str">
         <v>1675 Dinusha Guantillake</v>

</xml_diff>

<commit_message>
SGL FR Plan — 04/06/2026 09:56
</commit_message>
<xml_diff>
--- a/Production_Plan.xlsx
+++ b/Production_Plan.xlsx
@@ -1385,7 +1385,7 @@
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>SGL 02</v>
+        <v>SGL 01</v>
       </c>
       <c r="B16">
         <v>847</v>
@@ -1453,7 +1453,7 @@
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>SGL 02</v>
+        <v>SGL 01</v>
       </c>
       <c r="B17">
         <v>847</v>
@@ -1521,7 +1521,7 @@
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>SGL 02</v>
+        <v>SGL 01</v>
       </c>
       <c r="B18">
         <v>847</v>
@@ -1589,7 +1589,7 @@
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>SGL 02</v>
+        <v>SGL 01</v>
       </c>
       <c r="B19">
         <v>847</v>
@@ -1657,7 +1657,7 @@
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>SGL 02</v>
+        <v>SGL 01</v>
       </c>
       <c r="B20">
         <v>847</v>
@@ -1725,7 +1725,7 @@
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>SGL 02</v>
+        <v>SGL 01</v>
       </c>
       <c r="B21">
         <v>847</v>
@@ -1793,7 +1793,7 @@
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>SGL 02</v>
+        <v>SGL 01</v>
       </c>
       <c r="B22">
         <v>847</v>
@@ -1861,7 +1861,7 @@
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>SGL 02</v>
+        <v>SGL 01</v>
       </c>
       <c r="B23">
         <v>847</v>
@@ -1929,7 +1929,7 @@
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>SGL 02</v>
+        <v>SGL 01</v>
       </c>
       <c r="B24">
         <v>847</v>
@@ -1997,7 +1997,7 @@
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>SGL 02</v>
+        <v>SGL 01</v>
       </c>
       <c r="B25">
         <v>847</v>
@@ -2065,7 +2065,7 @@
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>SGL 02</v>
+        <v>SGL 01</v>
       </c>
       <c r="B26">
         <v>847</v>
@@ -2133,7 +2133,7 @@
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>SGL 02</v>
+        <v>SGL 01</v>
       </c>
       <c r="B27">
         <v>847</v>
@@ -2201,7 +2201,7 @@
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>SGL 02</v>
+        <v>SGL 01</v>
       </c>
       <c r="C28" t="str">
         <v>9676T::SGSGZIMER4233::BL</v>
@@ -2228,10 +2228,10 @@
         <v>-</v>
       </c>
       <c r="S28">
-        <v>46211</v>
+        <v>46171</v>
       </c>
       <c r="T28">
-        <v>46219</v>
+        <v>46179</v>
       </c>
       <c r="V28" t="str">
         <v>1675 Dinusha Guantillake</v>

</xml_diff>

<commit_message>
SGL FR Plan — 04/06/2026 10:01
</commit_message>
<xml_diff>
--- a/Production_Plan.xlsx
+++ b/Production_Plan.xlsx
@@ -1385,7 +1385,7 @@
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="B16">
         <v>847</v>
@@ -1453,7 +1453,7 @@
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="B17">
         <v>847</v>
@@ -1521,7 +1521,7 @@
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="B18">
         <v>847</v>
@@ -1589,7 +1589,7 @@
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="B19">
         <v>847</v>
@@ -1657,7 +1657,7 @@
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="B20">
         <v>847</v>
@@ -1725,7 +1725,7 @@
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="B21">
         <v>847</v>
@@ -1793,7 +1793,7 @@
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="B22">
         <v>847</v>
@@ -1861,7 +1861,7 @@
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="B23">
         <v>847</v>
@@ -1929,7 +1929,7 @@
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="B24">
         <v>847</v>
@@ -1997,7 +1997,7 @@
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="B25">
         <v>847</v>
@@ -2065,7 +2065,7 @@
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="B26">
         <v>847</v>
@@ -2133,7 +2133,7 @@
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="B27">
         <v>847</v>
@@ -2201,7 +2201,7 @@
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="C28" t="str">
         <v>9676T::SGSGZIMER4233::BL</v>
@@ -2228,10 +2228,10 @@
         <v>-</v>
       </c>
       <c r="S28">
-        <v>46171</v>
+        <v>46211</v>
       </c>
       <c r="T28">
-        <v>46179</v>
+        <v>46219</v>
       </c>
       <c r="V28" t="str">
         <v>1675 Dinusha Guantillake</v>

</xml_diff>

<commit_message>
SGL FR Plan — 04/06/2026 10:06
</commit_message>
<xml_diff>
--- a/Production_Plan.xlsx
+++ b/Production_Plan.xlsx
@@ -1385,7 +1385,7 @@
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>SGL 02</v>
+        <v>SGL 01</v>
       </c>
       <c r="B16">
         <v>847</v>
@@ -1453,7 +1453,7 @@
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>SGL 02</v>
+        <v>SGL 01</v>
       </c>
       <c r="B17">
         <v>847</v>
@@ -1521,7 +1521,7 @@
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>SGL 02</v>
+        <v>SGL 01</v>
       </c>
       <c r="B18">
         <v>847</v>
@@ -1589,7 +1589,7 @@
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>SGL 02</v>
+        <v>SGL 01</v>
       </c>
       <c r="B19">
         <v>847</v>
@@ -1657,7 +1657,7 @@
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>SGL 02</v>
+        <v>SGL 01</v>
       </c>
       <c r="B20">
         <v>847</v>
@@ -1725,7 +1725,7 @@
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>SGL 02</v>
+        <v>SGL 01</v>
       </c>
       <c r="B21">
         <v>847</v>
@@ -1793,7 +1793,7 @@
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>SGL 02</v>
+        <v>SGL 01</v>
       </c>
       <c r="B22">
         <v>847</v>
@@ -1861,7 +1861,7 @@
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>SGL 02</v>
+        <v>SGL 01</v>
       </c>
       <c r="B23">
         <v>847</v>
@@ -1929,7 +1929,7 @@
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>SGL 02</v>
+        <v>SGL 01</v>
       </c>
       <c r="B24">
         <v>847</v>
@@ -1997,7 +1997,7 @@
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>SGL 02</v>
+        <v>SGL 01</v>
       </c>
       <c r="B25">
         <v>847</v>
@@ -2065,7 +2065,7 @@
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>SGL 02</v>
+        <v>SGL 01</v>
       </c>
       <c r="B26">
         <v>847</v>
@@ -2133,7 +2133,7 @@
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>SGL 02</v>
+        <v>SGL 01</v>
       </c>
       <c r="B27">
         <v>847</v>
@@ -2201,7 +2201,7 @@
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>SGL 02</v>
+        <v>SGL 01</v>
       </c>
       <c r="C28" t="str">
         <v>9676T::SGSGZIMER4233::BL</v>
@@ -2228,10 +2228,10 @@
         <v>-</v>
       </c>
       <c r="S28">
-        <v>46211</v>
+        <v>46171</v>
       </c>
       <c r="T28">
-        <v>46219</v>
+        <v>46179</v>
       </c>
       <c r="V28" t="str">
         <v>1675 Dinusha Guantillake</v>

</xml_diff>

<commit_message>
SGL FR Plan — 04/06/2026 10:13
</commit_message>
<xml_diff>
--- a/Production_Plan.xlsx
+++ b/Production_Plan.xlsx
@@ -1385,7 +1385,7 @@
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="B16">
         <v>847</v>
@@ -1453,7 +1453,7 @@
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="B17">
         <v>847</v>
@@ -1521,7 +1521,7 @@
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="B18">
         <v>847</v>
@@ -1589,7 +1589,7 @@
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="B19">
         <v>847</v>
@@ -1657,7 +1657,7 @@
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="B20">
         <v>847</v>
@@ -1725,7 +1725,7 @@
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="B21">
         <v>847</v>
@@ -1793,7 +1793,7 @@
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="B22">
         <v>847</v>
@@ -1861,7 +1861,7 @@
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="B23">
         <v>847</v>
@@ -1929,7 +1929,7 @@
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="B24">
         <v>847</v>
@@ -1997,7 +1997,7 @@
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="B25">
         <v>847</v>
@@ -2065,7 +2065,7 @@
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="B26">
         <v>847</v>
@@ -2133,7 +2133,7 @@
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="B27">
         <v>847</v>
@@ -2201,7 +2201,7 @@
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="C28" t="str">
         <v>9676T::SGSGZIMER4233::BL</v>
@@ -2228,10 +2228,10 @@
         <v>-</v>
       </c>
       <c r="S28">
-        <v>46171</v>
+        <v>46211</v>
       </c>
       <c r="T28">
-        <v>46179</v>
+        <v>46219</v>
       </c>
       <c r="V28" t="str">
         <v>1675 Dinusha Guantillake</v>

</xml_diff>

<commit_message>
SGL FR Plan — 04/06/2026 10:17
</commit_message>
<xml_diff>
--- a/Production_Plan.xlsx
+++ b/Production_Plan.xlsx
@@ -1385,7 +1385,7 @@
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="B16">
         <v>847</v>
@@ -1453,7 +1453,7 @@
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="B17">
         <v>847</v>
@@ -1521,7 +1521,7 @@
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="B18">
         <v>847</v>
@@ -1589,7 +1589,7 @@
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="B19">
         <v>847</v>
@@ -1657,7 +1657,7 @@
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="B20">
         <v>847</v>
@@ -1725,7 +1725,7 @@
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="B21">
         <v>847</v>
@@ -1793,7 +1793,7 @@
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="B22">
         <v>847</v>
@@ -1861,7 +1861,7 @@
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="B23">
         <v>847</v>
@@ -1929,7 +1929,7 @@
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="B24">
         <v>847</v>
@@ -1997,7 +1997,7 @@
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="B25">
         <v>847</v>
@@ -2065,7 +2065,7 @@
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="B26">
         <v>847</v>
@@ -2133,7 +2133,7 @@
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="B27">
         <v>847</v>
@@ -2201,7 +2201,7 @@
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="C28" t="str">
         <v>9676T::SGSGZIMER4233::BL</v>
@@ -2228,10 +2228,10 @@
         <v>-</v>
       </c>
       <c r="S28">
-        <v>46171</v>
+        <v>46210</v>
       </c>
       <c r="T28">
-        <v>46179</v>
+        <v>46218</v>
       </c>
       <c r="V28" t="str">
         <v>1675 Dinusha Guantillake</v>

</xml_diff>

<commit_message>
SGL FR Plan — 04/06/2026 10:21
</commit_message>
<xml_diff>
--- a/Production_Plan.xlsx
+++ b/Production_Plan.xlsx
@@ -1385,7 +1385,7 @@
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>SGL 02</v>
+        <v>SGL 01</v>
       </c>
       <c r="B16">
         <v>847</v>
@@ -1453,7 +1453,7 @@
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>SGL 02</v>
+        <v>SGL 01</v>
       </c>
       <c r="B17">
         <v>847</v>
@@ -1521,7 +1521,7 @@
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>SGL 02</v>
+        <v>SGL 01</v>
       </c>
       <c r="B18">
         <v>847</v>
@@ -1589,7 +1589,7 @@
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>SGL 02</v>
+        <v>SGL 01</v>
       </c>
       <c r="B19">
         <v>847</v>
@@ -1657,7 +1657,7 @@
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>SGL 02</v>
+        <v>SGL 01</v>
       </c>
       <c r="B20">
         <v>847</v>
@@ -1725,7 +1725,7 @@
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>SGL 02</v>
+        <v>SGL 01</v>
       </c>
       <c r="B21">
         <v>847</v>
@@ -1793,7 +1793,7 @@
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>SGL 02</v>
+        <v>SGL 01</v>
       </c>
       <c r="B22">
         <v>847</v>
@@ -1861,7 +1861,7 @@
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>SGL 02</v>
+        <v>SGL 01</v>
       </c>
       <c r="B23">
         <v>847</v>
@@ -1929,7 +1929,7 @@
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>SGL 02</v>
+        <v>SGL 01</v>
       </c>
       <c r="B24">
         <v>847</v>
@@ -1997,7 +1997,7 @@
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>SGL 02</v>
+        <v>SGL 01</v>
       </c>
       <c r="B25">
         <v>847</v>
@@ -2065,7 +2065,7 @@
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>SGL 02</v>
+        <v>SGL 01</v>
       </c>
       <c r="B26">
         <v>847</v>
@@ -2133,7 +2133,7 @@
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>SGL 02</v>
+        <v>SGL 01</v>
       </c>
       <c r="B27">
         <v>847</v>
@@ -2201,7 +2201,7 @@
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>SGL 02</v>
+        <v>SGL 01</v>
       </c>
       <c r="C28" t="str">
         <v>9676T::SGSGZIMER4233::BL</v>
@@ -2228,10 +2228,10 @@
         <v>-</v>
       </c>
       <c r="S28">
-        <v>46210</v>
+        <v>46171</v>
       </c>
       <c r="T28">
-        <v>46218</v>
+        <v>46179</v>
       </c>
       <c r="V28" t="str">
         <v>1675 Dinusha Guantillake</v>

</xml_diff>

<commit_message>
SGL FR Plan — 04/06/2026 10:26
</commit_message>
<xml_diff>
--- a/Production_Plan.xlsx
+++ b/Production_Plan.xlsx
@@ -1385,7 +1385,7 @@
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="B16">
         <v>847</v>
@@ -1453,7 +1453,7 @@
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="B17">
         <v>847</v>
@@ -1521,7 +1521,7 @@
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="B18">
         <v>847</v>
@@ -1589,7 +1589,7 @@
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="B19">
         <v>847</v>
@@ -1657,7 +1657,7 @@
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="B20">
         <v>847</v>
@@ -1725,7 +1725,7 @@
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="B21">
         <v>847</v>
@@ -1793,7 +1793,7 @@
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="B22">
         <v>847</v>
@@ -1861,7 +1861,7 @@
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="B23">
         <v>847</v>
@@ -1929,7 +1929,7 @@
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="B24">
         <v>847</v>
@@ -1997,7 +1997,7 @@
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="B25">
         <v>847</v>
@@ -2065,7 +2065,7 @@
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="B26">
         <v>847</v>
@@ -2133,7 +2133,7 @@
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="B27">
         <v>847</v>
@@ -2201,7 +2201,7 @@
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="C28" t="str">
         <v>9676T::SGSGZIMER4233::BL</v>
@@ -2228,10 +2228,10 @@
         <v>-</v>
       </c>
       <c r="S28">
-        <v>46171</v>
+        <v>46211</v>
       </c>
       <c r="T28">
-        <v>46179</v>
+        <v>46219</v>
       </c>
       <c r="V28" t="str">
         <v>1675 Dinusha Guantillake</v>

</xml_diff>

<commit_message>
SGL FR Plan — 04/06/2026 10:31
</commit_message>
<xml_diff>
--- a/Production_Plan.xlsx
+++ b/Production_Plan.xlsx
@@ -12598,6 +12598,9 @@
       <c r="W205">
         <v>46219</v>
       </c>
+      <c r="X205" t="str">
+        <v>MG-r1bjbb</v>
+      </c>
     </row>
     <row r="206">
       <c r="A206" t="str">
@@ -12639,6 +12642,9 @@
       <c r="W206">
         <v>46219</v>
       </c>
+      <c r="X206" t="str">
+        <v>MG-r1bjbb</v>
+      </c>
     </row>
     <row r="207">
       <c r="A207" t="str">
@@ -12707,6 +12713,9 @@
       <c r="W207">
         <v>46219</v>
       </c>
+      <c r="X207" t="str">
+        <v>MG-r1bjbb</v>
+      </c>
     </row>
     <row r="208">
       <c r="A208" t="str">
@@ -12748,6 +12757,9 @@
       <c r="W208">
         <v>46219</v>
       </c>
+      <c r="X208" t="str">
+        <v>MG-r1bjbb</v>
+      </c>
     </row>
     <row r="209">
       <c r="A209" t="str">
@@ -12816,6 +12828,9 @@
       <c r="W209">
         <v>46219</v>
       </c>
+      <c r="X209" t="str">
+        <v>MG-r1bjbb</v>
+      </c>
     </row>
     <row r="210">
       <c r="A210" t="str">
@@ -12856,6 +12871,9 @@
       </c>
       <c r="W210">
         <v>46219</v>
+      </c>
+      <c r="X210" t="str">
+        <v>MG-r1bjbb</v>
       </c>
     </row>
     <row r="211">

</xml_diff>

<commit_message>
SGL FR Plan — 04/06/2026 10:32
</commit_message>
<xml_diff>
--- a/Production_Plan.xlsx
+++ b/Production_Plan.xlsx
@@ -12598,9 +12598,6 @@
       <c r="W205">
         <v>46219</v>
       </c>
-      <c r="X205" t="str">
-        <v>MG-r1bjbb</v>
-      </c>
     </row>
     <row r="206">
       <c r="A206" t="str">
@@ -12642,9 +12639,6 @@
       <c r="W206">
         <v>46219</v>
       </c>
-      <c r="X206" t="str">
-        <v>MG-r1bjbb</v>
-      </c>
     </row>
     <row r="207">
       <c r="A207" t="str">
@@ -12713,9 +12707,6 @@
       <c r="W207">
         <v>46219</v>
       </c>
-      <c r="X207" t="str">
-        <v>MG-r1bjbb</v>
-      </c>
     </row>
     <row r="208">
       <c r="A208" t="str">
@@ -12757,9 +12748,6 @@
       <c r="W208">
         <v>46219</v>
       </c>
-      <c r="X208" t="str">
-        <v>MG-r1bjbb</v>
-      </c>
     </row>
     <row r="209">
       <c r="A209" t="str">
@@ -12828,9 +12816,6 @@
       <c r="W209">
         <v>46219</v>
       </c>
-      <c r="X209" t="str">
-        <v>MG-r1bjbb</v>
-      </c>
     </row>
     <row r="210">
       <c r="A210" t="str">
@@ -12871,9 +12856,6 @@
       </c>
       <c r="W210">
         <v>46219</v>
-      </c>
-      <c r="X210" t="str">
-        <v>MG-r1bjbb</v>
       </c>
     </row>
     <row r="211">

</xml_diff>

<commit_message>
SGL FR Plan — 04/06/2026 10:39
</commit_message>
<xml_diff>
--- a/Production_Plan.xlsx
+++ b/Production_Plan.xlsx
@@ -12598,6 +12598,9 @@
       <c r="W205">
         <v>46219</v>
       </c>
+      <c r="X205" t="str">
+        <v>MG-0kqtxu</v>
+      </c>
     </row>
     <row r="206">
       <c r="A206" t="str">
@@ -12639,6 +12642,9 @@
       <c r="W206">
         <v>46219</v>
       </c>
+      <c r="X206" t="str">
+        <v>MG-0kqtxu</v>
+      </c>
     </row>
     <row r="207">
       <c r="A207" t="str">
@@ -12707,6 +12713,9 @@
       <c r="W207">
         <v>46219</v>
       </c>
+      <c r="X207" t="str">
+        <v>MG-0kqtxu</v>
+      </c>
     </row>
     <row r="208">
       <c r="A208" t="str">
@@ -12748,6 +12757,9 @@
       <c r="W208">
         <v>46219</v>
       </c>
+      <c r="X208" t="str">
+        <v>MG-0kqtxu</v>
+      </c>
     </row>
     <row r="209">
       <c r="A209" t="str">
@@ -12816,6 +12828,9 @@
       <c r="W209">
         <v>46219</v>
       </c>
+      <c r="X209" t="str">
+        <v>MG-0kqtxu</v>
+      </c>
     </row>
     <row r="210">
       <c r="A210" t="str">
@@ -12856,6 +12871,9 @@
       </c>
       <c r="W210">
         <v>46219</v>
+      </c>
+      <c r="X210" t="str">
+        <v>MG-0kqtxu</v>
       </c>
     </row>
     <row r="211">

</xml_diff>

<commit_message>
SGL FR Plan — 04/06/2026 14:25
</commit_message>
<xml_diff>
--- a/Production_Plan.xlsx
+++ b/Production_Plan.xlsx
@@ -1385,7 +1385,7 @@
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>SGL 02</v>
+        <v>SGL 01</v>
       </c>
       <c r="B16">
         <v>847</v>
@@ -1453,7 +1453,7 @@
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>SGL 02</v>
+        <v>SGL 01</v>
       </c>
       <c r="B17">
         <v>847</v>
@@ -1521,7 +1521,7 @@
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>SGL 02</v>
+        <v>SGL 01</v>
       </c>
       <c r="B18">
         <v>847</v>
@@ -1589,7 +1589,7 @@
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>SGL 02</v>
+        <v>SGL 01</v>
       </c>
       <c r="B19">
         <v>847</v>
@@ -1657,7 +1657,7 @@
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>SGL 02</v>
+        <v>SGL 01</v>
       </c>
       <c r="B20">
         <v>847</v>
@@ -1725,7 +1725,7 @@
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>SGL 02</v>
+        <v>SGL 01</v>
       </c>
       <c r="B21">
         <v>847</v>
@@ -1793,7 +1793,7 @@
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>SGL 02</v>
+        <v>SGL 01</v>
       </c>
       <c r="B22">
         <v>847</v>
@@ -1861,7 +1861,7 @@
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>SGL 02</v>
+        <v>SGL 01</v>
       </c>
       <c r="B23">
         <v>847</v>
@@ -1929,7 +1929,7 @@
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>SGL 02</v>
+        <v>SGL 01</v>
       </c>
       <c r="B24">
         <v>847</v>
@@ -1997,7 +1997,7 @@
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>SGL 02</v>
+        <v>SGL 01</v>
       </c>
       <c r="B25">
         <v>847</v>
@@ -2065,7 +2065,7 @@
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>SGL 02</v>
+        <v>SGL 01</v>
       </c>
       <c r="B26">
         <v>847</v>
@@ -2133,7 +2133,7 @@
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>SGL 02</v>
+        <v>SGL 01</v>
       </c>
       <c r="B27">
         <v>847</v>
@@ -2201,7 +2201,7 @@
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>SGL 02</v>
+        <v>SGL 01</v>
       </c>
       <c r="C28" t="str">
         <v>9676T::SGSGZIMER4233::BL</v>
@@ -2228,10 +2228,10 @@
         <v>-</v>
       </c>
       <c r="S28">
-        <v>46211</v>
+        <v>46171</v>
       </c>
       <c r="T28">
-        <v>46219</v>
+        <v>46179</v>
       </c>
       <c r="V28" t="str">
         <v>1675 Dinusha Guantillake</v>

</xml_diff>

<commit_message>
SGL FR Plan — 04/06/2026 15:33
</commit_message>
<xml_diff>
--- a/Production_Plan.xlsx
+++ b/Production_Plan.xlsx
@@ -1385,7 +1385,7 @@
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="B16">
         <v>847</v>
@@ -1453,7 +1453,7 @@
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="B17">
         <v>847</v>
@@ -1521,7 +1521,7 @@
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="B18">
         <v>847</v>
@@ -1589,7 +1589,7 @@
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="B19">
         <v>847</v>
@@ -1657,7 +1657,7 @@
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="B20">
         <v>847</v>
@@ -1725,7 +1725,7 @@
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="B21">
         <v>847</v>
@@ -1793,7 +1793,7 @@
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="B22">
         <v>847</v>
@@ -1861,7 +1861,7 @@
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="B23">
         <v>847</v>
@@ -1929,7 +1929,7 @@
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="B24">
         <v>847</v>
@@ -1997,7 +1997,7 @@
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="B25">
         <v>847</v>
@@ -2065,7 +2065,7 @@
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="B26">
         <v>847</v>
@@ -2133,7 +2133,7 @@
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="B27">
         <v>847</v>
@@ -2201,7 +2201,7 @@
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="C28" t="str">
         <v>9676T::SGSGZIMER4233::BL</v>
@@ -2228,10 +2228,10 @@
         <v>-</v>
       </c>
       <c r="S28">
-        <v>46171</v>
+        <v>46211</v>
       </c>
       <c r="T28">
-        <v>46179</v>
+        <v>46219</v>
       </c>
       <c r="V28" t="str">
         <v>1675 Dinusha Guantillake</v>

</xml_diff>

<commit_message>
SGL FR Plan — 04/06/2026 16:53
</commit_message>
<xml_diff>
--- a/Production_Plan.xlsx
+++ b/Production_Plan.xlsx
@@ -1385,7 +1385,7 @@
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>SGL 02</v>
+        <v>SGL 01</v>
       </c>
       <c r="B16">
         <v>847</v>
@@ -1453,7 +1453,7 @@
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>SGL 02</v>
+        <v>SGL 01</v>
       </c>
       <c r="B17">
         <v>847</v>
@@ -1521,7 +1521,7 @@
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>SGL 02</v>
+        <v>SGL 01</v>
       </c>
       <c r="B18">
         <v>847</v>
@@ -1589,7 +1589,7 @@
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>SGL 02</v>
+        <v>SGL 01</v>
       </c>
       <c r="B19">
         <v>847</v>
@@ -1657,7 +1657,7 @@
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>SGL 02</v>
+        <v>SGL 01</v>
       </c>
       <c r="B20">
         <v>847</v>
@@ -1725,7 +1725,7 @@
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>SGL 02</v>
+        <v>SGL 01</v>
       </c>
       <c r="B21">
         <v>847</v>
@@ -1793,7 +1793,7 @@
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>SGL 02</v>
+        <v>SGL 01</v>
       </c>
       <c r="B22">
         <v>847</v>
@@ -1861,7 +1861,7 @@
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>SGL 02</v>
+        <v>SGL 01</v>
       </c>
       <c r="B23">
         <v>847</v>
@@ -1929,7 +1929,7 @@
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>SGL 02</v>
+        <v>SGL 01</v>
       </c>
       <c r="B24">
         <v>847</v>
@@ -1997,7 +1997,7 @@
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>SGL 02</v>
+        <v>SGL 01</v>
       </c>
       <c r="B25">
         <v>847</v>
@@ -2065,7 +2065,7 @@
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>SGL 02</v>
+        <v>SGL 01</v>
       </c>
       <c r="B26">
         <v>847</v>
@@ -2133,7 +2133,7 @@
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>SGL 02</v>
+        <v>SGL 01</v>
       </c>
       <c r="B27">
         <v>847</v>
@@ -2201,7 +2201,7 @@
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>SGL 02</v>
+        <v>SGL 01</v>
       </c>
       <c r="C28" t="str">
         <v>9676T::SGSGZIMER4233::BL</v>
@@ -2228,10 +2228,10 @@
         <v>-</v>
       </c>
       <c r="S28">
-        <v>46211</v>
+        <v>46171</v>
       </c>
       <c r="T28">
-        <v>46219</v>
+        <v>46179</v>
       </c>
       <c r="V28" t="str">
         <v>1675 Dinusha Guantillake</v>

</xml_diff>

<commit_message>
SGL FR Plan — 05/06/2026 14:02
</commit_message>
<xml_diff>
--- a/Production_Plan.xlsx
+++ b/Production_Plan.xlsx
@@ -1385,7 +1385,7 @@
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="B16">
         <v>847</v>
@@ -1453,7 +1453,7 @@
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="B17">
         <v>847</v>
@@ -1521,7 +1521,7 @@
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="B18">
         <v>847</v>
@@ -1589,7 +1589,7 @@
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="B19">
         <v>847</v>
@@ -1657,7 +1657,7 @@
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="B20">
         <v>847</v>
@@ -1725,7 +1725,7 @@
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="B21">
         <v>847</v>
@@ -1793,7 +1793,7 @@
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="B22">
         <v>847</v>
@@ -1861,7 +1861,7 @@
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="B23">
         <v>847</v>
@@ -1929,7 +1929,7 @@
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="B24">
         <v>847</v>
@@ -1997,7 +1997,7 @@
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="B25">
         <v>847</v>
@@ -2065,7 +2065,7 @@
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="B26">
         <v>847</v>
@@ -2133,7 +2133,7 @@
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="B27">
         <v>847</v>
@@ -2201,7 +2201,7 @@
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="C28" t="str">
         <v>9676T::SGSGZIMER4233::BL</v>
@@ -2228,10 +2228,10 @@
         <v>-</v>
       </c>
       <c r="S28">
-        <v>46171</v>
+        <v>46211</v>
       </c>
       <c r="T28">
-        <v>46179</v>
+        <v>46219</v>
       </c>
       <c r="V28" t="str">
         <v>1675 Dinusha Guantillake</v>

</xml_diff>

<commit_message>
SGL FR Plan — 05/06/2026 14:41
</commit_message>
<xml_diff>
--- a/Production_Plan.xlsx
+++ b/Production_Plan.xlsx
@@ -1385,7 +1385,7 @@
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>SGL 02</v>
+        <v>SGL 01</v>
       </c>
       <c r="B16">
         <v>847</v>
@@ -1453,7 +1453,7 @@
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>SGL 02</v>
+        <v>SGL 01</v>
       </c>
       <c r="B17">
         <v>847</v>
@@ -1521,7 +1521,7 @@
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>SGL 02</v>
+        <v>SGL 01</v>
       </c>
       <c r="B18">
         <v>847</v>
@@ -1589,7 +1589,7 @@
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>SGL 02</v>
+        <v>SGL 01</v>
       </c>
       <c r="B19">
         <v>847</v>
@@ -1657,7 +1657,7 @@
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>SGL 02</v>
+        <v>SGL 01</v>
       </c>
       <c r="B20">
         <v>847</v>
@@ -1725,7 +1725,7 @@
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>SGL 02</v>
+        <v>SGL 01</v>
       </c>
       <c r="B21">
         <v>847</v>
@@ -1793,7 +1793,7 @@
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>SGL 02</v>
+        <v>SGL 01</v>
       </c>
       <c r="B22">
         <v>847</v>
@@ -1861,7 +1861,7 @@
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>SGL 02</v>
+        <v>SGL 01</v>
       </c>
       <c r="B23">
         <v>847</v>
@@ -1929,7 +1929,7 @@
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>SGL 02</v>
+        <v>SGL 01</v>
       </c>
       <c r="B24">
         <v>847</v>
@@ -1997,7 +1997,7 @@
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>SGL 02</v>
+        <v>SGL 01</v>
       </c>
       <c r="B25">
         <v>847</v>
@@ -2065,7 +2065,7 @@
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>SGL 02</v>
+        <v>SGL 01</v>
       </c>
       <c r="B26">
         <v>847</v>
@@ -2133,7 +2133,7 @@
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>SGL 02</v>
+        <v>SGL 01</v>
       </c>
       <c r="B27">
         <v>847</v>
@@ -2201,7 +2201,7 @@
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>SGL 02</v>
+        <v>SGL 01</v>
       </c>
       <c r="C28" t="str">
         <v>9676T::SGSGZIMER4233::BL</v>
@@ -2228,10 +2228,10 @@
         <v>-</v>
       </c>
       <c r="S28">
-        <v>46211</v>
+        <v>46170</v>
       </c>
       <c r="T28">
-        <v>46219</v>
+        <v>46178</v>
       </c>
       <c r="V28" t="str">
         <v>1675 Dinusha Guantillake</v>

</xml_diff>

<commit_message>
SGL FR Plan — 05/06/2026 14:46
</commit_message>
<xml_diff>
--- a/Production_Plan.xlsx
+++ b/Production_Plan.xlsx
@@ -1385,7 +1385,7 @@
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="B16">
         <v>847</v>
@@ -1453,7 +1453,7 @@
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="B17">
         <v>847</v>
@@ -1521,7 +1521,7 @@
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="B18">
         <v>847</v>
@@ -1589,7 +1589,7 @@
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="B19">
         <v>847</v>
@@ -1657,7 +1657,7 @@
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="B20">
         <v>847</v>
@@ -1725,7 +1725,7 @@
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="B21">
         <v>847</v>
@@ -1793,7 +1793,7 @@
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="B22">
         <v>847</v>
@@ -1861,7 +1861,7 @@
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="B23">
         <v>847</v>
@@ -1929,7 +1929,7 @@
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="B24">
         <v>847</v>
@@ -1997,7 +1997,7 @@
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="B25">
         <v>847</v>
@@ -2065,7 +2065,7 @@
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="B26">
         <v>847</v>
@@ -2133,7 +2133,7 @@
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="B27">
         <v>847</v>
@@ -2201,7 +2201,7 @@
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="C28" t="str">
         <v>9676T::SGSGZIMER4233::BL</v>
@@ -2228,10 +2228,10 @@
         <v>-</v>
       </c>
       <c r="S28">
-        <v>46170</v>
+        <v>46211</v>
       </c>
       <c r="T28">
-        <v>46178</v>
+        <v>46219</v>
       </c>
       <c r="V28" t="str">
         <v>1675 Dinusha Guantillake</v>

</xml_diff>

<commit_message>
SGL FR Plan — 08/06/2026 09:01
</commit_message>
<xml_diff>
--- a/Production_Plan.xlsx
+++ b/Production_Plan.xlsx
@@ -1385,7 +1385,7 @@
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>SGL 02</v>
+        <v>SGL 01</v>
       </c>
       <c r="B16">
         <v>847</v>
@@ -1453,7 +1453,7 @@
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>SGL 02</v>
+        <v>SGL 01</v>
       </c>
       <c r="B17">
         <v>847</v>
@@ -1521,7 +1521,7 @@
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>SGL 02</v>
+        <v>SGL 01</v>
       </c>
       <c r="B18">
         <v>847</v>
@@ -1589,7 +1589,7 @@
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>SGL 02</v>
+        <v>SGL 01</v>
       </c>
       <c r="B19">
         <v>847</v>
@@ -1657,7 +1657,7 @@
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>SGL 02</v>
+        <v>SGL 01</v>
       </c>
       <c r="B20">
         <v>847</v>
@@ -1725,7 +1725,7 @@
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>SGL 02</v>
+        <v>SGL 01</v>
       </c>
       <c r="B21">
         <v>847</v>
@@ -1793,7 +1793,7 @@
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>SGL 02</v>
+        <v>SGL 01</v>
       </c>
       <c r="B22">
         <v>847</v>
@@ -1861,7 +1861,7 @@
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>SGL 02</v>
+        <v>SGL 01</v>
       </c>
       <c r="B23">
         <v>847</v>
@@ -1929,7 +1929,7 @@
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>SGL 02</v>
+        <v>SGL 01</v>
       </c>
       <c r="B24">
         <v>847</v>
@@ -1997,7 +1997,7 @@
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>SGL 02</v>
+        <v>SGL 01</v>
       </c>
       <c r="B25">
         <v>847</v>
@@ -2065,7 +2065,7 @@
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>SGL 02</v>
+        <v>SGL 01</v>
       </c>
       <c r="B26">
         <v>847</v>
@@ -2133,7 +2133,7 @@
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>SGL 02</v>
+        <v>SGL 01</v>
       </c>
       <c r="B27">
         <v>847</v>
@@ -2201,7 +2201,7 @@
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>SGL 02</v>
+        <v>SGL 01</v>
       </c>
       <c r="C28" t="str">
         <v>9676T::SGSGZIMER4233::BL</v>
@@ -2228,10 +2228,10 @@
         <v>-</v>
       </c>
       <c r="S28">
-        <v>46211</v>
+        <v>46170</v>
       </c>
       <c r="T28">
-        <v>46219</v>
+        <v>46178</v>
       </c>
       <c r="V28" t="str">
         <v>1675 Dinusha Guantillake</v>

</xml_diff>

<commit_message>
SGL FR Plan — 20/07/2026 10:07
</commit_message>
<xml_diff>
--- a/Production_Plan.xlsx
+++ b/Production_Plan.xlsx
@@ -32,9 +32,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
-  <numFmts count="2">
+  <numFmts count="1">
     <numFmt numFmtId="56" formatCode="&quot;上午/下午 &quot;hh&quot;時&quot;mm&quot;分&quot;ss&quot;秒 &quot;"/>
-    <numFmt numFmtId="164" formatCode="M/d/yyyy"/>
   </numFmts>
   <fonts count="1">
     <font>
@@ -21957,10 +21956,10 @@
         <v>46214</v>
       </c>
       <c r="S382">
-        <v>46223</v>
+        <v>46225</v>
       </c>
       <c r="T382">
-        <v>46224</v>
+        <v>46226</v>
       </c>
       <c r="V382" t="str">
         <v>491 Nilu Udunuwaraarachchi</v>
@@ -22066,10 +22065,10 @@
         <v>46216</v>
       </c>
       <c r="S384">
-        <v>46224</v>
+        <v>46226</v>
       </c>
       <c r="T384">
-        <v>46225</v>
+        <v>46227</v>
       </c>
       <c r="V384" t="str">
         <v>491 Nilu Udunuwaraarachchi</v>

</xml_diff>

<commit_message>
SGL FR Plan — 20/07/2026 11:08
</commit_message>
<xml_diff>
--- a/Production_Plan.xlsx
+++ b/Production_Plan.xlsx
@@ -897,7 +897,7 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="B9">
         <v>847</v>
@@ -962,7 +962,7 @@
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="B10">
         <v>847</v>
@@ -1027,7 +1027,7 @@
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="B11">
         <v>847</v>
@@ -1092,7 +1092,7 @@
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="B12">
         <v>847</v>
@@ -1157,7 +1157,7 @@
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="B13">
         <v>847</v>
@@ -1222,7 +1222,7 @@
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="B14">
         <v>847</v>
@@ -1287,7 +1287,7 @@
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="B15">
         <v>847</v>
@@ -1352,7 +1352,7 @@
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="C16" t="str">
         <v>0794A::SGSGZIMER5207::SH</v>
@@ -1379,10 +1379,10 @@
         <v>46221</v>
       </c>
       <c r="S16">
-        <v>46224</v>
+        <v>46227</v>
       </c>
       <c r="T16">
-        <v>46227</v>
+        <v>46231</v>
       </c>
       <c r="V16" t="str">
         <v>1675 Dinusha Guantillake</v>
@@ -1875,10 +1875,10 @@
         <v>46225</v>
       </c>
       <c r="S24">
+        <v>46225</v>
+      </c>
+      <c r="T24">
         <v>46227</v>
-      </c>
-      <c r="T24">
-        <v>46231</v>
       </c>
       <c r="V24" t="str">
         <v>1675 Dinusha Guantillake</v>
@@ -2664,10 +2664,10 @@
         <v>46223</v>
       </c>
       <c r="S36">
+        <v>46228</v>
+      </c>
+      <c r="T36">
         <v>46231</v>
-      </c>
-      <c r="T36">
-        <v>46234</v>
       </c>
       <c r="V36" t="str">
         <v>1675 Dinusha Guantillake</v>
@@ -3420,10 +3420,10 @@
         <v>46226</v>
       </c>
       <c r="S48">
-        <v>46234</v>
+        <v>46232</v>
       </c>
       <c r="T48">
-        <v>46241</v>
+        <v>46238</v>
       </c>
       <c r="V48" t="str">
         <v>1675 Dinusha Guantillake</v>
@@ -3591,10 +3591,10 @@
         <v>46239</v>
       </c>
       <c r="S51">
-        <v>46241</v>
+        <v>46239</v>
       </c>
       <c r="T51">
-        <v>46248</v>
+        <v>46245</v>
       </c>
       <c r="V51" t="str">
         <v>1702 Piyumi Perera</v>
@@ -3697,10 +3697,10 @@
         <v>46246</v>
       </c>
       <c r="S53">
-        <v>46248</v>
+        <v>46246</v>
       </c>
       <c r="T53">
-        <v>46251</v>
+        <v>46247</v>
       </c>
       <c r="V53" t="str">
         <v>1702 Piyumi Perera</v>
@@ -3797,10 +3797,10 @@
         <v>46248</v>
       </c>
       <c r="S55">
-        <v>46251</v>
+        <v>46248</v>
       </c>
       <c r="T55">
-        <v>46258</v>
+        <v>46254</v>
       </c>
       <c r="V55" t="str">
         <v>275 Hashan De Mel</v>
@@ -4334,10 +4334,10 @@
         <v>46255</v>
       </c>
       <c r="S64">
-        <v>46258</v>
+        <v>46255</v>
       </c>
       <c r="T64">
-        <v>46265</v>
+        <v>46261</v>
       </c>
       <c r="W64">
         <v>46279</v>
@@ -4974,10 +4974,10 @@
         <v>46224</v>
       </c>
       <c r="S75">
-        <v>46226</v>
+        <v>46232</v>
       </c>
       <c r="T75">
-        <v>46230</v>
+        <v>46234</v>
       </c>
       <c r="V75" t="str">
         <v>1675 Dinusha Guantillake</v>
@@ -5763,10 +5763,10 @@
         <v>46227</v>
       </c>
       <c r="S87">
-        <v>46230</v>
+        <v>46235</v>
       </c>
       <c r="T87">
-        <v>46241</v>
+        <v>46246</v>
       </c>
       <c r="V87" t="str">
         <v>1675 Dinusha Guantillake</v>
@@ -6620,10 +6620,10 @@
         <v>46239</v>
       </c>
       <c r="S100">
-        <v>46241</v>
+        <v>46247</v>
       </c>
       <c r="T100">
-        <v>46251</v>
+        <v>46255</v>
       </c>
       <c r="V100" t="str">
         <v>1675 Dinusha Guantillake</v>
@@ -7343,10 +7343,10 @@
         <v>46251</v>
       </c>
       <c r="S112">
-        <v>46253</v>
+        <v>46256</v>
       </c>
       <c r="T112">
-        <v>46262</v>
+        <v>46266</v>
       </c>
       <c r="W112">
         <v>46275</v>

</xml_diff>

<commit_message>
SGL FR Plan — 20/07/2026 11:09
</commit_message>
<xml_diff>
--- a/Production_Plan.xlsx
+++ b/Production_Plan.xlsx
@@ -897,7 +897,7 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>SGL 02</v>
+        <v>SGL 01</v>
       </c>
       <c r="B9">
         <v>847</v>
@@ -962,7 +962,7 @@
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>SGL 02</v>
+        <v>SGL 01</v>
       </c>
       <c r="B10">
         <v>847</v>
@@ -1027,7 +1027,7 @@
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>SGL 02</v>
+        <v>SGL 01</v>
       </c>
       <c r="B11">
         <v>847</v>
@@ -1092,7 +1092,7 @@
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>SGL 02</v>
+        <v>SGL 01</v>
       </c>
       <c r="B12">
         <v>847</v>
@@ -1157,7 +1157,7 @@
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>SGL 02</v>
+        <v>SGL 01</v>
       </c>
       <c r="B13">
         <v>847</v>
@@ -1222,7 +1222,7 @@
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>SGL 02</v>
+        <v>SGL 01</v>
       </c>
       <c r="B14">
         <v>847</v>
@@ -1287,7 +1287,7 @@
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>SGL 02</v>
+        <v>SGL 01</v>
       </c>
       <c r="B15">
         <v>847</v>
@@ -1352,7 +1352,7 @@
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>SGL 02</v>
+        <v>SGL 01</v>
       </c>
       <c r="C16" t="str">
         <v>0794A::SGSGZIMER5207::SH</v>
@@ -1379,10 +1379,10 @@
         <v>46221</v>
       </c>
       <c r="S16">
+        <v>46224</v>
+      </c>
+      <c r="T16">
         <v>46227</v>
-      </c>
-      <c r="T16">
-        <v>46231</v>
       </c>
       <c r="V16" t="str">
         <v>1675 Dinusha Guantillake</v>
@@ -1875,10 +1875,10 @@
         <v>46225</v>
       </c>
       <c r="S24">
-        <v>46225</v>
+        <v>46227</v>
       </c>
       <c r="T24">
-        <v>46227</v>
+        <v>46231</v>
       </c>
       <c r="V24" t="str">
         <v>1675 Dinusha Guantillake</v>
@@ -2664,10 +2664,10 @@
         <v>46223</v>
       </c>
       <c r="S36">
-        <v>46228</v>
+        <v>46231</v>
       </c>
       <c r="T36">
-        <v>46231</v>
+        <v>46234</v>
       </c>
       <c r="V36" t="str">
         <v>1675 Dinusha Guantillake</v>
@@ -3420,10 +3420,10 @@
         <v>46226</v>
       </c>
       <c r="S48">
-        <v>46232</v>
+        <v>46234</v>
       </c>
       <c r="T48">
-        <v>46238</v>
+        <v>46241</v>
       </c>
       <c r="V48" t="str">
         <v>1675 Dinusha Guantillake</v>
@@ -3591,10 +3591,10 @@
         <v>46239</v>
       </c>
       <c r="S51">
-        <v>46239</v>
+        <v>46241</v>
       </c>
       <c r="T51">
-        <v>46245</v>
+        <v>46248</v>
       </c>
       <c r="V51" t="str">
         <v>1702 Piyumi Perera</v>
@@ -3697,10 +3697,10 @@
         <v>46246</v>
       </c>
       <c r="S53">
-        <v>46246</v>
+        <v>46248</v>
       </c>
       <c r="T53">
-        <v>46247</v>
+        <v>46251</v>
       </c>
       <c r="V53" t="str">
         <v>1702 Piyumi Perera</v>
@@ -3797,10 +3797,10 @@
         <v>46248</v>
       </c>
       <c r="S55">
-        <v>46248</v>
+        <v>46251</v>
       </c>
       <c r="T55">
-        <v>46254</v>
+        <v>46258</v>
       </c>
       <c r="V55" t="str">
         <v>275 Hashan De Mel</v>
@@ -4334,10 +4334,10 @@
         <v>46255</v>
       </c>
       <c r="S64">
-        <v>46255</v>
+        <v>46258</v>
       </c>
       <c r="T64">
-        <v>46261</v>
+        <v>46265</v>
       </c>
       <c r="W64">
         <v>46279</v>
@@ -4974,10 +4974,10 @@
         <v>46224</v>
       </c>
       <c r="S75">
-        <v>46232</v>
+        <v>46226</v>
       </c>
       <c r="T75">
-        <v>46234</v>
+        <v>46230</v>
       </c>
       <c r="V75" t="str">
         <v>1675 Dinusha Guantillake</v>
@@ -5763,10 +5763,10 @@
         <v>46227</v>
       </c>
       <c r="S87">
-        <v>46235</v>
+        <v>46230</v>
       </c>
       <c r="T87">
-        <v>46246</v>
+        <v>46241</v>
       </c>
       <c r="V87" t="str">
         <v>1675 Dinusha Guantillake</v>
@@ -6620,10 +6620,10 @@
         <v>46239</v>
       </c>
       <c r="S100">
-        <v>46247</v>
+        <v>46241</v>
       </c>
       <c r="T100">
-        <v>46255</v>
+        <v>46251</v>
       </c>
       <c r="V100" t="str">
         <v>1675 Dinusha Guantillake</v>
@@ -7343,10 +7343,10 @@
         <v>46251</v>
       </c>
       <c r="S112">
-        <v>46256</v>
+        <v>46253</v>
       </c>
       <c r="T112">
-        <v>46266</v>
+        <v>46262</v>
       </c>
       <c r="W112">
         <v>46275</v>

</xml_diff>

<commit_message>
SGL FR Plan — 21/07/2026 10:14
</commit_message>
<xml_diff>
--- a/Production_Plan.xlsx
+++ b/Production_Plan.xlsx
@@ -32,8 +32,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="56" formatCode="&quot;上午/下午 &quot;hh&quot;時&quot;mm&quot;分&quot;ss&quot;秒 &quot;"/>
+    <numFmt numFmtId="164" formatCode="M/d/yyyy"/>
   </numFmts>
   <fonts count="1">
     <font>
@@ -10919,6 +10920,9 @@
       <c r="W174">
         <v>46224</v>
       </c>
+      <c r="X174" t="str">
+        <v>MG-unf9oe</v>
+      </c>
     </row>
     <row r="175">
       <c r="A175" t="str">
@@ -10957,6 +10961,9 @@
       <c r="W175">
         <v>46224</v>
       </c>
+      <c r="X175" t="str">
+        <v>MG-unf9oe</v>
+      </c>
     </row>
     <row r="176">
       <c r="A176" t="str">
@@ -11019,6 +11026,9 @@
       <c r="W176">
         <v>46226</v>
       </c>
+      <c r="X176" t="str">
+        <v>MG-unf9oe</v>
+      </c>
     </row>
     <row r="177">
       <c r="A177" t="str">
@@ -11056,6 +11066,9 @@
       </c>
       <c r="W177">
         <v>46226</v>
+      </c>
+      <c r="X177" t="str">
+        <v>MG-unf9oe</v>
       </c>
     </row>
     <row r="178">

</xml_diff>

<commit_message>
SGL FR Plan — 21/07/2026 10:16
</commit_message>
<xml_diff>
--- a/Production_Plan.xlsx
+++ b/Production_Plan.xlsx
@@ -10920,9 +10920,6 @@
       <c r="W174">
         <v>46224</v>
       </c>
-      <c r="X174" t="str">
-        <v>MG-unf9oe</v>
-      </c>
     </row>
     <row r="175">
       <c r="A175" t="str">
@@ -10961,9 +10958,6 @@
       <c r="W175">
         <v>46224</v>
       </c>
-      <c r="X175" t="str">
-        <v>MG-unf9oe</v>
-      </c>
     </row>
     <row r="176">
       <c r="A176" t="str">
@@ -11026,9 +11020,6 @@
       <c r="W176">
         <v>46226</v>
       </c>
-      <c r="X176" t="str">
-        <v>MG-unf9oe</v>
-      </c>
     </row>
     <row r="177">
       <c r="A177" t="str">
@@ -11066,9 +11057,6 @@
       </c>
       <c r="W177">
         <v>46226</v>
-      </c>
-      <c r="X177" t="str">
-        <v>MG-unf9oe</v>
       </c>
     </row>
     <row r="178">

</xml_diff>

<commit_message>
SGL FR Plan — 21/07/2026 12:55
</commit_message>
<xml_diff>
--- a/Production_Plan.xlsx
+++ b/Production_Plan.xlsx
@@ -898,7 +898,7 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="B9">
         <v>847</v>
@@ -963,7 +963,7 @@
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="B10">
         <v>847</v>
@@ -1028,7 +1028,7 @@
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="B11">
         <v>847</v>
@@ -1093,7 +1093,7 @@
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="B12">
         <v>847</v>
@@ -1158,7 +1158,7 @@
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="B13">
         <v>847</v>
@@ -1223,7 +1223,7 @@
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="B14">
         <v>847</v>
@@ -1288,7 +1288,7 @@
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="B15">
         <v>847</v>
@@ -1353,7 +1353,7 @@
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="C16" t="str">
         <v>0794A::SGSGZIMER5207::SH</v>
@@ -1380,10 +1380,10 @@
         <v>46221</v>
       </c>
       <c r="S16">
-        <v>46224</v>
+        <v>46227</v>
       </c>
       <c r="T16">
-        <v>46227</v>
+        <v>46231</v>
       </c>
       <c r="V16" t="str">
         <v>1675 Dinusha Guantillake</v>
@@ -1876,10 +1876,10 @@
         <v>46225</v>
       </c>
       <c r="S24">
+        <v>46225</v>
+      </c>
+      <c r="T24">
         <v>46227</v>
-      </c>
-      <c r="T24">
-        <v>46231</v>
       </c>
       <c r="V24" t="str">
         <v>1675 Dinusha Guantillake</v>
@@ -2665,10 +2665,10 @@
         <v>46223</v>
       </c>
       <c r="S36">
+        <v>46228</v>
+      </c>
+      <c r="T36">
         <v>46231</v>
-      </c>
-      <c r="T36">
-        <v>46234</v>
       </c>
       <c r="V36" t="str">
         <v>1675 Dinusha Guantillake</v>
@@ -3421,10 +3421,10 @@
         <v>46226</v>
       </c>
       <c r="S48">
-        <v>46234</v>
+        <v>46232</v>
       </c>
       <c r="T48">
-        <v>46241</v>
+        <v>46238</v>
       </c>
       <c r="V48" t="str">
         <v>1675 Dinusha Guantillake</v>
@@ -3592,10 +3592,10 @@
         <v>46239</v>
       </c>
       <c r="S51">
-        <v>46241</v>
+        <v>46239</v>
       </c>
       <c r="T51">
-        <v>46248</v>
+        <v>46245</v>
       </c>
       <c r="V51" t="str">
         <v>1702 Piyumi Perera</v>
@@ -3698,10 +3698,10 @@
         <v>46246</v>
       </c>
       <c r="S53">
-        <v>46248</v>
+        <v>46246</v>
       </c>
       <c r="T53">
-        <v>46251</v>
+        <v>46247</v>
       </c>
       <c r="V53" t="str">
         <v>1702 Piyumi Perera</v>
@@ -3798,10 +3798,10 @@
         <v>46248</v>
       </c>
       <c r="S55">
-        <v>46251</v>
+        <v>46248</v>
       </c>
       <c r="T55">
-        <v>46258</v>
+        <v>46254</v>
       </c>
       <c r="V55" t="str">
         <v>275 Hashan De Mel</v>
@@ -4335,10 +4335,10 @@
         <v>46255</v>
       </c>
       <c r="S64">
-        <v>46258</v>
+        <v>46255</v>
       </c>
       <c r="T64">
-        <v>46265</v>
+        <v>46261</v>
       </c>
       <c r="W64">
         <v>46279</v>
@@ -4975,10 +4975,10 @@
         <v>46224</v>
       </c>
       <c r="S75">
-        <v>46226</v>
+        <v>46232</v>
       </c>
       <c r="T75">
-        <v>46230</v>
+        <v>46234</v>
       </c>
       <c r="V75" t="str">
         <v>1675 Dinusha Guantillake</v>
@@ -5764,10 +5764,10 @@
         <v>46227</v>
       </c>
       <c r="S87">
-        <v>46230</v>
+        <v>46235</v>
       </c>
       <c r="T87">
-        <v>46241</v>
+        <v>46246</v>
       </c>
       <c r="V87" t="str">
         <v>1675 Dinusha Guantillake</v>
@@ -6621,10 +6621,10 @@
         <v>46239</v>
       </c>
       <c r="S100">
-        <v>46241</v>
+        <v>46247</v>
       </c>
       <c r="T100">
-        <v>46251</v>
+        <v>46255</v>
       </c>
       <c r="V100" t="str">
         <v>1675 Dinusha Guantillake</v>
@@ -7344,10 +7344,10 @@
         <v>46251</v>
       </c>
       <c r="S112">
-        <v>46253</v>
+        <v>46256</v>
       </c>
       <c r="T112">
-        <v>46262</v>
+        <v>46266</v>
       </c>
       <c r="W112">
         <v>46275</v>

</xml_diff>

<commit_message>
SGL FR Plan — 21/07/2026 14:07
</commit_message>
<xml_diff>
--- a/Production_Plan.xlsx
+++ b/Production_Plan.xlsx
@@ -898,7 +898,7 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>SGL 02</v>
+        <v>SGL 01</v>
       </c>
       <c r="B9">
         <v>847</v>
@@ -963,7 +963,7 @@
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>SGL 02</v>
+        <v>SGL 01</v>
       </c>
       <c r="B10">
         <v>847</v>
@@ -1028,7 +1028,7 @@
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>SGL 02</v>
+        <v>SGL 01</v>
       </c>
       <c r="B11">
         <v>847</v>
@@ -1093,7 +1093,7 @@
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>SGL 02</v>
+        <v>SGL 01</v>
       </c>
       <c r="B12">
         <v>847</v>
@@ -1158,7 +1158,7 @@
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>SGL 02</v>
+        <v>SGL 01</v>
       </c>
       <c r="B13">
         <v>847</v>
@@ -1223,7 +1223,7 @@
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>SGL 02</v>
+        <v>SGL 01</v>
       </c>
       <c r="B14">
         <v>847</v>
@@ -1288,7 +1288,7 @@
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>SGL 02</v>
+        <v>SGL 01</v>
       </c>
       <c r="B15">
         <v>847</v>
@@ -1353,7 +1353,7 @@
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>SGL 02</v>
+        <v>SGL 01</v>
       </c>
       <c r="C16" t="str">
         <v>0794A::SGSGZIMER5207::SH</v>
@@ -1380,10 +1380,10 @@
         <v>46221</v>
       </c>
       <c r="S16">
+        <v>46224</v>
+      </c>
+      <c r="T16">
         <v>46227</v>
-      </c>
-      <c r="T16">
-        <v>46231</v>
       </c>
       <c r="V16" t="str">
         <v>1675 Dinusha Guantillake</v>
@@ -1876,10 +1876,10 @@
         <v>46225</v>
       </c>
       <c r="S24">
-        <v>46225</v>
+        <v>46228</v>
       </c>
       <c r="T24">
-        <v>46227</v>
+        <v>46231</v>
       </c>
       <c r="V24" t="str">
         <v>1675 Dinusha Guantillake</v>
@@ -2665,10 +2665,10 @@
         <v>46223</v>
       </c>
       <c r="S36">
-        <v>46228</v>
+        <v>46237</v>
       </c>
       <c r="T36">
-        <v>46231</v>
+        <v>46239</v>
       </c>
       <c r="V36" t="str">
         <v>1675 Dinusha Guantillake</v>
@@ -3421,10 +3421,10 @@
         <v>46226</v>
       </c>
       <c r="S48">
-        <v>46232</v>
+        <v>46240</v>
       </c>
       <c r="T48">
-        <v>46238</v>
+        <v>46246</v>
       </c>
       <c r="V48" t="str">
         <v>1675 Dinusha Guantillake</v>
@@ -3592,10 +3592,10 @@
         <v>46239</v>
       </c>
       <c r="S51">
-        <v>46239</v>
+        <v>46247</v>
       </c>
       <c r="T51">
-        <v>46245</v>
+        <v>46253</v>
       </c>
       <c r="V51" t="str">
         <v>1702 Piyumi Perera</v>
@@ -3698,10 +3698,10 @@
         <v>46246</v>
       </c>
       <c r="S53">
-        <v>46246</v>
+        <v>46254</v>
       </c>
       <c r="T53">
-        <v>46247</v>
+        <v>46255</v>
       </c>
       <c r="V53" t="str">
         <v>1702 Piyumi Perera</v>
@@ -3798,10 +3798,10 @@
         <v>46248</v>
       </c>
       <c r="S55">
-        <v>46248</v>
+        <v>46256</v>
       </c>
       <c r="T55">
-        <v>46254</v>
+        <v>46262</v>
       </c>
       <c r="V55" t="str">
         <v>275 Hashan De Mel</v>
@@ -4335,10 +4335,10 @@
         <v>46255</v>
       </c>
       <c r="S64">
-        <v>46255</v>
+        <v>46263</v>
       </c>
       <c r="T64">
-        <v>46261</v>
+        <v>46269</v>
       </c>
       <c r="W64">
         <v>46279</v>
@@ -4753,7 +4753,7 @@
     </row>
     <row r="72">
       <c r="A72" t="str">
-        <v>SGL 02</v>
+        <v>SGL 01</v>
       </c>
       <c r="B72">
         <v>847</v>
@@ -4818,7 +4818,7 @@
     </row>
     <row r="73">
       <c r="A73" t="str">
-        <v>SGL 02</v>
+        <v>SGL 01</v>
       </c>
       <c r="B73">
         <v>847</v>
@@ -4883,7 +4883,7 @@
     </row>
     <row r="74">
       <c r="A74" t="str">
-        <v>SGL 02</v>
+        <v>SGL 01</v>
       </c>
       <c r="B74">
         <v>847</v>
@@ -4948,7 +4948,7 @@
     </row>
     <row r="75">
       <c r="A75" t="str">
-        <v>SGL 02</v>
+        <v>SGL 01</v>
       </c>
       <c r="C75" t="str">
         <v>3497A::SGSGZIMER5060::SH</v>
@@ -4978,7 +4978,7 @@
         <v>46232</v>
       </c>
       <c r="T75">
-        <v>46234</v>
+        <v>46235</v>
       </c>
       <c r="V75" t="str">
         <v>1675 Dinusha Guantillake</v>
@@ -5764,10 +5764,10 @@
         <v>46227</v>
       </c>
       <c r="S87">
-        <v>46235</v>
+        <v>46227</v>
       </c>
       <c r="T87">
-        <v>46246</v>
+        <v>46238</v>
       </c>
       <c r="V87" t="str">
         <v>1675 Dinusha Guantillake</v>
@@ -6621,10 +6621,10 @@
         <v>46239</v>
       </c>
       <c r="S100">
+        <v>46239</v>
+      </c>
+      <c r="T100">
         <v>46247</v>
-      </c>
-      <c r="T100">
-        <v>46255</v>
       </c>
       <c r="V100" t="str">
         <v>1675 Dinusha Guantillake</v>
@@ -7344,10 +7344,10 @@
         <v>46251</v>
       </c>
       <c r="S112">
-        <v>46256</v>
+        <v>46248</v>
       </c>
       <c r="T112">
-        <v>46266</v>
+        <v>46258</v>
       </c>
       <c r="W112">
         <v>46275</v>

</xml_diff>

<commit_message>
SGL FR Plan — 22/07/2026 11:16
</commit_message>
<xml_diff>
--- a/Production_Plan.xlsx
+++ b/Production_Plan.xlsx
@@ -1394,7 +1394,7 @@
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="B17">
         <v>847</v>
@@ -1459,7 +1459,7 @@
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="B18">
         <v>847</v>
@@ -1524,7 +1524,7 @@
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="B19">
         <v>847</v>
@@ -1589,7 +1589,7 @@
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="B20">
         <v>847</v>
@@ -1654,7 +1654,7 @@
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="B21">
         <v>847</v>
@@ -1719,7 +1719,7 @@
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="B22">
         <v>847</v>
@@ -1784,7 +1784,7 @@
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="B23">
         <v>847</v>
@@ -1849,7 +1849,7 @@
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="C24" t="str">
         <v>0795T::SGSGZIMER5208::BL</v>
@@ -1876,10 +1876,10 @@
         <v>46225</v>
       </c>
       <c r="S24">
-        <v>46228</v>
+        <v>46227</v>
       </c>
       <c r="T24">
-        <v>46231</v>
+        <v>46230</v>
       </c>
       <c r="V24" t="str">
         <v>1675 Dinusha Guantillake</v>
@@ -2665,10 +2665,10 @@
         <v>46223</v>
       </c>
       <c r="S36">
-        <v>46237</v>
+        <v>46232</v>
       </c>
       <c r="T36">
-        <v>46239</v>
+        <v>46234</v>
       </c>
       <c r="V36" t="str">
         <v>1675 Dinusha Guantillake</v>
@@ -3421,10 +3421,10 @@
         <v>46226</v>
       </c>
       <c r="S48">
-        <v>46240</v>
+        <v>46235</v>
       </c>
       <c r="T48">
-        <v>46246</v>
+        <v>46241</v>
       </c>
       <c r="V48" t="str">
         <v>1675 Dinusha Guantillake</v>
@@ -3592,10 +3592,10 @@
         <v>46239</v>
       </c>
       <c r="S51">
-        <v>46247</v>
+        <v>46242</v>
       </c>
       <c r="T51">
-        <v>46253</v>
+        <v>46248</v>
       </c>
       <c r="V51" t="str">
         <v>1702 Piyumi Perera</v>
@@ -3698,10 +3698,10 @@
         <v>46246</v>
       </c>
       <c r="S53">
-        <v>46254</v>
+        <v>46249</v>
       </c>
       <c r="T53">
-        <v>46255</v>
+        <v>46251</v>
       </c>
       <c r="V53" t="str">
         <v>1702 Piyumi Perera</v>
@@ -3798,10 +3798,10 @@
         <v>46248</v>
       </c>
       <c r="S55">
-        <v>46256</v>
+        <v>46252</v>
       </c>
       <c r="T55">
-        <v>46262</v>
+        <v>46258</v>
       </c>
       <c r="V55" t="str">
         <v>275 Hashan De Mel</v>
@@ -4335,10 +4335,10 @@
         <v>46255</v>
       </c>
       <c r="S64">
-        <v>46263</v>
+        <v>46259</v>
       </c>
       <c r="T64">
-        <v>46269</v>
+        <v>46265</v>
       </c>
       <c r="W64">
         <v>46279</v>
@@ -4975,10 +4975,10 @@
         <v>46224</v>
       </c>
       <c r="S75">
-        <v>46232</v>
+        <v>46228</v>
       </c>
       <c r="T75">
-        <v>46235</v>
+        <v>46231</v>
       </c>
       <c r="V75" t="str">
         <v>1675 Dinusha Guantillake</v>
@@ -5764,10 +5764,10 @@
         <v>46227</v>
       </c>
       <c r="S87">
-        <v>46227</v>
+        <v>46231</v>
       </c>
       <c r="T87">
-        <v>46238</v>
+        <v>46241</v>
       </c>
       <c r="V87" t="str">
         <v>1675 Dinusha Guantillake</v>
@@ -6621,10 +6621,10 @@
         <v>46239</v>
       </c>
       <c r="S100">
-        <v>46239</v>
+        <v>46242</v>
       </c>
       <c r="T100">
-        <v>46247</v>
+        <v>46251</v>
       </c>
       <c r="V100" t="str">
         <v>1675 Dinusha Guantillake</v>
@@ -7344,10 +7344,10 @@
         <v>46251</v>
       </c>
       <c r="S112">
-        <v>46248</v>
+        <v>46252</v>
       </c>
       <c r="T112">
-        <v>46258</v>
+        <v>46261</v>
       </c>
       <c r="W112">
         <v>46275</v>

</xml_diff>

<commit_message>
SGL FR Plan — 31/07/2026 10:50
</commit_message>
<xml_diff>
--- a/Production_Plan.xlsx
+++ b/Production_Plan.xlsx
@@ -1394,7 +1394,7 @@
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>SGL 02</v>
+        <v>SGL 01</v>
       </c>
       <c r="B17">
         <v>847</v>
@@ -1459,7 +1459,7 @@
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>SGL 02</v>
+        <v>SGL 01</v>
       </c>
       <c r="B18">
         <v>847</v>
@@ -1524,7 +1524,7 @@
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>SGL 02</v>
+        <v>SGL 01</v>
       </c>
       <c r="B19">
         <v>847</v>
@@ -1589,7 +1589,7 @@
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>SGL 02</v>
+        <v>SGL 01</v>
       </c>
       <c r="B20">
         <v>847</v>
@@ -1654,7 +1654,7 @@
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>SGL 02</v>
+        <v>SGL 01</v>
       </c>
       <c r="B21">
         <v>847</v>
@@ -1719,7 +1719,7 @@
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>SGL 02</v>
+        <v>SGL 01</v>
       </c>
       <c r="B22">
         <v>847</v>
@@ -1784,7 +1784,7 @@
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>SGL 02</v>
+        <v>SGL 01</v>
       </c>
       <c r="B23">
         <v>847</v>
@@ -1849,7 +1849,7 @@
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>SGL 02</v>
+        <v>SGL 01</v>
       </c>
       <c r="C24" t="str">
         <v>0795T::SGSGZIMER5208::BL</v>
@@ -1879,7 +1879,7 @@
         <v>46227</v>
       </c>
       <c r="T24">
-        <v>46230</v>
+        <v>46231</v>
       </c>
       <c r="V24" t="str">
         <v>1675 Dinusha Guantillake</v>
@@ -2665,7 +2665,7 @@
         <v>46223</v>
       </c>
       <c r="S36">
-        <v>46232</v>
+        <v>46231</v>
       </c>
       <c r="T36">
         <v>46234</v>
@@ -3421,7 +3421,7 @@
         <v>46226</v>
       </c>
       <c r="S48">
-        <v>46235</v>
+        <v>46234</v>
       </c>
       <c r="T48">
         <v>46241</v>
@@ -3592,7 +3592,7 @@
         <v>46239</v>
       </c>
       <c r="S51">
-        <v>46242</v>
+        <v>46241</v>
       </c>
       <c r="T51">
         <v>46248</v>
@@ -3698,7 +3698,7 @@
         <v>46246</v>
       </c>
       <c r="S53">
-        <v>46249</v>
+        <v>46248</v>
       </c>
       <c r="T53">
         <v>46251</v>
@@ -3798,7 +3798,7 @@
         <v>46248</v>
       </c>
       <c r="S55">
-        <v>46252</v>
+        <v>46251</v>
       </c>
       <c r="T55">
         <v>46258</v>
@@ -4335,7 +4335,7 @@
         <v>46255</v>
       </c>
       <c r="S64">
-        <v>46259</v>
+        <v>46258</v>
       </c>
       <c r="T64">
         <v>46265</v>
@@ -4753,7 +4753,7 @@
     </row>
     <row r="72">
       <c r="A72" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="B72">
         <v>847</v>
@@ -4818,7 +4818,7 @@
     </row>
     <row r="73">
       <c r="A73" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="B73">
         <v>847</v>
@@ -4883,7 +4883,7 @@
     </row>
     <row r="74">
       <c r="A74" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="B74">
         <v>847</v>
@@ -4948,7 +4948,7 @@
     </row>
     <row r="75">
       <c r="A75" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="C75" t="str">
         <v>3497A::SGSGZIMER5060::SH</v>
@@ -4975,10 +4975,10 @@
         <v>46224</v>
       </c>
       <c r="S75">
-        <v>46228</v>
+        <v>46226</v>
       </c>
       <c r="T75">
-        <v>46231</v>
+        <v>46230</v>
       </c>
       <c r="V75" t="str">
         <v>1675 Dinusha Guantillake</v>
@@ -5764,7 +5764,7 @@
         <v>46227</v>
       </c>
       <c r="S87">
-        <v>46231</v>
+        <v>46230</v>
       </c>
       <c r="T87">
         <v>46241</v>
@@ -6621,7 +6621,7 @@
         <v>46239</v>
       </c>
       <c r="S100">
-        <v>46242</v>
+        <v>46241</v>
       </c>
       <c r="T100">
         <v>46251</v>
@@ -7344,10 +7344,10 @@
         <v>46251</v>
       </c>
       <c r="S112">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="T112">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="W112">
         <v>46275</v>

</xml_diff>

<commit_message>
SGL FR Plan — 03/08/2026 16:17
</commit_message>
<xml_diff>
--- a/Production_Plan.xlsx
+++ b/Production_Plan.xlsx
@@ -17698,6 +17698,9 @@
       <c r="W302">
         <v>46240</v>
       </c>
+      <c r="X302" t="str">
+        <v>MG-4628g0</v>
+      </c>
     </row>
     <row r="303">
       <c r="A303" t="str">
@@ -17736,6 +17739,9 @@
       <c r="W303">
         <v>46240</v>
       </c>
+      <c r="X303" t="str">
+        <v>MG-4628g0</v>
+      </c>
     </row>
     <row r="304">
       <c r="A304" t="str">
@@ -17801,6 +17807,9 @@
       <c r="W304">
         <v>46240</v>
       </c>
+      <c r="X304" t="str">
+        <v>MG-4628g0</v>
+      </c>
     </row>
     <row r="305">
       <c r="A305" t="str">
@@ -17838,6 +17847,9 @@
       </c>
       <c r="W305">
         <v>46240</v>
+      </c>
+      <c r="X305" t="str">
+        <v>MG-4628g0</v>
       </c>
     </row>
     <row r="306">

</xml_diff>

<commit_message>
SGL FR Plan — 12/08/2026 15:57
</commit_message>
<xml_diff>
--- a/Production_Plan.xlsx
+++ b/Production_Plan.xlsx
@@ -32,10 +32,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
-  <numFmts count="3">
+  <numFmts count="2">
     <numFmt numFmtId="56" formatCode="&quot;上午/下午 &quot;hh&quot;時&quot;mm&quot;分&quot;ss&quot;秒 &quot;"/>
     <numFmt numFmtId="60" formatCode="m/d/yyyy"/>
-    <numFmt numFmtId="164" formatCode="M/d/yyyy"/>
   </numFmts>
   <fonts count="1">
     <font>
@@ -5228,7 +5227,7 @@
     </row>
     <row r="74">
       <c r="A74" t="str">
-        <v>SGL 02</v>
+        <v>SGL 01</v>
       </c>
       <c r="B74">
         <v>847</v>
@@ -5282,13 +5281,13 @@
         <v>46295</v>
       </c>
       <c r="T74" s="2">
-        <v>0.2986111111111111</v>
+        <v>0.6104166666666667</v>
       </c>
       <c r="U74" s="1">
         <v>46296</v>
       </c>
       <c r="V74" s="2">
-        <v>0.6715277777777777</v>
+        <v>0.5041666666666667</v>
       </c>
       <c r="Y74" s="1">
         <v>46317</v>
@@ -5296,7 +5295,7 @@
     </row>
     <row r="75">
       <c r="A75" t="str">
-        <v>SGL 02</v>
+        <v>SGL 01</v>
       </c>
       <c r="C75" t="str">
         <v>3573T/R1-A1::SGSGZIMER6486::BL</v>
@@ -5323,10 +5322,10 @@
         <v>46293</v>
       </c>
       <c r="S75" s="1">
-        <v>46293</v>
+        <v>46295</v>
       </c>
       <c r="U75" s="1">
-        <v>46294</v>
+        <v>46297</v>
       </c>
       <c r="Y75" s="1">
         <v>46317</v>
@@ -8493,7 +8492,7 @@
         <v>46283</v>
       </c>
       <c r="T121" s="2">
-        <v>0.30416666666666664</v>
+        <v>0.5673611111111111</v>
       </c>
       <c r="U121" s="1">
         <v>46283</v>
@@ -8635,7 +8634,7 @@
         <v>46293</v>
       </c>
       <c r="V123" s="2">
-        <v>0.29791666666666666</v>
+        <v>0.5611111111111111</v>
       </c>
       <c r="Y123" s="1">
         <v>46305</v>
@@ -8670,10 +8669,10 @@
         <v>46281</v>
       </c>
       <c r="S124" s="1">
-        <v>46283</v>
+        <v>46266</v>
       </c>
       <c r="U124" s="1">
-        <v>46293</v>
+        <v>46275</v>
       </c>
       <c r="Y124" s="1">
         <v>46305</v>
@@ -8738,13 +8737,13 @@
         <v>46293</v>
       </c>
       <c r="T125" s="2">
-        <v>0.6722222222222223</v>
+        <v>0.5618055555555556</v>
       </c>
       <c r="U125" s="1">
         <v>46301</v>
       </c>
       <c r="V125" s="2">
-        <v>0.38333333333333336</v>
+        <v>0.7520833333333333</v>
       </c>
       <c r="Y125" s="1">
         <v>46305</v>
@@ -8779,10 +8778,10 @@
         <v>46290</v>
       </c>
       <c r="S126" s="1">
-        <v>46294</v>
+        <v>46275</v>
       </c>
       <c r="U126" s="1">
-        <v>46303</v>
+        <v>46283</v>
       </c>
       <c r="Y126" s="1">
         <v>46305</v>
@@ -11640,7 +11639,7 @@
     </row>
     <row r="169">
       <c r="A169" t="str">
-        <v>SGL 03</v>
+        <v>SGL 02</v>
       </c>
       <c r="B169">
         <v>547</v>
@@ -11697,13 +11696,13 @@
         <v>46265</v>
       </c>
       <c r="T169" s="2">
-        <v>0.3548611111111111</v>
+        <v>0.42777777777777776</v>
       </c>
       <c r="U169" s="1">
         <v>46266</v>
       </c>
       <c r="V169" s="2">
-        <v>0.49375</v>
+        <v>0.5666666666666667</v>
       </c>
       <c r="Y169" s="1">
         <v>46247</v>
@@ -11711,7 +11710,7 @@
     </row>
     <row r="170">
       <c r="A170" t="str">
-        <v>SGL 03</v>
+        <v>SGL 02</v>
       </c>
       <c r="C170" t="str">
         <v>559784P::OVOVLE-BO4466::BZ</v>
@@ -11806,13 +11805,13 @@
         <v>46266</v>
       </c>
       <c r="T171" s="2">
-        <v>0.49444444444444446</v>
+        <v>0.3548611111111111</v>
       </c>
       <c r="U171" s="1">
         <v>46269</v>
       </c>
       <c r="V171" s="2">
-        <v>0.3819444444444444</v>
+        <v>0.7215277777777778</v>
       </c>
       <c r="Y171" s="1">
         <v>46247</v>
@@ -11847,10 +11846,10 @@
         <v>46263</v>
       </c>
       <c r="S172" s="1">
-        <v>46266</v>
+        <v>46265</v>
       </c>
       <c r="U172" s="1">
-        <v>46269</v>
+        <v>46267</v>
       </c>
       <c r="Y172" s="1">
         <v>46247</v>
@@ -11915,13 +11914,13 @@
         <v>46269</v>
       </c>
       <c r="T173" s="2">
-        <v>0.38263888888888886</v>
+        <v>0.7222222222222222</v>
       </c>
       <c r="U173" s="1">
         <v>46272</v>
       </c>
       <c r="V173" s="2">
-        <v>0.3215277777777778</v>
+        <v>0.6611111111111111</v>
       </c>
       <c r="Y173" s="1">
         <v>46247</v>
@@ -11956,10 +11955,10 @@
         <v>46267</v>
       </c>
       <c r="S174" s="1">
+        <v>46267</v>
+      </c>
+      <c r="U174" s="1">
         <v>46269</v>
-      </c>
-      <c r="U174" s="1">
-        <v>46272</v>
       </c>
       <c r="Y174" s="1">
         <v>46247</v>
@@ -12021,13 +12020,13 @@
         <v>46283</v>
       </c>
       <c r="T175" s="2">
-        <v>0.2916666666666667</v>
+        <v>0.6618055555555555</v>
       </c>
       <c r="U175" s="1">
         <v>46284</v>
       </c>
       <c r="V175" s="2">
-        <v>0.4388888888888889</v>
+        <v>0.3298611111111111</v>
       </c>
       <c r="X175" t="str">
         <v>1702 Piyumi Perera</v>
@@ -12065,10 +12064,10 @@
         <v>46281</v>
       </c>
       <c r="S176" s="1">
-        <v>46283</v>
+        <v>46269</v>
       </c>
       <c r="U176" s="1">
-        <v>46284</v>
+        <v>46272</v>
       </c>
       <c r="X176" t="str">
         <v>1702 Piyumi Perera</v>
@@ -12133,7 +12132,7 @@
         <v>46284</v>
       </c>
       <c r="T177" s="2">
-        <v>0.4395833333333333</v>
+        <v>0.33055555555555555</v>
       </c>
       <c r="U177" s="1">
         <v>46286</v>
@@ -12207,7 +12206,7 @@
         <v>46298</v>
       </c>
       <c r="V178" s="2">
-        <v>0.3736111111111111</v>
+        <v>0.74375</v>
       </c>
       <c r="Y178" s="1">
         <v>46305</v>
@@ -12242,10 +12241,10 @@
         <v>46282</v>
       </c>
       <c r="S179" s="1">
-        <v>46284</v>
+        <v>46272</v>
       </c>
       <c r="U179" s="1">
-        <v>46301</v>
+        <v>46287</v>
       </c>
       <c r="Y179" s="1">
         <v>46305</v>

</xml_diff>

<commit_message>
SGL FR Plan — 12/08/2026 16:37
</commit_message>
<xml_diff>
--- a/Production_Plan.xlsx
+++ b/Production_Plan.xlsx
@@ -8492,7 +8492,7 @@
         <v>46283</v>
       </c>
       <c r="T121" s="2">
-        <v>0.5673611111111111</v>
+        <v>0.30416666666666664</v>
       </c>
       <c r="U121" s="1">
         <v>46283</v>
@@ -8634,7 +8634,7 @@
         <v>46293</v>
       </c>
       <c r="V123" s="2">
-        <v>0.5611111111111111</v>
+        <v>0.29791666666666666</v>
       </c>
       <c r="Y123" s="1">
         <v>46305</v>
@@ -8669,10 +8669,10 @@
         <v>46281</v>
       </c>
       <c r="S124" s="1">
-        <v>46266</v>
+        <v>46283</v>
       </c>
       <c r="U124" s="1">
-        <v>46275</v>
+        <v>46293</v>
       </c>
       <c r="Y124" s="1">
         <v>46305</v>
@@ -8737,13 +8737,13 @@
         <v>46293</v>
       </c>
       <c r="T125" s="2">
-        <v>0.5618055555555556</v>
+        <v>0.2986111111111111</v>
       </c>
       <c r="U125" s="1">
         <v>46301</v>
       </c>
       <c r="V125" s="2">
-        <v>0.7520833333333333</v>
+        <v>0.4888888888888889</v>
       </c>
       <c r="Y125" s="1">
         <v>46305</v>
@@ -8778,10 +8778,10 @@
         <v>46290</v>
       </c>
       <c r="S126" s="1">
-        <v>46275</v>
+        <v>46293</v>
       </c>
       <c r="U126" s="1">
-        <v>46283</v>
+        <v>46301</v>
       </c>
       <c r="Y126" s="1">
         <v>46305</v>
@@ -11639,7 +11639,7 @@
     </row>
     <row r="169">
       <c r="A169" t="str">
-        <v>SGL 02</v>
+        <v>SGL 03</v>
       </c>
       <c r="B169">
         <v>547</v>
@@ -11696,13 +11696,13 @@
         <v>46265</v>
       </c>
       <c r="T169" s="2">
-        <v>0.42777777777777776</v>
+        <v>0.3548611111111111</v>
       </c>
       <c r="U169" s="1">
         <v>46266</v>
       </c>
       <c r="V169" s="2">
-        <v>0.5666666666666667</v>
+        <v>0.49375</v>
       </c>
       <c r="Y169" s="1">
         <v>46247</v>
@@ -11710,7 +11710,7 @@
     </row>
     <row r="170">
       <c r="A170" t="str">
-        <v>SGL 02</v>
+        <v>SGL 03</v>
       </c>
       <c r="C170" t="str">
         <v>559784P::OVOVLE-BO4466::BZ</v>
@@ -11805,13 +11805,13 @@
         <v>46266</v>
       </c>
       <c r="T171" s="2">
-        <v>0.3548611111111111</v>
+        <v>0.49444444444444446</v>
       </c>
       <c r="U171" s="1">
         <v>46269</v>
       </c>
       <c r="V171" s="2">
-        <v>0.7215277777777778</v>
+        <v>0.3819444444444444</v>
       </c>
       <c r="Y171" s="1">
         <v>46247</v>
@@ -11846,10 +11846,10 @@
         <v>46263</v>
       </c>
       <c r="S172" s="1">
-        <v>46265</v>
+        <v>46266</v>
       </c>
       <c r="U172" s="1">
-        <v>46267</v>
+        <v>46269</v>
       </c>
       <c r="Y172" s="1">
         <v>46247</v>
@@ -11914,13 +11914,13 @@
         <v>46269</v>
       </c>
       <c r="T173" s="2">
-        <v>0.7222222222222222</v>
+        <v>0.38263888888888886</v>
       </c>
       <c r="U173" s="1">
         <v>46272</v>
       </c>
       <c r="V173" s="2">
-        <v>0.6611111111111111</v>
+        <v>0.3215277777777778</v>
       </c>
       <c r="Y173" s="1">
         <v>46247</v>
@@ -11955,10 +11955,10 @@
         <v>46267</v>
       </c>
       <c r="S174" s="1">
-        <v>46267</v>
+        <v>46269</v>
       </c>
       <c r="U174" s="1">
-        <v>46269</v>
+        <v>46272</v>
       </c>
       <c r="Y174" s="1">
         <v>46247</v>
@@ -12020,13 +12020,13 @@
         <v>46283</v>
       </c>
       <c r="T175" s="2">
-        <v>0.6618055555555555</v>
+        <v>0.2916666666666667</v>
       </c>
       <c r="U175" s="1">
         <v>46284</v>
       </c>
       <c r="V175" s="2">
-        <v>0.3298611111111111</v>
+        <v>0.4388888888888889</v>
       </c>
       <c r="X175" t="str">
         <v>1702 Piyumi Perera</v>
@@ -12064,10 +12064,10 @@
         <v>46281</v>
       </c>
       <c r="S176" s="1">
-        <v>46269</v>
+        <v>46283</v>
       </c>
       <c r="U176" s="1">
-        <v>46272</v>
+        <v>46284</v>
       </c>
       <c r="X176" t="str">
         <v>1702 Piyumi Perera</v>
@@ -12132,7 +12132,7 @@
         <v>46284</v>
       </c>
       <c r="T177" s="2">
-        <v>0.33055555555555555</v>
+        <v>0.4395833333333333</v>
       </c>
       <c r="U177" s="1">
         <v>46286</v>
@@ -12206,7 +12206,7 @@
         <v>46298</v>
       </c>
       <c r="V178" s="2">
-        <v>0.74375</v>
+        <v>0.3736111111111111</v>
       </c>
       <c r="Y178" s="1">
         <v>46305</v>
@@ -12241,10 +12241,10 @@
         <v>46282</v>
       </c>
       <c r="S179" s="1">
-        <v>46272</v>
+        <v>46284</v>
       </c>
       <c r="U179" s="1">
-        <v>46287</v>
+        <v>46301</v>
       </c>
       <c r="Y179" s="1">
         <v>46305</v>
@@ -17748,7 +17748,7 @@
         <v>1515 Sanjaya Mihiran</v>
       </c>
       <c r="Y276" s="1">
-        <v>46219</v>
+        <v>46254</v>
       </c>
     </row>
     <row r="277">

</xml_diff>

<commit_message>
SGL FR Plan — 16/08/2026 19:54
</commit_message>
<xml_diff>
--- a/Production_Plan.xlsx
+++ b/Production_Plan.xlsx
@@ -32,9 +32,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="56" formatCode="&quot;上午/下午 &quot;hh&quot;時&quot;mm&quot;分&quot;ss&quot;秒 &quot;"/>
     <numFmt numFmtId="60" formatCode="m/d/yyyy"/>
+    <numFmt numFmtId="164" formatCode="M/d/yyyy"/>
   </numFmts>
   <fonts count="1">
     <font>
@@ -1010,7 +1011,7 @@
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="B10">
         <v>847</v>
@@ -1067,7 +1068,7 @@
         <v>46241</v>
       </c>
       <c r="T10" s="2">
-        <v>0.2951388888888889</v>
+        <v>0.5770833333333333</v>
       </c>
       <c r="U10" s="1">
         <v>46241</v>
@@ -1084,7 +1085,7 @@
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="B11">
         <v>847</v>
@@ -1158,7 +1159,7 @@
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="B12">
         <v>847</v>
@@ -1232,7 +1233,7 @@
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="B13">
         <v>847</v>
@@ -1306,7 +1307,7 @@
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="B14">
         <v>847</v>
@@ -1380,7 +1381,7 @@
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="B15">
         <v>847</v>
@@ -1454,7 +1455,7 @@
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="B16">
         <v>847</v>
@@ -1528,7 +1529,7 @@
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="B17">
         <v>847</v>
@@ -1602,7 +1603,7 @@
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="B18">
         <v>847</v>
@@ -1676,7 +1677,7 @@
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="B19">
         <v>847</v>
@@ -1750,7 +1751,7 @@
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="B20">
         <v>847</v>
@@ -1813,7 +1814,7 @@
         <v>46245</v>
       </c>
       <c r="V20" s="2">
-        <v>0.325</v>
+        <v>0.6069444444444444</v>
       </c>
       <c r="X20" t="str">
         <v>1675 Dinusha Guantillake</v>
@@ -1824,7 +1825,7 @@
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="C21" t="str">
         <v>1500P/R1::SGSGZIMER5206::PN</v>
@@ -1851,10 +1852,10 @@
         <v>-</v>
       </c>
       <c r="S21" s="1">
-        <v>46241</v>
+        <v>46244</v>
       </c>
       <c r="U21" s="1">
-        <v>46245</v>
+        <v>46247</v>
       </c>
       <c r="X21" t="str">
         <v>1675 Dinusha Guantillake</v>
@@ -1922,7 +1923,7 @@
         <v>46245</v>
       </c>
       <c r="T22" s="2">
-        <v>0.32569444444444445</v>
+        <v>0.2951388888888889</v>
       </c>
       <c r="U22" s="1">
         <v>46245</v>
@@ -3038,7 +3039,7 @@
         <v>46251</v>
       </c>
       <c r="V37" s="2">
-        <v>0.6930555555555555</v>
+        <v>0.6625</v>
       </c>
       <c r="X37" t="str">
         <v>1702 Piyumi Perera</v>
@@ -3076,10 +3077,10 @@
         <v>46242</v>
       </c>
       <c r="S38" s="1">
-        <v>46245</v>
+        <v>46241</v>
       </c>
       <c r="U38" s="1">
-        <v>46251</v>
+        <v>46247</v>
       </c>
       <c r="X38" t="str">
         <v>1702 Piyumi Perera</v>
@@ -3147,7 +3148,7 @@
         <v>46251</v>
       </c>
       <c r="T39" s="2">
-        <v>0.69375</v>
+        <v>0.6631944444444444</v>
       </c>
       <c r="U39" s="1">
         <v>46255</v>
@@ -3650,7 +3651,7 @@
         <v>46259</v>
       </c>
       <c r="V46" s="2">
-        <v>0.5284722222222222</v>
+        <v>0.4979166666666667</v>
       </c>
       <c r="Y46" s="1">
         <v>46266</v>
@@ -3685,10 +3686,10 @@
         <v>46248</v>
       </c>
       <c r="S47" s="1">
-        <v>46251</v>
+        <v>46247</v>
       </c>
       <c r="U47" s="1">
-        <v>46259</v>
+        <v>46255</v>
       </c>
       <c r="Y47" s="1">
         <v>46266</v>
@@ -3750,13 +3751,13 @@
         <v>46259</v>
       </c>
       <c r="T48" s="2">
-        <v>0.5291666666666667</v>
+        <v>0.4986111111111111</v>
       </c>
       <c r="U48" s="1">
         <v>46262</v>
       </c>
       <c r="V48" s="2">
-        <v>0.6326388888888889</v>
+        <v>0.6020833333333333</v>
       </c>
       <c r="Y48" s="1">
         <v>46265</v>
@@ -3791,10 +3792,10 @@
         <v>46256</v>
       </c>
       <c r="S49" s="1">
+        <v>46255</v>
+      </c>
+      <c r="U49" s="1">
         <v>46259</v>
-      </c>
-      <c r="U49" s="1">
-        <v>46262</v>
       </c>
       <c r="Y49" s="1">
         <v>46265</v>
@@ -3859,7 +3860,7 @@
         <v>46262</v>
       </c>
       <c r="T50" s="2">
-        <v>0.6333333333333333</v>
+        <v>0.6027777777777777</v>
       </c>
       <c r="U50" s="1">
         <v>46263</v>
@@ -4235,7 +4236,7 @@
         <v>46266</v>
       </c>
       <c r="V55" s="2">
-        <v>0.6055555555555555</v>
+        <v>0.575</v>
       </c>
       <c r="X55" t="str">
         <v>1702 Piyumi Perera</v>
@@ -4273,10 +4274,10 @@
         <v>46260</v>
       </c>
       <c r="S56" s="1">
+        <v>46259</v>
+      </c>
+      <c r="U56" s="1">
         <v>46262</v>
-      </c>
-      <c r="U56" s="1">
-        <v>46266</v>
       </c>
       <c r="X56" t="str">
         <v>1702 Piyumi Perera</v>
@@ -4344,13 +4345,13 @@
         <v>46266</v>
       </c>
       <c r="T57" s="2">
-        <v>0.60625</v>
+        <v>0.5756944444444444</v>
       </c>
       <c r="U57" s="1">
         <v>46267</v>
       </c>
       <c r="V57" s="2">
-        <v>0.48055555555555557</v>
+        <v>0.45</v>
       </c>
       <c r="X57" t="str">
         <v>1702 Piyumi Perera</v>
@@ -4388,10 +4389,10 @@
         <v>46263</v>
       </c>
       <c r="S58" s="1">
-        <v>46266</v>
+        <v>46262</v>
       </c>
       <c r="U58" s="1">
-        <v>46267</v>
+        <v>46263</v>
       </c>
       <c r="X58" t="str">
         <v>1702 Piyumi Perera</v>
@@ -4456,13 +4457,13 @@
         <v>46267</v>
       </c>
       <c r="T59" s="2">
-        <v>0.48125</v>
+        <v>0.45069444444444445</v>
       </c>
       <c r="U59" s="1">
         <v>46269</v>
       </c>
       <c r="V59" s="2">
-        <v>0.34652777777777777</v>
+        <v>0.3159722222222222</v>
       </c>
       <c r="Y59" s="1">
         <v>46277</v>
@@ -4497,10 +4498,10 @@
         <v>46265</v>
       </c>
       <c r="S60" s="1">
-        <v>46267</v>
+        <v>46263</v>
       </c>
       <c r="U60" s="1">
-        <v>46269</v>
+        <v>46266</v>
       </c>
       <c r="Y60" s="1">
         <v>46277</v>
@@ -4565,13 +4566,13 @@
         <v>46269</v>
       </c>
       <c r="T61" s="2">
-        <v>0.34791666666666665</v>
+        <v>0.31666666666666665</v>
       </c>
       <c r="U61" s="1">
         <v>46276</v>
       </c>
       <c r="V61" s="2">
-        <v>0.3263888888888889</v>
+        <v>0.2951388888888889</v>
       </c>
       <c r="X61" t="str">
         <v>1702 Piyumi Perera</v>
@@ -4609,10 +4610,10 @@
         <v>46267</v>
       </c>
       <c r="S62" s="1">
-        <v>46269</v>
+        <v>46266</v>
       </c>
       <c r="U62" s="1">
-        <v>46276</v>
+        <v>46273</v>
       </c>
       <c r="X62" t="str">
         <v>1702 Piyumi Perera</v>
@@ -4680,7 +4681,7 @@
         <v>46276</v>
       </c>
       <c r="T63" s="2">
-        <v>0.32708333333333334</v>
+        <v>0.29583333333333334</v>
       </c>
       <c r="U63" s="1">
         <v>46276</v>
@@ -4757,7 +4758,7 @@
         <v>46279</v>
       </c>
       <c r="V64" s="2">
-        <v>0.33055555555555555</v>
+        <v>0.29930555555555555</v>
       </c>
       <c r="Y64" s="1">
         <v>46298</v>
@@ -4792,10 +4793,10 @@
         <v>46274</v>
       </c>
       <c r="S65" s="1">
-        <v>46276</v>
+        <v>46273</v>
       </c>
       <c r="U65" s="1">
-        <v>46279</v>
+        <v>46275</v>
       </c>
       <c r="Y65" s="1">
         <v>46298</v>
@@ -4857,13 +4858,13 @@
         <v>46279</v>
       </c>
       <c r="T66" s="2">
-        <v>0.33125</v>
+        <v>0.3</v>
       </c>
       <c r="U66" s="1">
         <v>46283</v>
       </c>
       <c r="V66" s="2">
-        <v>0.4625</v>
+        <v>0.43125</v>
       </c>
       <c r="Y66" s="1">
         <v>46301</v>
@@ -4898,10 +4899,10 @@
         <v>46276</v>
       </c>
       <c r="S67" s="1">
-        <v>46279</v>
+        <v>46275</v>
       </c>
       <c r="U67" s="1">
-        <v>46283</v>
+        <v>46280</v>
       </c>
       <c r="Y67" s="1">
         <v>46301</v>
@@ -4963,13 +4964,13 @@
         <v>46283</v>
       </c>
       <c r="T68" s="2">
-        <v>0.46319444444444446</v>
+        <v>0.43194444444444446</v>
       </c>
       <c r="U68" s="1">
         <v>46286</v>
       </c>
       <c r="V68" s="2">
-        <v>0.5381944444444444</v>
+        <v>0.5069444444444444</v>
       </c>
       <c r="Y68" s="1">
         <v>46304</v>
@@ -5004,10 +5005,10 @@
         <v>46281</v>
       </c>
       <c r="S69" s="1">
-        <v>46283</v>
+        <v>46280</v>
       </c>
       <c r="U69" s="1">
-        <v>46286</v>
+        <v>46282</v>
       </c>
       <c r="Y69" s="1">
         <v>46304</v>
@@ -5069,13 +5070,13 @@
         <v>46286</v>
       </c>
       <c r="T70" s="2">
-        <v>0.5388888888888889</v>
+        <v>0.5076388888888889</v>
       </c>
       <c r="U70" s="1">
         <v>46293</v>
       </c>
       <c r="V70" s="2">
-        <v>0.49444444444444446</v>
+        <v>0.46319444444444446</v>
       </c>
       <c r="Y70" s="1">
         <v>46301</v>
@@ -5110,10 +5111,10 @@
         <v>46283</v>
       </c>
       <c r="S71" s="1">
-        <v>46286</v>
+        <v>46282</v>
       </c>
       <c r="U71" s="1">
-        <v>46293</v>
+        <v>46289</v>
       </c>
       <c r="Y71" s="1">
         <v>46301</v>
@@ -5175,13 +5176,13 @@
         <v>46293</v>
       </c>
       <c r="T72" s="2">
-        <v>0.4951388888888889</v>
+        <v>0.4638888888888889</v>
       </c>
       <c r="U72" s="1">
         <v>46295</v>
       </c>
       <c r="V72" s="2">
-        <v>0.6097222222222223</v>
+        <v>0.5784722222222223</v>
       </c>
       <c r="Y72" s="1">
         <v>46304</v>
@@ -5216,10 +5217,10 @@
         <v>46290</v>
       </c>
       <c r="S73" s="1">
-        <v>46293</v>
+        <v>46289</v>
       </c>
       <c r="U73" s="1">
-        <v>46295</v>
+        <v>46291</v>
       </c>
       <c r="Y73" s="1">
         <v>46304</v>
@@ -5281,13 +5282,13 @@
         <v>46295</v>
       </c>
       <c r="T74" s="2">
-        <v>0.6104166666666667</v>
+        <v>0.5791666666666667</v>
       </c>
       <c r="U74" s="1">
         <v>46296</v>
       </c>
       <c r="V74" s="2">
-        <v>0.5041666666666667</v>
+        <v>0.47291666666666665</v>
       </c>
       <c r="Y74" s="1">
         <v>46317</v>
@@ -5322,10 +5323,10 @@
         <v>46293</v>
       </c>
       <c r="S75" s="1">
-        <v>46295</v>
+        <v>46291</v>
       </c>
       <c r="U75" s="1">
-        <v>46297</v>
+        <v>46294</v>
       </c>
       <c r="Y75" s="1">
         <v>46317</v>
@@ -6245,7 +6246,7 @@
         <v>46244</v>
       </c>
       <c r="T88" s="2">
-        <v>0.5770833333333333</v>
+        <v>0.6076388888888888</v>
       </c>
       <c r="U88" s="1">
         <v>46245</v>
@@ -7065,7 +7066,7 @@
         <v>46253</v>
       </c>
       <c r="V99" s="2">
-        <v>0.6222222222222222</v>
+        <v>0.6527777777777778</v>
       </c>
       <c r="X99" t="str">
         <v>1675 Dinusha Guantillake</v>
@@ -7103,10 +7104,10 @@
         <v>46241</v>
       </c>
       <c r="S100" s="1">
-        <v>46244</v>
+        <v>46247</v>
       </c>
       <c r="U100" s="1">
-        <v>46253</v>
+        <v>46256</v>
       </c>
       <c r="X100" t="str">
         <v>1675 Dinusha Guantillake</v>
@@ -7171,7 +7172,7 @@
         <v>46253</v>
       </c>
       <c r="T101" s="2">
-        <v>0.6229166666666667</v>
+        <v>0.6534722222222222</v>
       </c>
       <c r="U101" s="1">
         <v>46254</v>
@@ -7461,7 +7462,7 @@
         <v>46255</v>
       </c>
       <c r="V105" s="2">
-        <v>0.5631944444444444</v>
+        <v>0.59375</v>
       </c>
       <c r="X105" t="str">
         <v>1702 Piyumi Perera</v>
@@ -7499,10 +7500,10 @@
         <v>46251</v>
       </c>
       <c r="S106" s="1">
-        <v>46253</v>
+        <v>46256</v>
       </c>
       <c r="U106" s="1">
-        <v>46255</v>
+        <v>46259</v>
       </c>
       <c r="X106" t="str">
         <v>1702 Piyumi Perera</v>
@@ -7567,13 +7568,13 @@
         <v>46255</v>
       </c>
       <c r="T107" s="2">
-        <v>0.5638888888888889</v>
+        <v>0.5944444444444444</v>
       </c>
       <c r="U107" s="1">
         <v>46259</v>
       </c>
       <c r="V107" s="2">
-        <v>0.5270833333333333</v>
+        <v>0.5576388888888889</v>
       </c>
       <c r="Y107" s="1">
         <v>46265</v>
@@ -7608,10 +7609,10 @@
         <v>46253</v>
       </c>
       <c r="S108" s="1">
-        <v>46255</v>
+        <v>46259</v>
       </c>
       <c r="U108" s="1">
-        <v>46259</v>
+        <v>46262</v>
       </c>
       <c r="Y108" s="1">
         <v>46265</v>
@@ -7676,7 +7677,7 @@
         <v>46259</v>
       </c>
       <c r="T109" s="2">
-        <v>0.5277777777777778</v>
+        <v>0.5583333333333333</v>
       </c>
       <c r="U109" s="1">
         <v>46262</v>
@@ -8392,7 +8393,7 @@
         <v>46265</v>
       </c>
       <c r="V119" s="2">
-        <v>0.4270833333333333</v>
+        <v>0.4576388888888889</v>
       </c>
       <c r="Y119" s="1">
         <v>46275</v>
@@ -8427,10 +8428,10 @@
         <v>46256</v>
       </c>
       <c r="S120" s="1">
-        <v>46259</v>
+        <v>46262</v>
       </c>
       <c r="U120" s="1">
-        <v>46265</v>
+        <v>46268</v>
       </c>
       <c r="Y120" s="1">
         <v>46275</v>
@@ -8492,7 +8493,7 @@
         <v>46283</v>
       </c>
       <c r="T121" s="2">
-        <v>0.30416666666666664</v>
+        <v>0.4583333333333333</v>
       </c>
       <c r="U121" s="1">
         <v>46283</v>
@@ -8634,7 +8635,7 @@
         <v>46293</v>
       </c>
       <c r="V123" s="2">
-        <v>0.29791666666666666</v>
+        <v>0.45208333333333334</v>
       </c>
       <c r="Y123" s="1">
         <v>46305</v>
@@ -8669,10 +8670,10 @@
         <v>46281</v>
       </c>
       <c r="S124" s="1">
-        <v>46283</v>
+        <v>46268</v>
       </c>
       <c r="U124" s="1">
-        <v>46293</v>
+        <v>46277</v>
       </c>
       <c r="Y124" s="1">
         <v>46305</v>
@@ -8737,13 +8738,13 @@
         <v>46293</v>
       </c>
       <c r="T125" s="2">
-        <v>0.2986111111111111</v>
+        <v>0.4527777777777778</v>
       </c>
       <c r="U125" s="1">
         <v>46301</v>
       </c>
       <c r="V125" s="2">
-        <v>0.4888888888888889</v>
+        <v>0.6430555555555556</v>
       </c>
       <c r="Y125" s="1">
         <v>46305</v>
@@ -8778,10 +8779,10 @@
         <v>46290</v>
       </c>
       <c r="S126" s="1">
-        <v>46293</v>
+        <v>46277</v>
       </c>
       <c r="U126" s="1">
-        <v>46301</v>
+        <v>46286</v>
       </c>
       <c r="Y126" s="1">
         <v>46305</v>

</xml_diff>

<commit_message>
SGL FR Plan — 17/08/2026 09:25
</commit_message>
<xml_diff>
--- a/Production_Plan.xlsx
+++ b/Production_Plan.xlsx
@@ -13651,6 +13651,9 @@
       <c r="Y203" s="1">
         <v>46254</v>
       </c>
+      <c r="Z203" t="str">
+        <v>MG-k0t91m</v>
+      </c>
     </row>
     <row r="204">
       <c r="A204" t="str">
@@ -13692,6 +13695,9 @@
       <c r="Y204" s="1">
         <v>46254</v>
       </c>
+      <c r="Z204" t="str">
+        <v>MG-k0t91m</v>
+      </c>
     </row>
     <row r="205">
       <c r="A205" t="str">
@@ -13766,6 +13772,9 @@
       <c r="Y205" s="1">
         <v>46254</v>
       </c>
+      <c r="Z205" t="str">
+        <v>MG-k0t91m</v>
+      </c>
     </row>
     <row r="206">
       <c r="A206" t="str">
@@ -13806,6 +13815,9 @@
       </c>
       <c r="Y206" s="1">
         <v>46254</v>
+      </c>
+      <c r="Z206" t="str">
+        <v>MG-k0t91m</v>
       </c>
     </row>
     <row r="207">

</xml_diff>

<commit_message>
SGL FR Plan — 17/08/2026 20:51
</commit_message>
<xml_diff>
--- a/Production_Plan.xlsx
+++ b/Production_Plan.xlsx
@@ -748,7 +748,7 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="B6">
         <v>847</v>
@@ -805,7 +805,7 @@
         <v>46238</v>
       </c>
       <c r="T6" s="2">
-        <v>0.4486111111111111</v>
+        <v>0.4395833333333333</v>
       </c>
       <c r="U6" s="1">
         <v>46240</v>
@@ -822,7 +822,7 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="B7">
         <v>847</v>
@@ -896,7 +896,7 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="B8">
         <v>847</v>
@@ -959,7 +959,7 @@
         <v>46241</v>
       </c>
       <c r="V8" s="2">
-        <v>0.29444444444444445</v>
+        <v>0.7645833333333333</v>
       </c>
       <c r="X8" t="str">
         <v>1675 Dinusha Guantillake</v>
@@ -970,7 +970,7 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>SGL 01</v>
+        <v>SGL 02</v>
       </c>
       <c r="C9" t="str">
         <v>3497A::SGSGZIMER5060::SH</v>
@@ -997,10 +997,10 @@
         <v>0</v>
       </c>
       <c r="S9" s="1">
-        <v>46238</v>
+        <v>46245</v>
       </c>
       <c r="U9" s="1">
-        <v>46241</v>
+        <v>46247</v>
       </c>
       <c r="X9" t="str">
         <v>1675 Dinusha Guantillake</v>
@@ -1068,7 +1068,7 @@
         <v>46241</v>
       </c>
       <c r="T10" s="2">
-        <v>0.5770833333333333</v>
+        <v>0.7652777777777777</v>
       </c>
       <c r="U10" s="1">
         <v>46241</v>
@@ -1814,7 +1814,7 @@
         <v>46245</v>
       </c>
       <c r="V20" s="2">
-        <v>0.6069444444444444</v>
+        <v>0.3159722222222222</v>
       </c>
       <c r="X20" t="str">
         <v>1675 Dinusha Guantillake</v>
@@ -1852,10 +1852,10 @@
         <v>-</v>
       </c>
       <c r="S21" s="1">
-        <v>46244</v>
+        <v>46247</v>
       </c>
       <c r="U21" s="1">
-        <v>46247</v>
+        <v>46252</v>
       </c>
       <c r="X21" t="str">
         <v>1675 Dinusha Guantillake</v>
@@ -1923,7 +1923,7 @@
         <v>46245</v>
       </c>
       <c r="T22" s="2">
-        <v>0.2951388888888889</v>
+        <v>0.4486111111111111</v>
       </c>
       <c r="U22" s="1">
         <v>46245</v>
@@ -3039,7 +3039,7 @@
         <v>46251</v>
       </c>
       <c r="V37" s="2">
-        <v>0.6625</v>
+        <v>0.3368055555555556</v>
       </c>
       <c r="X37" t="str">
         <v>1702 Piyumi Perera</v>
@@ -3077,10 +3077,10 @@
         <v>46242</v>
       </c>
       <c r="S38" s="1">
-        <v>46241</v>
+        <v>46238</v>
       </c>
       <c r="U38" s="1">
-        <v>46247</v>
+        <v>46245</v>
       </c>
       <c r="X38" t="str">
         <v>1702 Piyumi Perera</v>
@@ -3148,7 +3148,7 @@
         <v>46251</v>
       </c>
       <c r="T39" s="2">
-        <v>0.6631944444444444</v>
+        <v>0.3375</v>
       </c>
       <c r="U39" s="1">
         <v>46255</v>
@@ -3651,7 +3651,7 @@
         <v>46259</v>
       </c>
       <c r="V46" s="2">
-        <v>0.4979166666666667</v>
+        <v>0.6513888888888889</v>
       </c>
       <c r="Y46" s="1">
         <v>46266</v>
@@ -3686,10 +3686,10 @@
         <v>46248</v>
       </c>
       <c r="S47" s="1">
-        <v>46247</v>
+        <v>46245</v>
       </c>
       <c r="U47" s="1">
-        <v>46255</v>
+        <v>46252</v>
       </c>
       <c r="Y47" s="1">
         <v>46266</v>
@@ -3751,13 +3751,13 @@
         <v>46259</v>
       </c>
       <c r="T48" s="2">
-        <v>0.4986111111111111</v>
+        <v>0.6520833333333333</v>
       </c>
       <c r="U48" s="1">
         <v>46262</v>
       </c>
       <c r="V48" s="2">
-        <v>0.6020833333333333</v>
+        <v>0.7555555555555555</v>
       </c>
       <c r="Y48" s="1">
         <v>46265</v>
@@ -3792,10 +3792,10 @@
         <v>46256</v>
       </c>
       <c r="S49" s="1">
+        <v>46252</v>
+      </c>
+      <c r="U49" s="1">
         <v>46255</v>
-      </c>
-      <c r="U49" s="1">
-        <v>46259</v>
       </c>
       <c r="Y49" s="1">
         <v>46265</v>
@@ -3860,7 +3860,7 @@
         <v>46262</v>
       </c>
       <c r="T50" s="2">
-        <v>0.6027777777777777</v>
+        <v>0.75625</v>
       </c>
       <c r="U50" s="1">
         <v>46263</v>
@@ -4236,7 +4236,7 @@
         <v>46266</v>
       </c>
       <c r="V55" s="2">
-        <v>0.575</v>
+        <v>0.7284722222222222</v>
       </c>
       <c r="X55" t="str">
         <v>1702 Piyumi Perera</v>
@@ -4274,10 +4274,10 @@
         <v>46260</v>
       </c>
       <c r="S56" s="1">
+        <v>46255</v>
+      </c>
+      <c r="U56" s="1">
         <v>46259</v>
-      </c>
-      <c r="U56" s="1">
-        <v>46262</v>
       </c>
       <c r="X56" t="str">
         <v>1702 Piyumi Perera</v>
@@ -4345,13 +4345,13 @@
         <v>46266</v>
       </c>
       <c r="T57" s="2">
-        <v>0.5756944444444444</v>
+        <v>0.7291666666666666</v>
       </c>
       <c r="U57" s="1">
         <v>46267</v>
       </c>
       <c r="V57" s="2">
-        <v>0.45</v>
+        <v>0.6034722222222222</v>
       </c>
       <c r="X57" t="str">
         <v>1702 Piyumi Perera</v>
@@ -4389,10 +4389,10 @@
         <v>46263</v>
       </c>
       <c r="S58" s="1">
-        <v>46262</v>
+        <v>46259</v>
       </c>
       <c r="U58" s="1">
-        <v>46263</v>
+        <v>46260</v>
       </c>
       <c r="X58" t="str">
         <v>1702 Piyumi Perera</v>
@@ -4457,13 +4457,13 @@
         <v>46267</v>
       </c>
       <c r="T59" s="2">
-        <v>0.45069444444444445</v>
+        <v>0.6041666666666666</v>
       </c>
       <c r="U59" s="1">
         <v>46269</v>
       </c>
       <c r="V59" s="2">
-        <v>0.3159722222222222</v>
+        <v>0.46944444444444444</v>
       </c>
       <c r="Y59" s="1">
         <v>46277</v>
@@ -4498,10 +4498,10 @@
         <v>46265</v>
       </c>
       <c r="S60" s="1">
-        <v>46263</v>
+        <v>46260</v>
       </c>
       <c r="U60" s="1">
-        <v>46266</v>
+        <v>46262</v>
       </c>
       <c r="Y60" s="1">
         <v>46277</v>
@@ -4566,13 +4566,13 @@
         <v>46269</v>
       </c>
       <c r="T61" s="2">
-        <v>0.31666666666666665</v>
+        <v>0.4701388888888889</v>
       </c>
       <c r="U61" s="1">
         <v>46276</v>
       </c>
       <c r="V61" s="2">
-        <v>0.2951388888888889</v>
+        <v>0.4486111111111111</v>
       </c>
       <c r="X61" t="str">
         <v>1702 Piyumi Perera</v>
@@ -4610,10 +4610,10 @@
         <v>46267</v>
       </c>
       <c r="S62" s="1">
-        <v>46266</v>
+        <v>46262</v>
       </c>
       <c r="U62" s="1">
-        <v>46273</v>
+        <v>46269</v>
       </c>
       <c r="X62" t="str">
         <v>1702 Piyumi Perera</v>
@@ -4681,7 +4681,7 @@
         <v>46276</v>
       </c>
       <c r="T63" s="2">
-        <v>0.29583333333333334</v>
+        <v>0.44930555555555557</v>
       </c>
       <c r="U63" s="1">
         <v>46276</v>
@@ -4758,7 +4758,7 @@
         <v>46279</v>
       </c>
       <c r="V64" s="2">
-        <v>0.29930555555555555</v>
+        <v>0.4527777777777778</v>
       </c>
       <c r="Y64" s="1">
         <v>46298</v>
@@ -4793,10 +4793,10 @@
         <v>46274</v>
       </c>
       <c r="S65" s="1">
-        <v>46273</v>
+        <v>46269</v>
       </c>
       <c r="U65" s="1">
-        <v>46275</v>
+        <v>46272</v>
       </c>
       <c r="Y65" s="1">
         <v>46298</v>
@@ -4858,13 +4858,13 @@
         <v>46279</v>
       </c>
       <c r="T66" s="2">
-        <v>0.3</v>
+        <v>0.4534722222222222</v>
       </c>
       <c r="U66" s="1">
         <v>46283</v>
       </c>
       <c r="V66" s="2">
-        <v>0.43125</v>
+        <v>0.5847222222222223</v>
       </c>
       <c r="Y66" s="1">
         <v>46301</v>
@@ -4899,10 +4899,10 @@
         <v>46276</v>
       </c>
       <c r="S67" s="1">
-        <v>46275</v>
+        <v>46272</v>
       </c>
       <c r="U67" s="1">
-        <v>46280</v>
+        <v>46276</v>
       </c>
       <c r="Y67" s="1">
         <v>46301</v>
@@ -4964,13 +4964,13 @@
         <v>46283</v>
       </c>
       <c r="T68" s="2">
-        <v>0.43194444444444446</v>
+        <v>0.5854166666666667</v>
       </c>
       <c r="U68" s="1">
         <v>46286</v>
       </c>
       <c r="V68" s="2">
-        <v>0.5069444444444444</v>
+        <v>0.6604166666666667</v>
       </c>
       <c r="Y68" s="1">
         <v>46304</v>
@@ -5005,10 +5005,10 @@
         <v>46281</v>
       </c>
       <c r="S69" s="1">
-        <v>46280</v>
+        <v>46276</v>
       </c>
       <c r="U69" s="1">
-        <v>46282</v>
+        <v>46279</v>
       </c>
       <c r="Y69" s="1">
         <v>46304</v>
@@ -5070,13 +5070,13 @@
         <v>46286</v>
       </c>
       <c r="T70" s="2">
-        <v>0.5076388888888889</v>
+        <v>0.6611111111111111</v>
       </c>
       <c r="U70" s="1">
         <v>46293</v>
       </c>
       <c r="V70" s="2">
-        <v>0.46319444444444446</v>
+        <v>0.6166666666666667</v>
       </c>
       <c r="Y70" s="1">
         <v>46301</v>
@@ -5111,10 +5111,10 @@
         <v>46283</v>
       </c>
       <c r="S71" s="1">
-        <v>46282</v>
+        <v>46279</v>
       </c>
       <c r="U71" s="1">
-        <v>46289</v>
+        <v>46286</v>
       </c>
       <c r="Y71" s="1">
         <v>46301</v>
@@ -5176,13 +5176,13 @@
         <v>46293</v>
       </c>
       <c r="T72" s="2">
-        <v>0.4638888888888889</v>
+        <v>0.6173611111111111</v>
       </c>
       <c r="U72" s="1">
         <v>46295</v>
       </c>
       <c r="V72" s="2">
-        <v>0.5784722222222223</v>
+        <v>0.7319444444444444</v>
       </c>
       <c r="Y72" s="1">
         <v>46304</v>
@@ -5217,10 +5217,10 @@
         <v>46290</v>
       </c>
       <c r="S73" s="1">
-        <v>46289</v>
+        <v>46286</v>
       </c>
       <c r="U73" s="1">
-        <v>46291</v>
+        <v>46288</v>
       </c>
       <c r="Y73" s="1">
         <v>46304</v>
@@ -5282,13 +5282,13 @@
         <v>46295</v>
       </c>
       <c r="T74" s="2">
-        <v>0.5791666666666667</v>
+        <v>0.7326388888888888</v>
       </c>
       <c r="U74" s="1">
         <v>46296</v>
       </c>
       <c r="V74" s="2">
-        <v>0.47291666666666665</v>
+        <v>0.6263888888888889</v>
       </c>
       <c r="Y74" s="1">
         <v>46317</v>
@@ -5323,10 +5323,10 @@
         <v>46293</v>
       </c>
       <c r="S75" s="1">
-        <v>46291</v>
+        <v>46288</v>
       </c>
       <c r="U75" s="1">
-        <v>46294</v>
+        <v>46290</v>
       </c>
       <c r="Y75" s="1">
         <v>46317</v>
@@ -6137,7 +6137,7 @@
         <v>46244</v>
       </c>
       <c r="V86" s="2">
-        <v>0.5763888888888888</v>
+        <v>0.4388888888888889</v>
       </c>
       <c r="X86" t="str">
         <v>1675 Dinusha Guantillake</v>
@@ -6178,7 +6178,7 @@
         <v>46235</v>
       </c>
       <c r="U87" s="1">
-        <v>46244</v>
+        <v>46245</v>
       </c>
       <c r="X87" t="str">
         <v>1675 Dinusha Guantillake</v>
@@ -6246,7 +6246,7 @@
         <v>46244</v>
       </c>
       <c r="T88" s="2">
-        <v>0.6076388888888888</v>
+        <v>0.31666666666666665</v>
       </c>
       <c r="U88" s="1">
         <v>46245</v>
@@ -7066,7 +7066,7 @@
         <v>46253</v>
       </c>
       <c r="V99" s="2">
-        <v>0.6527777777777778</v>
+        <v>0.36180555555555555</v>
       </c>
       <c r="X99" t="str">
         <v>1675 Dinusha Guantillake</v>
@@ -7104,10 +7104,10 @@
         <v>46241</v>
       </c>
       <c r="S100" s="1">
-        <v>46247</v>
+        <v>46252</v>
       </c>
       <c r="U100" s="1">
-        <v>46256</v>
+        <v>46261</v>
       </c>
       <c r="X100" t="str">
         <v>1675 Dinusha Guantillake</v>
@@ -7172,7 +7172,7 @@
         <v>46253</v>
       </c>
       <c r="T101" s="2">
-        <v>0.6534722222222222</v>
+        <v>0.3625</v>
       </c>
       <c r="U101" s="1">
         <v>46254</v>
@@ -7462,7 +7462,7 @@
         <v>46255</v>
       </c>
       <c r="V105" s="2">
-        <v>0.59375</v>
+        <v>0.30277777777777776</v>
       </c>
       <c r="X105" t="str">
         <v>1702 Piyumi Perera</v>
@@ -7500,10 +7500,10 @@
         <v>46251</v>
       </c>
       <c r="S106" s="1">
-        <v>46256</v>
+        <v>46261</v>
       </c>
       <c r="U106" s="1">
-        <v>46259</v>
+        <v>46263</v>
       </c>
       <c r="X106" t="str">
         <v>1702 Piyumi Perera</v>
@@ -7568,13 +7568,13 @@
         <v>46255</v>
       </c>
       <c r="T107" s="2">
-        <v>0.5944444444444444</v>
+        <v>0.3034722222222222</v>
       </c>
       <c r="U107" s="1">
         <v>46259</v>
       </c>
       <c r="V107" s="2">
-        <v>0.5576388888888889</v>
+        <v>0.7458333333333333</v>
       </c>
       <c r="Y107" s="1">
         <v>46265</v>
@@ -7609,10 +7609,10 @@
         <v>46253</v>
       </c>
       <c r="S108" s="1">
-        <v>46259</v>
+        <v>46263</v>
       </c>
       <c r="U108" s="1">
-        <v>46262</v>
+        <v>46266</v>
       </c>
       <c r="Y108" s="1">
         <v>46265</v>
@@ -7677,7 +7677,7 @@
         <v>46259</v>
       </c>
       <c r="T109" s="2">
-        <v>0.5583333333333333</v>
+        <v>0.7465277777777778</v>
       </c>
       <c r="U109" s="1">
         <v>46262</v>
@@ -8393,7 +8393,7 @@
         <v>46265</v>
       </c>
       <c r="V119" s="2">
-        <v>0.4576388888888889</v>
+        <v>0.6458333333333334</v>
       </c>
       <c r="Y119" s="1">
         <v>46275</v>
@@ -8428,10 +8428,10 @@
         <v>46256</v>
       </c>
       <c r="S120" s="1">
-        <v>46262</v>
+        <v>46266</v>
       </c>
       <c r="U120" s="1">
-        <v>46268</v>
+        <v>46272</v>
       </c>
       <c r="Y120" s="1">
         <v>46275</v>
@@ -8493,7 +8493,7 @@
         <v>46283</v>
       </c>
       <c r="T121" s="2">
-        <v>0.4583333333333333</v>
+        <v>0.6465277777777778</v>
       </c>
       <c r="U121" s="1">
         <v>46283</v>
@@ -8635,7 +8635,7 @@
         <v>46293</v>
       </c>
       <c r="V123" s="2">
-        <v>0.45208333333333334</v>
+        <v>0.6402777777777777</v>
       </c>
       <c r="Y123" s="1">
         <v>46305</v>
@@ -8670,10 +8670,10 @@
         <v>46281</v>
       </c>
       <c r="S124" s="1">
-        <v>46268</v>
+        <v>46272</v>
       </c>
       <c r="U124" s="1">
-        <v>46277</v>
+        <v>46281</v>
       </c>
       <c r="Y124" s="1">
         <v>46305</v>
@@ -8738,13 +8738,13 @@
         <v>46293</v>
       </c>
       <c r="T125" s="2">
-        <v>0.4527777777777778</v>
+        <v>0.6409722222222223</v>
       </c>
       <c r="U125" s="1">
         <v>46301</v>
       </c>
       <c r="V125" s="2">
-        <v>0.6430555555555556</v>
+        <v>0.35208333333333336</v>
       </c>
       <c r="Y125" s="1">
         <v>46305</v>
@@ -8779,10 +8779,10 @@
         <v>46290</v>
       </c>
       <c r="S126" s="1">
-        <v>46277</v>
+        <v>46281</v>
       </c>
       <c r="U126" s="1">
-        <v>46286</v>
+        <v>46290</v>
       </c>
       <c r="Y126" s="1">
         <v>46305</v>

</xml_diff>

<commit_message>
SGL FR Plan — 17/08/2026 20:56
</commit_message>
<xml_diff>
--- a/Production_Plan.xlsx
+++ b/Production_Plan.xlsx
@@ -748,7 +748,7 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>SGL 01</v>
+        <v>SGL 03</v>
       </c>
       <c r="B6">
         <v>847</v>
@@ -805,7 +805,7 @@
         <v>46238</v>
       </c>
       <c r="T6" s="2">
-        <v>0.4486111111111111</v>
+        <v>0.39166666666666666</v>
       </c>
       <c r="U6" s="1">
         <v>46240</v>
@@ -822,7 +822,7 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>SGL 01</v>
+        <v>SGL 03</v>
       </c>
       <c r="B7">
         <v>847</v>
@@ -896,7 +896,7 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>SGL 01</v>
+        <v>SGL 03</v>
       </c>
       <c r="B8">
         <v>847</v>
@@ -959,7 +959,7 @@
         <v>46241</v>
       </c>
       <c r="V8" s="2">
-        <v>0.29444444444444445</v>
+        <v>0.7166666666666667</v>
       </c>
       <c r="X8" t="str">
         <v>1675 Dinusha Guantillake</v>
@@ -970,7 +970,7 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>SGL 01</v>
+        <v>SGL 03</v>
       </c>
       <c r="C9" t="str">
         <v>3497A::SGSGZIMER5060::SH</v>
@@ -997,10 +997,10 @@
         <v>0</v>
       </c>
       <c r="S9" s="1">
-        <v>46238</v>
+        <v>46245</v>
       </c>
       <c r="U9" s="1">
-        <v>46241</v>
+        <v>46247</v>
       </c>
       <c r="X9" t="str">
         <v>1675 Dinusha Guantillake</v>
@@ -1923,7 +1923,7 @@
         <v>46245</v>
       </c>
       <c r="T22" s="2">
-        <v>0.2951388888888889</v>
+        <v>0.4486111111111111</v>
       </c>
       <c r="U22" s="1">
         <v>46245</v>
@@ -3039,7 +3039,7 @@
         <v>46251</v>
       </c>
       <c r="V37" s="2">
-        <v>0.6625</v>
+        <v>0.3368055555555556</v>
       </c>
       <c r="X37" t="str">
         <v>1702 Piyumi Perera</v>
@@ -3077,10 +3077,10 @@
         <v>46242</v>
       </c>
       <c r="S38" s="1">
-        <v>46241</v>
+        <v>46238</v>
       </c>
       <c r="U38" s="1">
-        <v>46247</v>
+        <v>46245</v>
       </c>
       <c r="X38" t="str">
         <v>1702 Piyumi Perera</v>
@@ -3148,7 +3148,7 @@
         <v>46251</v>
       </c>
       <c r="T39" s="2">
-        <v>0.6631944444444444</v>
+        <v>0.3375</v>
       </c>
       <c r="U39" s="1">
         <v>46255</v>
@@ -3651,7 +3651,7 @@
         <v>46259</v>
       </c>
       <c r="V46" s="2">
-        <v>0.4979166666666667</v>
+        <v>0.6513888888888889</v>
       </c>
       <c r="Y46" s="1">
         <v>46266</v>
@@ -3686,10 +3686,10 @@
         <v>46248</v>
       </c>
       <c r="S47" s="1">
-        <v>46247</v>
+        <v>46245</v>
       </c>
       <c r="U47" s="1">
-        <v>46255</v>
+        <v>46252</v>
       </c>
       <c r="Y47" s="1">
         <v>46266</v>
@@ -3751,13 +3751,13 @@
         <v>46259</v>
       </c>
       <c r="T48" s="2">
-        <v>0.4986111111111111</v>
+        <v>0.6520833333333333</v>
       </c>
       <c r="U48" s="1">
         <v>46262</v>
       </c>
       <c r="V48" s="2">
-        <v>0.6020833333333333</v>
+        <v>0.7555555555555555</v>
       </c>
       <c r="Y48" s="1">
         <v>46265</v>
@@ -3792,10 +3792,10 @@
         <v>46256</v>
       </c>
       <c r="S49" s="1">
+        <v>46252</v>
+      </c>
+      <c r="U49" s="1">
         <v>46255</v>
-      </c>
-      <c r="U49" s="1">
-        <v>46259</v>
       </c>
       <c r="Y49" s="1">
         <v>46265</v>
@@ -3860,7 +3860,7 @@
         <v>46262</v>
       </c>
       <c r="T50" s="2">
-        <v>0.6027777777777777</v>
+        <v>0.75625</v>
       </c>
       <c r="U50" s="1">
         <v>46263</v>
@@ -4236,7 +4236,7 @@
         <v>46266</v>
       </c>
       <c r="V55" s="2">
-        <v>0.575</v>
+        <v>0.7284722222222222</v>
       </c>
       <c r="X55" t="str">
         <v>1702 Piyumi Perera</v>
@@ -4274,10 +4274,10 @@
         <v>46260</v>
       </c>
       <c r="S56" s="1">
+        <v>46255</v>
+      </c>
+      <c r="U56" s="1">
         <v>46259</v>
-      </c>
-      <c r="U56" s="1">
-        <v>46262</v>
       </c>
       <c r="X56" t="str">
         <v>1702 Piyumi Perera</v>
@@ -4345,13 +4345,13 @@
         <v>46266</v>
       </c>
       <c r="T57" s="2">
-        <v>0.5756944444444444</v>
+        <v>0.7291666666666666</v>
       </c>
       <c r="U57" s="1">
         <v>46267</v>
       </c>
       <c r="V57" s="2">
-        <v>0.45</v>
+        <v>0.6034722222222222</v>
       </c>
       <c r="X57" t="str">
         <v>1702 Piyumi Perera</v>
@@ -4389,10 +4389,10 @@
         <v>46263</v>
       </c>
       <c r="S58" s="1">
-        <v>46262</v>
+        <v>46259</v>
       </c>
       <c r="U58" s="1">
-        <v>46263</v>
+        <v>46260</v>
       </c>
       <c r="X58" t="str">
         <v>1702 Piyumi Perera</v>
@@ -4457,13 +4457,13 @@
         <v>46267</v>
       </c>
       <c r="T59" s="2">
-        <v>0.45069444444444445</v>
+        <v>0.6041666666666666</v>
       </c>
       <c r="U59" s="1">
         <v>46269</v>
       </c>
       <c r="V59" s="2">
-        <v>0.3159722222222222</v>
+        <v>0.46944444444444444</v>
       </c>
       <c r="Y59" s="1">
         <v>46277</v>
@@ -4498,10 +4498,10 @@
         <v>46265</v>
       </c>
       <c r="S60" s="1">
-        <v>46263</v>
+        <v>46260</v>
       </c>
       <c r="U60" s="1">
-        <v>46266</v>
+        <v>46262</v>
       </c>
       <c r="Y60" s="1">
         <v>46277</v>
@@ -4566,13 +4566,13 @@
         <v>46269</v>
       </c>
       <c r="T61" s="2">
-        <v>0.31666666666666665</v>
+        <v>0.4701388888888889</v>
       </c>
       <c r="U61" s="1">
         <v>46276</v>
       </c>
       <c r="V61" s="2">
-        <v>0.2951388888888889</v>
+        <v>0.4486111111111111</v>
       </c>
       <c r="X61" t="str">
         <v>1702 Piyumi Perera</v>
@@ -4610,10 +4610,10 @@
         <v>46267</v>
       </c>
       <c r="S62" s="1">
-        <v>46266</v>
+        <v>46262</v>
       </c>
       <c r="U62" s="1">
-        <v>46273</v>
+        <v>46269</v>
       </c>
       <c r="X62" t="str">
         <v>1702 Piyumi Perera</v>
@@ -4681,7 +4681,7 @@
         <v>46276</v>
       </c>
       <c r="T63" s="2">
-        <v>0.29583333333333334</v>
+        <v>0.44930555555555557</v>
       </c>
       <c r="U63" s="1">
         <v>46276</v>
@@ -4758,7 +4758,7 @@
         <v>46279</v>
       </c>
       <c r="V64" s="2">
-        <v>0.29930555555555555</v>
+        <v>0.4527777777777778</v>
       </c>
       <c r="Y64" s="1">
         <v>46298</v>
@@ -4793,10 +4793,10 @@
         <v>46274</v>
       </c>
       <c r="S65" s="1">
-        <v>46273</v>
+        <v>46269</v>
       </c>
       <c r="U65" s="1">
-        <v>46275</v>
+        <v>46272</v>
       </c>
       <c r="Y65" s="1">
         <v>46298</v>
@@ -4858,13 +4858,13 @@
         <v>46279</v>
       </c>
       <c r="T66" s="2">
-        <v>0.3</v>
+        <v>0.4534722222222222</v>
       </c>
       <c r="U66" s="1">
         <v>46283</v>
       </c>
       <c r="V66" s="2">
-        <v>0.43125</v>
+        <v>0.5847222222222223</v>
       </c>
       <c r="Y66" s="1">
         <v>46301</v>
@@ -4899,10 +4899,10 @@
         <v>46276</v>
       </c>
       <c r="S67" s="1">
-        <v>46275</v>
+        <v>46272</v>
       </c>
       <c r="U67" s="1">
-        <v>46280</v>
+        <v>46276</v>
       </c>
       <c r="Y67" s="1">
         <v>46301</v>
@@ -4964,13 +4964,13 @@
         <v>46283</v>
       </c>
       <c r="T68" s="2">
-        <v>0.43194444444444446</v>
+        <v>0.5854166666666667</v>
       </c>
       <c r="U68" s="1">
         <v>46286</v>
       </c>
       <c r="V68" s="2">
-        <v>0.5069444444444444</v>
+        <v>0.6604166666666667</v>
       </c>
       <c r="Y68" s="1">
         <v>46304</v>
@@ -5005,10 +5005,10 @@
         <v>46281</v>
       </c>
       <c r="S69" s="1">
-        <v>46280</v>
+        <v>46276</v>
       </c>
       <c r="U69" s="1">
-        <v>46282</v>
+        <v>46279</v>
       </c>
       <c r="Y69" s="1">
         <v>46304</v>
@@ -5070,13 +5070,13 @@
         <v>46286</v>
       </c>
       <c r="T70" s="2">
-        <v>0.5076388888888889</v>
+        <v>0.6611111111111111</v>
       </c>
       <c r="U70" s="1">
         <v>46293</v>
       </c>
       <c r="V70" s="2">
-        <v>0.46319444444444446</v>
+        <v>0.6166666666666667</v>
       </c>
       <c r="Y70" s="1">
         <v>46301</v>
@@ -5111,10 +5111,10 @@
         <v>46283</v>
       </c>
       <c r="S71" s="1">
-        <v>46282</v>
+        <v>46279</v>
       </c>
       <c r="U71" s="1">
-        <v>46289</v>
+        <v>46286</v>
       </c>
       <c r="Y71" s="1">
         <v>46301</v>
@@ -5176,13 +5176,13 @@
         <v>46293</v>
       </c>
       <c r="T72" s="2">
-        <v>0.4638888888888889</v>
+        <v>0.6173611111111111</v>
       </c>
       <c r="U72" s="1">
         <v>46295</v>
       </c>
       <c r="V72" s="2">
-        <v>0.5784722222222223</v>
+        <v>0.7319444444444444</v>
       </c>
       <c r="Y72" s="1">
         <v>46304</v>
@@ -5217,10 +5217,10 @@
         <v>46290</v>
       </c>
       <c r="S73" s="1">
-        <v>46289</v>
+        <v>46286</v>
       </c>
       <c r="U73" s="1">
-        <v>46291</v>
+        <v>46288</v>
       </c>
       <c r="Y73" s="1">
         <v>46304</v>
@@ -5282,13 +5282,13 @@
         <v>46295</v>
       </c>
       <c r="T74" s="2">
-        <v>0.5791666666666667</v>
+        <v>0.7326388888888888</v>
       </c>
       <c r="U74" s="1">
         <v>46296</v>
       </c>
       <c r="V74" s="2">
-        <v>0.47291666666666665</v>
+        <v>0.6263888888888889</v>
       </c>
       <c r="Y74" s="1">
         <v>46317</v>
@@ -5323,10 +5323,10 @@
         <v>46293</v>
       </c>
       <c r="S75" s="1">
-        <v>46291</v>
+        <v>46288</v>
       </c>
       <c r="U75" s="1">
-        <v>46294</v>
+        <v>46290</v>
       </c>
       <c r="Y75" s="1">
         <v>46317</v>
@@ -9705,7 +9705,7 @@
         <v>46245</v>
       </c>
       <c r="V139" s="2">
-        <v>0.3236111111111111</v>
+        <v>0.3909722222222222</v>
       </c>
       <c r="X139" t="str">
         <v>1675 Dinusha Guantillake</v>
@@ -9814,7 +9814,7 @@
         <v>46245</v>
       </c>
       <c r="T141" s="2">
-        <v>0.32430555555555557</v>
+        <v>0.7173611111111111</v>
       </c>
       <c r="U141" s="1">
         <v>46245</v>
@@ -10338,7 +10338,7 @@
         <v>46249</v>
       </c>
       <c r="V148" s="2">
-        <v>0.30694444444444446</v>
+        <v>0.7</v>
       </c>
       <c r="X148" t="str">
         <v>1675 Dinusha Guantillake</v>
@@ -10376,10 +10376,10 @@
         <v>46242</v>
       </c>
       <c r="S149" s="1">
-        <v>46245</v>
+        <v>46247</v>
       </c>
       <c r="U149" s="1">
-        <v>46249</v>
+        <v>46252</v>
       </c>
       <c r="X149" t="str">
         <v>1675 Dinusha Guantillake</v>
@@ -10447,7 +10447,7 @@
         <v>46249</v>
       </c>
       <c r="T150" s="2">
-        <v>0.3076388888888889</v>
+        <v>0.7006944444444444</v>
       </c>
       <c r="U150" s="1">
         <v>46251</v>
@@ -10524,7 +10524,7 @@
         <v>46251</v>
       </c>
       <c r="V151" s="2">
-        <v>0.4125</v>
+        <v>0.3263888888888889</v>
       </c>
       <c r="Y151" s="1">
         <v>46255</v>
@@ -10559,10 +10559,10 @@
         <v>46247</v>
       </c>
       <c r="S152" s="1">
-        <v>46249</v>
+        <v>46252</v>
       </c>
       <c r="U152" s="1">
-        <v>46251</v>
+        <v>46254</v>
       </c>
       <c r="Y152" s="1">
         <v>46255</v>
@@ -10627,7 +10627,7 @@
         <v>46251</v>
       </c>
       <c r="T153" s="2">
-        <v>0.4131944444444444</v>
+        <v>0.32708333333333334</v>
       </c>
       <c r="U153" s="1">
         <v>46251</v>
@@ -10704,7 +10704,7 @@
         <v>46251</v>
       </c>
       <c r="V154" s="2">
-        <v>0.5423611111111111</v>
+        <v>0.45625</v>
       </c>
       <c r="Y154" s="1">
         <v>46226</v>
@@ -10739,10 +10739,10 @@
         <v>46242</v>
       </c>
       <c r="S155" s="1">
-        <v>46251</v>
+        <v>46254</v>
       </c>
       <c r="U155" s="1">
-        <v>46251</v>
+        <v>46254</v>
       </c>
       <c r="Y155" s="1">
         <v>46226</v>
@@ -10807,7 +10807,7 @@
         <v>46251</v>
       </c>
       <c r="T156" s="2">
-        <v>0.5430555555555555</v>
+        <v>0.45694444444444443</v>
       </c>
       <c r="U156" s="1">
         <v>46256</v>
@@ -11594,7 +11594,7 @@
         <v>46265</v>
       </c>
       <c r="V167" s="2">
-        <v>0.3541666666666667</v>
+        <v>0.7472222222222222</v>
       </c>
       <c r="Y167" s="1">
         <v>46270</v>
@@ -11629,10 +11629,10 @@
         <v>46248</v>
       </c>
       <c r="S168" s="1">
-        <v>46251</v>
+        <v>46254</v>
       </c>
       <c r="U168" s="1">
-        <v>46265</v>
+        <v>46267</v>
       </c>
       <c r="Y168" s="1">
         <v>46270</v>
@@ -11697,13 +11697,13 @@
         <v>46265</v>
       </c>
       <c r="T169" s="2">
-        <v>0.3548611111111111</v>
+        <v>0.7479166666666667</v>
       </c>
       <c r="U169" s="1">
         <v>46266</v>
       </c>
       <c r="V169" s="2">
-        <v>0.49375</v>
+        <v>0.4076388888888889</v>
       </c>
       <c r="Y169" s="1">
         <v>46247</v>
@@ -11738,10 +11738,10 @@
         <v>46262</v>
       </c>
       <c r="S170" s="1">
-        <v>46265</v>
+        <v>46267</v>
       </c>
       <c r="U170" s="1">
-        <v>46266</v>
+        <v>46269</v>
       </c>
       <c r="Y170" s="1">
         <v>46247</v>
@@ -11806,13 +11806,13 @@
         <v>46266</v>
       </c>
       <c r="T171" s="2">
-        <v>0.49444444444444446</v>
+        <v>0.4083333333333333</v>
       </c>
       <c r="U171" s="1">
         <v>46269</v>
       </c>
       <c r="V171" s="2">
-        <v>0.3819444444444444</v>
+        <v>0.29583333333333334</v>
       </c>
       <c r="Y171" s="1">
         <v>46247</v>
@@ -11847,10 +11847,10 @@
         <v>46263</v>
       </c>
       <c r="S172" s="1">
-        <v>46266</v>
+        <v>46269</v>
       </c>
       <c r="U172" s="1">
-        <v>46269</v>
+        <v>46273</v>
       </c>
       <c r="Y172" s="1">
         <v>46247</v>
@@ -11915,13 +11915,13 @@
         <v>46269</v>
       </c>
       <c r="T173" s="2">
-        <v>0.38263888888888886</v>
+        <v>0.2965277777777778</v>
       </c>
       <c r="U173" s="1">
         <v>46272</v>
       </c>
       <c r="V173" s="2">
-        <v>0.3215277777777778</v>
+        <v>0.7145833333333333</v>
       </c>
       <c r="Y173" s="1">
         <v>46247</v>
@@ -11956,10 +11956,10 @@
         <v>46267</v>
       </c>
       <c r="S174" s="1">
-        <v>46269</v>
+        <v>46273</v>
       </c>
       <c r="U174" s="1">
-        <v>46272</v>
+        <v>46274</v>
       </c>
       <c r="Y174" s="1">
         <v>46247</v>
@@ -12021,13 +12021,13 @@
         <v>46283</v>
       </c>
       <c r="T175" s="2">
-        <v>0.2916666666666667</v>
+        <v>0.7152777777777778</v>
       </c>
       <c r="U175" s="1">
         <v>46284</v>
       </c>
       <c r="V175" s="2">
-        <v>0.4388888888888889</v>
+        <v>0.38333333333333336</v>
       </c>
       <c r="X175" t="str">
         <v>1702 Piyumi Perera</v>
@@ -12065,10 +12065,10 @@
         <v>46281</v>
       </c>
       <c r="S176" s="1">
-        <v>46283</v>
+        <v>46274</v>
       </c>
       <c r="U176" s="1">
-        <v>46284</v>
+        <v>46276</v>
       </c>
       <c r="X176" t="str">
         <v>1702 Piyumi Perera</v>
@@ -12133,7 +12133,7 @@
         <v>46284</v>
       </c>
       <c r="T177" s="2">
-        <v>0.4395833333333333</v>
+        <v>0.3840277777777778</v>
       </c>
       <c r="U177" s="1">
         <v>46286</v>
@@ -12207,7 +12207,7 @@
         <v>46298</v>
       </c>
       <c r="V178" s="2">
-        <v>0.3736111111111111</v>
+        <v>0.31805555555555554</v>
       </c>
       <c r="Y178" s="1">
         <v>46305</v>
@@ -12242,10 +12242,10 @@
         <v>46282</v>
       </c>
       <c r="S179" s="1">
-        <v>46284</v>
+        <v>46276</v>
       </c>
       <c r="U179" s="1">
-        <v>46301</v>
+        <v>46293</v>
       </c>
       <c r="Y179" s="1">
         <v>46305</v>

</xml_diff>

<commit_message>
SGL FR Plan — 03/09/2026 22:08
</commit_message>
<xml_diff>
--- a/Production_Plan.xlsx
+++ b/Production_Plan.xlsx
@@ -6499,7 +6499,7 @@
         <v>46274</v>
       </c>
       <c r="V96" s="2">
-        <v>0.5847222222222223</v>
+        <v>0.7597222222222222</v>
       </c>
       <c r="Y96" s="1">
         <v>46282</v>
@@ -6602,7 +6602,7 @@
         <v>46275</v>
       </c>
       <c r="T98" s="2">
-        <v>0.2916666666666667</v>
+        <v>0.7604166666666666</v>
       </c>
       <c r="U98" s="1">
         <v>46277</v>
@@ -6682,7 +6682,7 @@
         <v>46279</v>
       </c>
       <c r="V99" s="2">
-        <v>0.3020833333333333</v>
+        <v>0.7708333333333334</v>
       </c>
       <c r="X99" t="str">
         <v>1675 Dinusha Guantillake</v>
@@ -6720,10 +6720,10 @@
         <v>46272</v>
       </c>
       <c r="S100" s="1">
-        <v>46275</v>
+        <v>46274</v>
       </c>
       <c r="U100" s="1">
-        <v>46279</v>
+        <v>46277</v>
       </c>
       <c r="X100" t="str">
         <v>1675 Dinusha Guantillake</v>
@@ -6791,13 +6791,13 @@
         <v>46279</v>
       </c>
       <c r="T101" s="2">
-        <v>0.31666666666666665</v>
+        <v>0.2916666666666667</v>
       </c>
       <c r="U101" s="1">
         <v>46286</v>
       </c>
       <c r="V101" s="2">
-        <v>0.34305555555555556</v>
+        <v>0.31805555555555554</v>
       </c>
       <c r="X101" t="str">
         <v>1553 Niwya Diwanjana</v>
@@ -6906,7 +6906,7 @@
         <v>46286</v>
       </c>
       <c r="T103" s="2">
-        <v>0.34375</v>
+        <v>0.31875</v>
       </c>
       <c r="U103" s="1">
         <v>46286</v>
@@ -7134,7 +7134,7 @@
         <v>46300</v>
       </c>
       <c r="V106" s="2">
-        <v>0.29930555555555555</v>
+        <v>0.7534722222222222</v>
       </c>
       <c r="X106" t="str">
         <v>1675 Dinusha Guantillake</v>
@@ -7175,7 +7175,7 @@
         <v>46286</v>
       </c>
       <c r="U107" s="1">
-        <v>46300</v>
+        <v>46298</v>
       </c>
       <c r="X107" t="str">
         <v>1675 Dinusha Guantillake</v>
@@ -7243,7 +7243,7 @@
         <v>46300</v>
       </c>
       <c r="T108" s="2">
-        <v>0.3</v>
+        <v>0.7541666666666667</v>
       </c>
       <c r="U108" s="1">
         <v>46303</v>
@@ -7323,7 +7323,7 @@
         <v>46304</v>
       </c>
       <c r="V109" s="2">
-        <v>0.38263888888888886</v>
+        <v>0.3576388888888889</v>
       </c>
       <c r="X109" t="str">
         <v>1675 Dinusha Guantillake</v>
@@ -7361,7 +7361,7 @@
         <v>46297</v>
       </c>
       <c r="S110" s="1">
-        <v>46300</v>
+        <v>46298</v>
       </c>
       <c r="U110" s="1">
         <v>46304</v>
@@ -7432,13 +7432,13 @@
         <v>46317</v>
       </c>
       <c r="T111" s="2">
-        <v>0.46458333333333335</v>
+        <v>0.35833333333333334</v>
       </c>
       <c r="U111" s="1">
         <v>46322</v>
       </c>
       <c r="V111" s="2">
-        <v>0.29375</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="Y111" s="1">
         <v>46338</v>
@@ -7473,10 +7473,10 @@
         <v>46315</v>
       </c>
       <c r="S112" s="1">
-        <v>46317</v>
+        <v>46304</v>
       </c>
       <c r="U112" s="1">
-        <v>46322</v>
+        <v>46308</v>
       </c>
       <c r="Y112" s="1">
         <v>46338</v>
@@ -7541,7 +7541,7 @@
         <v>46322</v>
       </c>
       <c r="T113" s="2">
-        <v>0.29444444444444445</v>
+        <v>0.6673611111111111</v>
       </c>
       <c r="U113" s="1">
         <v>46323</v>
@@ -7618,7 +7618,7 @@
         <v>46324</v>
       </c>
       <c r="V114" s="2">
-        <v>0.6513888888888889</v>
+        <v>0.5451388888888888</v>
       </c>
       <c r="Y114" s="1">
         <v>46338</v>
@@ -7653,10 +7653,10 @@
         <v>46319</v>
       </c>
       <c r="S115" s="1">
-        <v>46322</v>
+        <v>46308</v>
       </c>
       <c r="U115" s="1">
-        <v>46324</v>
+        <v>46311</v>
       </c>
       <c r="Y115" s="1">
         <v>46338</v>
@@ -7721,13 +7721,13 @@
         <v>46324</v>
       </c>
       <c r="T116" s="2">
-        <v>0.6520833333333333</v>
+        <v>0.5458333333333333</v>
       </c>
       <c r="U116" s="1">
         <v>46325</v>
       </c>
       <c r="V116" s="2">
-        <v>0.45625</v>
+        <v>0.35</v>
       </c>
       <c r="Y116" s="1">
         <v>46338</v>
@@ -7762,10 +7762,10 @@
         <v>46322</v>
       </c>
       <c r="S117" s="1">
-        <v>46324</v>
+        <v>46311</v>
       </c>
       <c r="U117" s="1">
-        <v>46325</v>
+        <v>46312</v>
       </c>
       <c r="Y117" s="1">
         <v>46338</v>
@@ -11690,7 +11690,7 @@
         <v>46269</v>
       </c>
       <c r="V185" s="2">
-        <v>0.2965277777777778</v>
+        <v>0.4479166666666667</v>
       </c>
       <c r="X185" t="str">
         <v>305 Ishan Jayathilaka</v>
@@ -11731,7 +11731,7 @@
         <v>46267</v>
       </c>
       <c r="U186" s="1">
-        <v>46269</v>
+        <v>46274</v>
       </c>
       <c r="X186" t="str">
         <v>305 Ishan Jayathilaka</v>
@@ -11799,7 +11799,7 @@
         <v>46279</v>
       </c>
       <c r="T187" s="2">
-        <v>0.2916666666666667</v>
+        <v>0.4486111111111111</v>
       </c>
       <c r="U187" s="1">
         <v>46280</v>
@@ -12619,7 +12619,7 @@
         <v>46289</v>
       </c>
       <c r="V198" s="2">
-        <v>0.3993055555555556</v>
+        <v>0.55625</v>
       </c>
       <c r="X198" t="str">
         <v>1675 Dinusha Guantillake</v>
@@ -12657,10 +12657,10 @@
         <v>46276</v>
       </c>
       <c r="S199" s="1">
-        <v>46279</v>
+        <v>46274</v>
       </c>
       <c r="U199" s="1">
-        <v>46289</v>
+        <v>46284</v>
       </c>
       <c r="X199" t="str">
         <v>1675 Dinusha Guantillake</v>
@@ -12728,7 +12728,7 @@
         <v>46289</v>
       </c>
       <c r="T200" s="2">
-        <v>0.40902777777777777</v>
+        <v>0.5569444444444445</v>
       </c>
       <c r="U200" s="1">
         <v>46289</v>
@@ -12808,7 +12808,7 @@
         <v>46294</v>
       </c>
       <c r="V201" s="2">
-        <v>0.47291666666666665</v>
+        <v>0.6208333333333333</v>
       </c>
       <c r="X201" t="str">
         <v>1675 Dinusha Guantillake</v>
@@ -12846,10 +12846,10 @@
         <v>46287</v>
       </c>
       <c r="S202" s="1">
+        <v>46284</v>
+      </c>
+      <c r="U202" s="1">
         <v>46289</v>
-      </c>
-      <c r="U202" s="1">
-        <v>46294</v>
       </c>
       <c r="X202" t="str">
         <v>1675 Dinusha Guantillake</v>
@@ -12917,13 +12917,13 @@
         <v>46294</v>
       </c>
       <c r="T203" s="2">
-        <v>0.47708333333333336</v>
+        <v>0.6215277777777778</v>
       </c>
       <c r="U203" s="1">
         <v>46301</v>
       </c>
       <c r="V203" s="2">
-        <v>0.3527777777777778</v>
+        <v>0.49722222222222223</v>
       </c>
       <c r="X203" t="str">
         <v>1675 Dinusha Guantillake</v>
@@ -12961,10 +12961,10 @@
         <v>46291</v>
       </c>
       <c r="S204" s="1">
-        <v>46294</v>
+        <v>46289</v>
       </c>
       <c r="U204" s="1">
-        <v>46301</v>
+        <v>46296</v>
       </c>
       <c r="X204" t="str">
         <v>1675 Dinusha Guantillake</v>
@@ -13032,7 +13032,7 @@
         <v>46301</v>
       </c>
       <c r="T205" s="2">
-        <v>0.35347222222222224</v>
+        <v>0.4979166666666667</v>
       </c>
       <c r="U205" s="1">
         <v>46301</v>
@@ -13186,7 +13186,7 @@
         <v>46304</v>
       </c>
       <c r="V207" s="2">
-        <v>0.7041666666666667</v>
+        <v>0.36944444444444446</v>
       </c>
       <c r="X207" t="str">
         <v>1702 Piyumi Perera</v>
@@ -13224,10 +13224,10 @@
         <v>46293</v>
       </c>
       <c r="S208" s="1">
+        <v>46296</v>
+      </c>
+      <c r="U208" s="1">
         <v>46301</v>
-      </c>
-      <c r="U208" s="1">
-        <v>46304</v>
       </c>
       <c r="X208" t="str">
         <v>1702 Piyumi Perera</v>
@@ -13295,7 +13295,7 @@
         <v>46305</v>
       </c>
       <c r="T209" s="2">
-        <v>0.3326388888888889</v>
+        <v>0.3701388888888889</v>
       </c>
       <c r="U209" s="1">
         <v>46310</v>
@@ -13375,7 +13375,7 @@
         <v>46310</v>
       </c>
       <c r="V210" s="2">
-        <v>0.5486111111111112</v>
+        <v>0.5861111111111111</v>
       </c>
       <c r="X210" t="str">
         <v>1675 Dinusha Guantillake</v>
@@ -13413,10 +13413,10 @@
         <v>46303</v>
       </c>
       <c r="S211" s="1">
+        <v>46301</v>
+      </c>
+      <c r="U211" s="1">
         <v>46305</v>
-      </c>
-      <c r="U211" s="1">
-        <v>46310</v>
       </c>
       <c r="X211" t="str">
         <v>1675 Dinusha Guantillake</v>
@@ -13484,13 +13484,13 @@
         <v>46310</v>
       </c>
       <c r="T212" s="2">
-        <v>0.5493055555555556</v>
+        <v>0.5868055555555556</v>
       </c>
       <c r="U212" s="1">
         <v>46310</v>
       </c>
       <c r="V212" s="2">
-        <v>0.5527777777777778</v>
+        <v>0.5902777777777778</v>
       </c>
       <c r="Y212" s="1">
         <v>46338</v>
@@ -13525,10 +13525,10 @@
         <v>46308</v>
       </c>
       <c r="S213" s="1">
-        <v>46310</v>
+        <v>46305</v>
       </c>
       <c r="U213" s="1">
-        <v>46310</v>
+        <v>46305</v>
       </c>
       <c r="Y213" s="1">
         <v>46338</v>
@@ -13593,13 +13593,13 @@
         <v>46310</v>
       </c>
       <c r="T214" s="2">
-        <v>0.5534722222222223</v>
+        <v>0.5909722222222222</v>
       </c>
       <c r="U214" s="1">
         <v>46314</v>
       </c>
       <c r="V214" s="2">
-        <v>0.41805555555555557</v>
+        <v>0.45555555555555555</v>
       </c>
       <c r="Y214" s="1">
         <v>46338</v>
@@ -13634,10 +13634,10 @@
         <v>46308</v>
       </c>
       <c r="S215" s="1">
-        <v>46310</v>
+        <v>46305</v>
       </c>
       <c r="U215" s="1">
-        <v>46314</v>
+        <v>46309</v>
       </c>
       <c r="Y215" s="1">
         <v>46338</v>
@@ -13702,13 +13702,13 @@
         <v>46314</v>
       </c>
       <c r="T216" s="2">
-        <v>0.41875</v>
+        <v>0.45625</v>
       </c>
       <c r="U216" s="1">
         <v>46314</v>
       </c>
       <c r="V216" s="2">
-        <v>0.6104166666666667</v>
+        <v>0.6479166666666667</v>
       </c>
       <c r="Y216" s="1">
         <v>46338</v>
@@ -13743,10 +13743,10 @@
         <v>46311</v>
       </c>
       <c r="S217" s="1">
-        <v>46314</v>
+        <v>46309</v>
       </c>
       <c r="U217" s="1">
-        <v>46314</v>
+        <v>46309</v>
       </c>
       <c r="Y217" s="1">
         <v>46338</v>
@@ -13811,13 +13811,13 @@
         <v>46314</v>
       </c>
       <c r="T218" s="2">
-        <v>0.6111111111111112</v>
+        <v>0.6486111111111111</v>
       </c>
       <c r="U218" s="1">
         <v>46315</v>
       </c>
       <c r="V218" s="2">
-        <v>0.29305555555555557</v>
+        <v>0.33055555555555555</v>
       </c>
       <c r="Y218" s="1">
         <v>46338</v>
@@ -13852,10 +13852,10 @@
         <v>46311</v>
       </c>
       <c r="S219" s="1">
-        <v>46314</v>
+        <v>46309</v>
       </c>
       <c r="U219" s="1">
-        <v>46315</v>
+        <v>46310</v>
       </c>
       <c r="Y219" s="1">
         <v>46338</v>
@@ -13920,13 +13920,13 @@
         <v>46315</v>
       </c>
       <c r="T220" s="2">
-        <v>0.29375</v>
+        <v>0.33125</v>
       </c>
       <c r="U220" s="1">
         <v>46315</v>
       </c>
       <c r="V220" s="2">
-        <v>0.4465277777777778</v>
+        <v>0.4840277777777778</v>
       </c>
       <c r="Y220" s="1">
         <v>46338</v>
@@ -13961,10 +13961,10 @@
         <v>46312</v>
       </c>
       <c r="S221" s="1">
-        <v>46315</v>
+        <v>46310</v>
       </c>
       <c r="U221" s="1">
-        <v>46315</v>
+        <v>46310</v>
       </c>
       <c r="Y221" s="1">
         <v>46338</v>
@@ -14029,13 +14029,13 @@
         <v>46315</v>
       </c>
       <c r="T222" s="2">
-        <v>0.4486111111111111</v>
+        <v>0.4847222222222222</v>
       </c>
       <c r="U222" s="1">
         <v>46316</v>
       </c>
       <c r="V222" s="2">
-        <v>0.5493055555555556</v>
+        <v>0.5854166666666667</v>
       </c>
       <c r="Y222" s="1">
         <v>46338</v>
@@ -14070,10 +14070,10 @@
         <v>46312</v>
       </c>
       <c r="S223" s="1">
-        <v>46315</v>
+        <v>46310</v>
       </c>
       <c r="U223" s="1">
-        <v>46316</v>
+        <v>46311</v>
       </c>
       <c r="Y223" s="1">
         <v>46338</v>
@@ -14138,7 +14138,7 @@
         <v>46316</v>
       </c>
       <c r="T224" s="2">
-        <v>0.55</v>
+        <v>0.5861111111111111</v>
       </c>
       <c r="U224" s="1">
         <v>46318</v>
@@ -14440,7 +14440,7 @@
         <v>46328</v>
       </c>
       <c r="V228" s="2">
-        <v>0.49583333333333335</v>
+        <v>0.5319444444444444</v>
       </c>
       <c r="X228" t="str">
         <v>762 Thesantha Hettiarachchi</v>
@@ -14478,10 +14478,10 @@
         <v>46314</v>
       </c>
       <c r="S229" s="1">
-        <v>46316</v>
+        <v>46311</v>
       </c>
       <c r="U229" s="1">
-        <v>46328</v>
+        <v>46323</v>
       </c>
       <c r="X229" t="str">
         <v>762 Thesantha Hettiarachchi</v>
@@ -14549,7 +14549,7 @@
         <v>46328</v>
       </c>
       <c r="T230" s="2">
-        <v>0.4965277777777778</v>
+        <v>0.5326388888888889</v>
       </c>
       <c r="U230" s="1">
         <v>46329</v>
@@ -14777,7 +14777,7 @@
         <v>46335</v>
       </c>
       <c r="V233" s="2">
-        <v>0.43125</v>
+        <v>0.4673611111111111</v>
       </c>
       <c r="X233" t="str">
         <v>1654 Mali Karunarathna</v>
@@ -14815,10 +14815,10 @@
         <v>46325</v>
       </c>
       <c r="S234" s="1">
-        <v>46328</v>
+        <v>46323</v>
       </c>
       <c r="U234" s="1">
-        <v>46335</v>
+        <v>46330</v>
       </c>
       <c r="X234" t="str">
         <v>1654 Mali Karunarathna</v>
@@ -14886,7 +14886,7 @@
         <v>46335</v>
       </c>
       <c r="T235" s="2">
-        <v>0.43194444444444446</v>
+        <v>0.46805555555555556</v>
       </c>
       <c r="U235" s="1">
         <v>46338</v>
@@ -15040,7 +15040,7 @@
         <v>46342</v>
       </c>
       <c r="V237" s="2">
-        <v>0.3173611111111111</v>
+        <v>0.35347222222222224</v>
       </c>
       <c r="X237" t="str">
         <v>762 Thesantha Hettiarachchi</v>
@@ -15078,10 +15078,10 @@
         <v>46332</v>
       </c>
       <c r="S238" s="1">
-        <v>46335</v>
+        <v>46330</v>
       </c>
       <c r="U238" s="1">
-        <v>46342</v>
+        <v>46337</v>
       </c>
       <c r="X238" t="str">
         <v>762 Thesantha Hettiarachchi</v>
@@ -15149,7 +15149,7 @@
         <v>46342</v>
       </c>
       <c r="T239" s="2">
-        <v>0.31805555555555554</v>
+        <v>0.3541666666666667</v>
       </c>
       <c r="U239" s="1">
         <v>46343</v>
@@ -15451,7 +15451,7 @@
         <v>46345</v>
       </c>
       <c r="V243" s="2">
-        <v>0.4125</v>
+        <v>0.4486111111111111</v>
       </c>
       <c r="X243" t="str">
         <v>1515 Sanjaya Mihiran</v>
@@ -15489,10 +15489,10 @@
         <v>46333</v>
       </c>
       <c r="S244" s="1">
-        <v>46342</v>
+        <v>46337</v>
       </c>
       <c r="U244" s="1">
-        <v>46345</v>
+        <v>46340</v>
       </c>
       <c r="X244" t="str">
         <v>1515 Sanjaya Mihiran</v>
@@ -15560,13 +15560,13 @@
         <v>46345</v>
       </c>
       <c r="T245" s="2">
-        <v>0.4131944444444444</v>
+        <v>0.44930555555555557</v>
       </c>
       <c r="U245" s="1">
         <v>46345</v>
       </c>
       <c r="V245" s="2">
-        <v>0.6472222222222223</v>
+        <v>0.6833333333333333</v>
       </c>
       <c r="Y245" s="1">
         <v>46377</v>
@@ -15601,10 +15601,10 @@
         <v>46343</v>
       </c>
       <c r="S246" s="1">
-        <v>46345</v>
+        <v>46340</v>
       </c>
       <c r="U246" s="1">
-        <v>46345</v>
+        <v>46340</v>
       </c>
       <c r="Y246" s="1">
         <v>46377</v>
@@ -15669,13 +15669,13 @@
         <v>46345</v>
       </c>
       <c r="T247" s="2">
-        <v>0.6479166666666667</v>
+        <v>0.6840277777777778</v>
       </c>
       <c r="U247" s="1">
         <v>46351</v>
       </c>
       <c r="V247" s="2">
-        <v>0.36527777777777776</v>
+        <v>0.4013888888888889</v>
       </c>
       <c r="Y247" s="1">
         <v>46377</v>
@@ -15710,10 +15710,10 @@
         <v>46343</v>
       </c>
       <c r="S248" s="1">
-        <v>46345</v>
+        <v>46340</v>
       </c>
       <c r="U248" s="1">
-        <v>46351</v>
+        <v>46346</v>
       </c>
       <c r="Y248" s="1">
         <v>46377</v>
@@ -15778,13 +15778,13 @@
         <v>46351</v>
       </c>
       <c r="T249" s="2">
-        <v>0.3659722222222222</v>
+        <v>0.40208333333333335</v>
       </c>
       <c r="U249" s="1">
         <v>46358</v>
       </c>
       <c r="V249" s="2">
-        <v>0.5777777777777777</v>
+        <v>0.6138888888888889</v>
       </c>
       <c r="Y249" s="1">
         <v>46377</v>
@@ -15819,10 +15819,10 @@
         <v>46349</v>
       </c>
       <c r="S250" s="1">
-        <v>46351</v>
+        <v>46346</v>
       </c>
       <c r="U250" s="1">
-        <v>46358</v>
+        <v>46353</v>
       </c>
       <c r="Y250" s="1">
         <v>46377</v>

</xml_diff>